<commit_message>
Verify promotion KPI workbook rendering
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rceadef3cced34b06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R561a8af8f1824262"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="Rff7528702d31411c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="R113d3b2ec72d439a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6704ecc042014d3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rc38da7dd23d44e8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="Ra584a941913f4ad1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="Rbc86560a7e304b50"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Normalize promotion KPI workbook artifact
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6704ecc042014d3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rc38da7dd23d44e8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="Ra584a941913f4ad1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="Rbc86560a7e304b50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc5422af04b54443e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R65ed3ebff88c46ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="R825bc13bfc5d45b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="Rba42b2b795f94a05"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Add promotion publishing status checks
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc5422af04b54443e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R65ed3ebff88c46ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="R825bc13bfc5d45b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="Rba42b2b795f94a05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R36a68556e77a494e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R4667c199d2634be0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="R99c9ac1ebc0446bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="R1b07c47ec595464f"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Refresh promotion KPI workbook
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Ree5459e1fb8344a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R79e71874c34e45fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R5afdce89cde6460a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R30d7b74ec0214714"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="Rcc4fe77d75284a86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="Rff22422243ac4d0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="R0b4f3a9c9dd84d8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="Re1544862cef44df2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="R3ddfc5bbb39e4bb9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="R37c35aaaba69475f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="R731aab57235646bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb600bf9b84da487b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R946eb202880d4463"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="Rb921e879bc4a4de7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R2e58fba31a634b41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="Rb1698d7894e0402b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="R39d20af021ba47de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="R3a0cb10eca554a56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="Rd789b09492674871"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="R1409a4d1667e47dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="Rd9e04fb9bf1f4aac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="R53118ec982264c6b"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Add first week platform launch brief
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R36a68556e77a494e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R4667c199d2634be0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="R99c9ac1ebc0446bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="R1b07c47ec595464f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R102d3940c1fa4600"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rc8c6a82d23674d7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="R96a1a9ab69484778"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="Rf4f6a40a463d461f"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Expand platform launch briefs to full campaign
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R102d3940c1fa4600"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rc8c6a82d23674d7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="R96a1a9ab69484778"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="Rf4f6a40a463d461f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3ff384ea971d42a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R2eafaedc5a61458a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="Rb3357453be7046e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="R99db3d90710a4e8d"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Add promotion revenue decision matrix
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3ff384ea971d42a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R2eafaedc5a61458a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="Rb3357453be7046e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="R99db3d90710a4e8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R9c6ec218182e431b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rca3a44e3c22846fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="R359a39d936e442e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="Rcb36c8c937244d6d"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Normalize promotion workbook after decision matrix
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R9c6ec218182e431b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rca3a44e3c22846fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="R359a39d936e442e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="Rcb36c8c937244d6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4f8be8bbb3b04809"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rd8139c4d4ff34bcc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="R50d18d77a1d5491e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="Rd49b1d2cfdbd4604"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Add guardian monetization asset backlog
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4f8be8bbb3b04809"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rd8139c4d4ff34bcc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="R50d18d77a1d5491e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="Rd49b1d2cfdbd4604"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R63acb63ff43f425c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R6e903379bfe44d31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="Re57b428e79ca4307"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="Rc5930c5212c04923"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Add now asset production pack
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R63acb63ff43f425c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R6e903379bfe44d31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="Re57b428e79ca4307"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="Rc5930c5212c04923"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R2b05bf2827724790"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R4154cf2164bc4204"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="R2834446cbdc0428a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="Rd70588afa2bd4328"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Add now asset production queue
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R2b05bf2827724790"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R4154cf2164bc4204"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="R2834446cbdc0428a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="Rd70588afa2bd4328"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb882a52617ad4dff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R5001ca5835dc47d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="Rf27be89481c640b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="R3de6b6712504422e"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Add now asset production briefs
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb882a52617ad4dff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R5001ca5835dc47d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="Rf27be89481c640b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="R3de6b6712504422e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Reb276cdcee374ec0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Raf54da9e2ccc4d6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="R777564a3ebc545e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="R210b864e1bb84013"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Add platform profile launch setup
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Reb276cdcee374ec0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Raf54da9e2ccc4d6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="R777564a3ebc545e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="R210b864e1bb84013"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R308b4e46a07049f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rf35ea0a3063e4a57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="R97e45591b9674dba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="Rd7b70bd1db314a3f"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Expose platform profile setup in promotion kit
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R308b4e46a07049f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rf35ea0a3063e4a57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="R97e45591b9674dba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="Rd7b70bd1db314a3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb4c49914f5ee4bb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R6b20303a81a04e13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="R2b4687cba289487b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="R553f42a4724e4ecf"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Add platform profile KPI tracker
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb4c49914f5ee4bb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R6b20303a81a04e13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="R2b4687cba289487b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="R553f42a4724e4ecf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R71aad862421a4411"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rfb9e699861594a69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="R77394362d9f74685"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="R509530247ce54f81"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Include platform profile metrics in weekly summary
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R71aad862421a4411"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rfb9e699861594a69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="R77394362d9f74685"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="R509530247ce54f81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R04f01ef97b604aaf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rc364a179d7254953"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="R11a630da9af14d26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="Rc44588ed810d4ab4"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Include platform profile intent in revenue matrix
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R04f01ef97b604aaf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rc364a179d7254953"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="R11a630da9af14d26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="Rc44588ed810d4ab4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R79524dbcb8444f26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Reb979b0cf2fe4f1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="R864271dabf3f4703"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="Rceb780e09e444ce4"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Surface platform profile setup in next actions
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R79524dbcb8444f26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Reb979b0cf2fe4f1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="R864271dabf3f4703"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="Rceb780e09e444ce4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R52b4b51d0dd647a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Re46d6d7bcc624b6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="Ra911313bdb6840d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="Rdc6347da1a75471f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -328,9 +328,25 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>發布前同步完成 YouTube、TikTok、Instagram 的 Bio/Profile link，使用平台專屬 UTM。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>平台首頁設定後回填 platform-profile-tracker.csv 的 status、profile_link_set_date、profile_clicks、site_clicks、quiz_starts、quiz_completions。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
         <x:v>medium</x:v>
       </x:c>
-      <x:c r="B19" t="str">
+      <x:c r="B21" t="str">
         <x:v>目前沒有回填數據，不調整商品、守護者優先序或付費 CTA。</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Add weekly promotion execution sheets
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R52b4b51d0dd647a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Re46d6d7bcc624b6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="Ra911313bdb6840d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="Rdc6347da1a75471f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Raa1c57dfcadd45aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rb99efa0640a04083"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="R088e080180204f83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="R705dbce8871d4039"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Add execution tabs to promotion workbook
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,10 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Raa1c57dfcadd45aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rb99efa0640a04083"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="3" r:id="R088e080180204f83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="4" r:id="R705dbce8871d4039"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R56df33bfb522424a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rc7532a120c39422f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="Rf58cf532355a44c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="4" r:id="R7a7be3db56884f32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="5" r:id="R255e0c797cce490c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="6" r:id="R7ace26f1d50444ce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -226,59 +228,59 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>Empty data safety mode</x:v>
-      </x:c>
-      <x:c r="B5" t="str">
-        <x:v>YES</x:v>
+        <x:v>Platform profile rows with activity</x:v>
+      </x:c>
+      <x:c r="B5" t="n">
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" t="str"/>
-      <x:c r="B6" t="str"/>
+      <x:c r="A6" t="str">
+        <x:v>Platform profile rows total</x:v>
+      </x:c>
+      <x:c r="B6" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>Metric</x:v>
-      </x:c>
-      <x:c r="B7" t="str">
-        <x:v>Value</x:v>
+        <x:v>Week 1 profile gates pending</x:v>
+      </x:c>
+      <x:c r="B7" t="n">
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>Views</x:v>
+        <x:v>Week 1 platform posts</x:v>
       </x:c>
       <x:c r="B8" t="n">
-        <x:v>0</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>Site clicks</x:v>
-      </x:c>
-      <x:c r="B9" t="n">
-        <x:v>0</x:v>
+        <x:v>Empty data safety mode</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>YES</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" t="str">
-        <x:v>Quiz starts</x:v>
-      </x:c>
-      <x:c r="B10" t="n">
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="A10" t="str"/>
+      <x:c r="B10" t="str"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
-        <x:v>Quiz completions</x:v>
-      </x:c>
-      <x:c r="B11" t="n">
-        <x:v>0</x:v>
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>Value</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
-        <x:v>Route interest</x:v>
+        <x:v>Views</x:v>
       </x:c>
       <x:c r="B12" t="n">
         <x:v>0</x:v>
@@ -286,7 +288,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
-        <x:v>Revenue intent</x:v>
+        <x:v>Site clicks</x:v>
       </x:c>
       <x:c r="B13" t="n">
         <x:v>0</x:v>
@@ -294,59 +296,91 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
-        <x:v>Lead intent</x:v>
+        <x:v>Quiz starts</x:v>
       </x:c>
       <x:c r="B14" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" t="str"/>
-      <x:c r="B15" t="str"/>
+      <x:c r="A15" t="str">
+        <x:v>Quiz completions</x:v>
+      </x:c>
+      <x:c r="B15" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
-        <x:v>Recommended actions</x:v>
-      </x:c>
-      <x:c r="B16" t="str"/>
+        <x:v>Route interest</x:v>
+      </x:c>
+      <x:c r="B16" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">
-        <x:v>high</x:v>
-      </x:c>
-      <x:c r="B17" t="str">
-        <x:v>發布 Week 1 前 3 支 Shorts，先取得測驗完成樣本。</x:v>
+        <x:v>Revenue intent</x:v>
+      </x:c>
+      <x:c r="B17" t="n">
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="str">
-        <x:v>high</x:v>
-      </x:c>
-      <x:c r="B18" t="str">
-        <x:v>發布後至少回填 post_url、site_clicks、quiz_starts、quiz_completions。</x:v>
+        <x:v>Lead intent</x:v>
+      </x:c>
+      <x:c r="B18" t="n">
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" t="str">
-        <x:v>high</x:v>
-      </x:c>
-      <x:c r="B19" t="str">
-        <x:v>發布前同步完成 YouTube、TikTok、Instagram 的 Bio/Profile link，使用平台專屬 UTM。</x:v>
-      </x:c>
+      <x:c r="A19" t="str"/>
+      <x:c r="B19" t="str"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" t="str">
-        <x:v>high</x:v>
-      </x:c>
-      <x:c r="B20" t="str">
-        <x:v>平台首頁設定後回填 platform-profile-tracker.csv 的 status、profile_link_set_date、profile_clicks、site_clicks、quiz_starts、quiz_completions。</x:v>
-      </x:c>
+        <x:v>Recommended actions</x:v>
+      </x:c>
+      <x:c r="B20" t="str"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>發布 Week 1 前 3 支 Shorts，先取得測驗完成樣本。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>發布後至少回填 post_url、site_clicks、quiz_starts、quiz_completions。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>發布前同步完成 YouTube、TikTok、Instagram 的 Bio/Profile link，使用平台專屬 UTM。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>平台首頁設定後回填 platform-profile-tracker.csv 的 status、profile_link_set_date、profile_clicks、site_clicks、quiz_starts、quiz_completions。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="str">
         <x:v>medium</x:v>
       </x:c>
-      <x:c r="B21" t="str">
+      <x:c r="B25" t="str">
         <x:v>目前沒有回填數據，不調整商品、守護者優先序或付費 CTA。</x:v>
       </x:c>
     </x:row>
@@ -1260,166 +1294,208 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
-        <x:v>taskId</x:v>
+        <x:v>platform</x:v>
       </x:c>
       <x:c r="B1" t="str">
-        <x:v>week</x:v>
+        <x:v>label</x:v>
       </x:c>
       <x:c r="C1" t="str">
-        <x:v>slot</x:v>
+        <x:v>profile_link</x:v>
       </x:c>
       <x:c r="D1" t="str">
-        <x:v>guardianId</x:v>
+        <x:v>utm_source</x:v>
       </x:c>
       <x:c r="E1" t="str">
-        <x:v>guardianName</x:v>
+        <x:v>utm_medium</x:v>
       </x:c>
       <x:c r="F1" t="str">
-        <x:v>contentAngle</x:v>
+        <x:v>utm_campaign</x:v>
       </x:c>
       <x:c r="G1" t="str">
-        <x:v>title</x:v>
+        <x:v>utm_content</x:v>
       </x:c>
       <x:c r="H1" t="str">
-        <x:v>trackedUrl</x:v>
+        <x:v>status</x:v>
       </x:c>
       <x:c r="I1" t="str">
-        <x:v>primaryFreeItemId</x:v>
+        <x:v>profile_link_set_date</x:v>
       </x:c>
       <x:c r="J1" t="str">
-        <x:v>ownedLeadItemId</x:v>
+        <x:v>profile_clicks</x:v>
       </x:c>
       <x:c r="K1" t="str">
-        <x:v>supplyRoute</x:v>
+        <x:v>site_clicks</x:v>
       </x:c>
       <x:c r="L1" t="str">
-        <x:v>lunaScene</x:v>
+        <x:v>quiz_starts</x:v>
       </x:c>
       <x:c r="M1" t="str">
-        <x:v>keepsake</x:v>
+        <x:v>quiz_completions</x:v>
+      </x:c>
+      <x:c r="N1" t="str">
+        <x:v>guardian_result_clicks</x:v>
+      </x:c>
+      <x:c r="O1" t="str">
+        <x:v>resources_clicks</x:v>
+      </x:c>
+      <x:c r="P1" t="str">
+        <x:v>repair_plan_clicks</x:v>
+      </x:c>
+      <x:c r="Q1" t="str">
+        <x:v>luna_clicks</x:v>
+      </x:c>
+      <x:c r="R1" t="str">
+        <x:v>keepsake_clicks</x:v>
+      </x:c>
+      <x:c r="S1" t="str">
+        <x:v>free_keepsake_downloads</x:v>
+      </x:c>
+      <x:c r="T1" t="str">
+        <x:v>supply_lead_requests</x:v>
+      </x:c>
+      <x:c r="U1" t="str">
+        <x:v>luna_pack_clicks</x:v>
+      </x:c>
+      <x:c r="V1" t="str">
+        <x:v>affiliate_book_clicks</x:v>
+      </x:c>
+      <x:c r="W1" t="str">
+        <x:v>contact_requests</x:v>
+      </x:c>
+      <x:c r="X1" t="str">
+        <x:v>notes</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>publish-lt-s01-iris-silence</x:v>
-      </x:c>
-      <x:c r="B2" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C2" t="n">
-        <x:v>1</x:v>
+        <x:v>youtube_shorts</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>YouTube Shorts</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=youtube&amp;utm_medium=social_profile&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=youtube_shorts_bio</x:v>
       </x:c>
       <x:c r="D2" t="str">
-        <x:v>iris</x:v>
+        <x:v>youtube</x:v>
       </x:c>
       <x:c r="E2" t="str">
-        <x:v>艾莉絲</x:v>
+        <x:v>social_profile</x:v>
       </x:c>
       <x:c r="F2" t="str">
-        <x:v>情感錯頻情境</x:v>
+        <x:v>first_round_quiz_completion</x:v>
       </x:c>
       <x:c r="G2" t="str">
-        <x:v>他沉默時，你最想聽見哪一句話？</x:v>
+        <x:v>youtube_shorts_bio</x:v>
       </x:c>
       <x:c r="H2" t="str">
-        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_silence</x:v>
-      </x:c>
-      <x:c r="I2" t="str">
-        <x:v>free-keepsake-iris</x:v>
-      </x:c>
-      <x:c r="J2" t="str">
-        <x:v>supply-wishlist-iris</x:v>
-      </x:c>
-      <x:c r="K2" t="str">
-        <x:v>https://lovetypes.tw/resources/#supply-iris</x:v>
-      </x:c>
-      <x:c r="L2" t="str">
-        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-iris</x:v>
-      </x:c>
-      <x:c r="M2" t="str">
-        <x:v>https://lovetypes.tw/keepsakes/#keepsake-iris</x:v>
+        <x:v>planned</x:v>
+      </x:c>
+      <x:c r="I2" t="str"/>
+      <x:c r="J2" t="str"/>
+      <x:c r="K2" t="str"/>
+      <x:c r="L2" t="str"/>
+      <x:c r="M2" t="str"/>
+      <x:c r="N2" t="str"/>
+      <x:c r="O2" t="str"/>
+      <x:c r="P2" t="str"/>
+      <x:c r="Q2" t="str"/>
+      <x:c r="R2" t="str"/>
+      <x:c r="S2" t="str"/>
+      <x:c r="T2" t="str"/>
+      <x:c r="U2" t="str"/>
+      <x:c r="V2" t="str"/>
+      <x:c r="W2" t="str"/>
+      <x:c r="X2" t="str">
+        <x:v>YouTube 說明欄可放完整追蹤連結；置頂留言也放同一條。</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>publish-lt-s02-iris-affirmation</x:v>
-      </x:c>
-      <x:c r="B3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C3" t="n">
-        <x:v>2</x:v>
+        <x:v>tiktok</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>TikTok</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=tiktok&amp;utm_medium=social_profile&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=tiktok_bio</x:v>
       </x:c>
       <x:c r="D3" t="str">
-        <x:v>iris</x:v>
+        <x:v>tiktok</x:v>
       </x:c>
       <x:c r="E3" t="str">
-        <x:v>艾莉絲</x:v>
+        <x:v>social_profile</x:v>
       </x:c>
       <x:c r="F3" t="str">
-        <x:v>守護者人格認同</x:v>
+        <x:v>first_round_quiz_completion</x:v>
       </x:c>
       <x:c r="G3" t="str">
-        <x:v>哪一句肯定，會讓你瞬間安心？</x:v>
+        <x:v>tiktok_bio</x:v>
       </x:c>
       <x:c r="H3" t="str">
-        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_affirmation</x:v>
-      </x:c>
-      <x:c r="I3" t="str">
-        <x:v>free-keepsake-iris</x:v>
-      </x:c>
-      <x:c r="J3" t="str">
-        <x:v>supply-wishlist-iris</x:v>
-      </x:c>
-      <x:c r="K3" t="str">
-        <x:v>https://lovetypes.tw/resources/#supply-iris</x:v>
-      </x:c>
-      <x:c r="L3" t="str">
-        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-iris</x:v>
-      </x:c>
-      <x:c r="M3" t="str">
-        <x:v>https://lovetypes.tw/keepsakes/#keepsake-iris</x:v>
+        <x:v>planned</x:v>
+      </x:c>
+      <x:c r="I3" t="str"/>
+      <x:c r="J3" t="str"/>
+      <x:c r="K3" t="str"/>
+      <x:c r="L3" t="str"/>
+      <x:c r="M3" t="str"/>
+      <x:c r="N3" t="str"/>
+      <x:c r="O3" t="str"/>
+      <x:c r="P3" t="str"/>
+      <x:c r="Q3" t="str"/>
+      <x:c r="R3" t="str"/>
+      <x:c r="S3" t="str"/>
+      <x:c r="T3" t="str"/>
+      <x:c r="U3" t="str"/>
+      <x:c r="V3" t="str"/>
+      <x:c r="W3" t="str"/>
+      <x:c r="X3" t="str">
+        <x:v>若 caption 不能放可點連結，Bio/個人頁連結必須使用平台專屬追蹤連結。</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>publish-lt-s03-iris-too-sensitive</x:v>
-      </x:c>
-      <x:c r="B4" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C4" t="n">
-        <x:v>3</x:v>
+        <x:v>instagram_reels</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>Instagram Reels</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=instagram&amp;utm_medium=social_profile&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=instagram_reels_bio</x:v>
       </x:c>
       <x:c r="D4" t="str">
-        <x:v>iris</x:v>
+        <x:v>instagram</x:v>
       </x:c>
       <x:c r="E4" t="str">
-        <x:v>艾莉絲</x:v>
+        <x:v>social_profile</x:v>
       </x:c>
       <x:c r="F4" t="str">
-        <x:v>測驗入口</x:v>
+        <x:v>first_round_quiz_completion</x:v>
       </x:c>
       <x:c r="G4" t="str">
-        <x:v>你真的太敏感嗎？還是你只是等一句清楚的話？</x:v>
+        <x:v>instagram_reels_bio</x:v>
       </x:c>
       <x:c r="H4" t="str">
-        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_too_sensitive</x:v>
-      </x:c>
-      <x:c r="I4" t="str">
-        <x:v>free-keepsake-iris</x:v>
-      </x:c>
-      <x:c r="J4" t="str">
-        <x:v>supply-wishlist-iris</x:v>
-      </x:c>
-      <x:c r="K4" t="str">
-        <x:v>https://lovetypes.tw/resources/#supply-iris</x:v>
-      </x:c>
-      <x:c r="L4" t="str">
-        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-iris</x:v>
-      </x:c>
-      <x:c r="M4" t="str">
-        <x:v>https://lovetypes.tw/keepsakes/#keepsake-iris</x:v>
+        <x:v>planned</x:v>
+      </x:c>
+      <x:c r="I4" t="str"/>
+      <x:c r="J4" t="str"/>
+      <x:c r="K4" t="str"/>
+      <x:c r="L4" t="str"/>
+      <x:c r="M4" t="str"/>
+      <x:c r="N4" t="str"/>
+      <x:c r="O4" t="str"/>
+      <x:c r="P4" t="str"/>
+      <x:c r="Q4" t="str"/>
+      <x:c r="R4" t="str"/>
+      <x:c r="S4" t="str"/>
+      <x:c r="T4" t="str"/>
+      <x:c r="U4" t="str"/>
+      <x:c r="V4" t="str"/>
+      <x:c r="W4" t="str"/>
+      <x:c r="X4" t="str">
+        <x:v>IG Reels caption 以個人檔案連結承接；Bio 連結需先於發布前更新。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1433,6 +1509,883 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
+        <x:v>Week 1 Profile Gates</x:v>
+      </x:c>
+      <x:c r="B1" t="str"/>
+      <x:c r="C1" t="str"/>
+      <x:c r="D1" t="str"/>
+      <x:c r="E1" t="str"/>
+      <x:c r="F1" t="str"/>
+      <x:c r="G1" t="str"/>
+      <x:c r="H1" t="str"/>
+      <x:c r="I1" t="str"/>
+      <x:c r="J1" t="str"/>
+      <x:c r="K1" t="str"/>
+      <x:c r="L1" t="str"/>
+      <x:c r="M1" t="str"/>
+      <x:c r="N1" t="str"/>
+      <x:c r="O1" t="str"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>platform</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>label</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="E2" t="str">
+        <x:v>profileLinkLabel</x:v>
+      </x:c>
+      <x:c r="F2" t="str">
+        <x:v>profileLink</x:v>
+      </x:c>
+      <x:c r="G2" t="str">
+        <x:v>bio</x:v>
+      </x:c>
+      <x:c r="H2" t="str">
+        <x:v>pinnedComment</x:v>
+      </x:c>
+      <x:c r="I2" t="str">
+        <x:v>writeback</x:v>
+      </x:c>
+      <x:c r="J2" t="str"/>
+      <x:c r="K2" t="str"/>
+      <x:c r="L2" t="str"/>
+      <x:c r="M2" t="str"/>
+      <x:c r="N2" t="str"/>
+      <x:c r="O2" t="str"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>youtube_shorts</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>YouTube Shorts</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>planned</x:v>
+      </x:c>
+      <x:c r="E3" t="str">
+        <x:v>Channel description / video description</x:v>
+      </x:c>
+      <x:c r="F3" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=youtube&amp;utm_medium=social_profile&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=youtube_shorts_bio</x:v>
+      </x:c>
+      <x:c r="G3" t="str">
+        <x:v>LoveTypes 心語庭園｜完成 15 題測驗，找到你的情感守護者。</x:v>
+      </x:c>
+      <x:c r="H3" t="str">
+        <x:v>完成 15 題測驗，找到你的情感守護者：https://lovetypes.tw/start/?utm_source=youtube&amp;utm_medium=social_profile&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=youtube_shorts_bio
+留言 A/B/C，我們會用守護者路線回覆你。</x:v>
+      </x:c>
+      <x:c r="I3" t="str">
+        <x:v>status=set/live, profile_link_set_date, profile_clicks, site_clicks, quiz_starts, quiz_completions</x:v>
+      </x:c>
+      <x:c r="J3" t="str"/>
+      <x:c r="K3" t="str"/>
+      <x:c r="L3" t="str"/>
+      <x:c r="M3" t="str"/>
+      <x:c r="N3" t="str"/>
+      <x:c r="O3" t="str"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>tiktok</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>TikTok</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>planned</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>Profile website link</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=tiktok&amp;utm_medium=social_profile&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=tiktok_bio</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>五種愛之語測驗｜進入心語庭園，找到你的情感守護者。</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>完成 15 題測驗，找到你的情感守護者。入口在個人頁連結。
+留言 A/B/C，選出最像你的心語。</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>status=set/live, profile_link_set_date, profile_clicks, site_clicks, quiz_starts, quiz_completions</x:v>
+      </x:c>
+      <x:c r="J4" t="str"/>
+      <x:c r="K4" t="str"/>
+      <x:c r="L4" t="str"/>
+      <x:c r="M4" t="str"/>
+      <x:c r="N4" t="str"/>
+      <x:c r="O4" t="str"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>instagram_reels</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>Instagram Reels</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>planned</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>Profile link in bio</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=instagram&amp;utm_medium=social_profile&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=instagram_reels_bio</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
+        <x:v>LoveTypes 心語庭園｜15 題找到你的情感守護者。</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
+        <x:v>完成 15 題測驗，找到你的情感守護者。入口在個人檔案連結。
+留言你的 A/B/C，讓守護者把心語接住。</x:v>
+      </x:c>
+      <x:c r="I5" t="str">
+        <x:v>status=set/live, profile_link_set_date, profile_clicks, site_clicks, quiz_starts, quiz_completions</x:v>
+      </x:c>
+      <x:c r="J5" t="str"/>
+      <x:c r="K5" t="str"/>
+      <x:c r="L5" t="str"/>
+      <x:c r="M5" t="str"/>
+      <x:c r="N5" t="str"/>
+      <x:c r="O5" t="str"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str"/>
+      <x:c r="B6" t="str"/>
+      <x:c r="C6" t="str"/>
+      <x:c r="D6" t="str"/>
+      <x:c r="E6" t="str"/>
+      <x:c r="F6" t="str"/>
+      <x:c r="G6" t="str"/>
+      <x:c r="H6" t="str"/>
+      <x:c r="I6" t="str"/>
+      <x:c r="J6" t="str"/>
+      <x:c r="K6" t="str"/>
+      <x:c r="L6" t="str"/>
+      <x:c r="M6" t="str"/>
+      <x:c r="N6" t="str"/>
+      <x:c r="O6" t="str"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>Week 1 Platform Posts</x:v>
+      </x:c>
+      <x:c r="B7" t="str"/>
+      <x:c r="C7" t="str"/>
+      <x:c r="D7" t="str"/>
+      <x:c r="E7" t="str"/>
+      <x:c r="F7" t="str"/>
+      <x:c r="G7" t="str"/>
+      <x:c r="H7" t="str"/>
+      <x:c r="I7" t="str"/>
+      <x:c r="J7" t="str"/>
+      <x:c r="K7" t="str"/>
+      <x:c r="L7" t="str"/>
+      <x:c r="M7" t="str"/>
+      <x:c r="N7" t="str"/>
+      <x:c r="O7" t="str"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>week</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>taskId</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>scriptId</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>guardianId</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>guardianName</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>contentAngle</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>title</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>platform</x:v>
+      </x:c>
+      <x:c r="I8" t="str">
+        <x:v>label</x:v>
+      </x:c>
+      <x:c r="J8" t="str">
+        <x:v>scheduledDate</x:v>
+      </x:c>
+      <x:c r="K8" t="str">
+        <x:v>scheduledTime</x:v>
+      </x:c>
+      <x:c r="L8" t="str">
+        <x:v>timezone</x:v>
+      </x:c>
+      <x:c r="M8" t="str">
+        <x:v>trackedUrl</x:v>
+      </x:c>
+      <x:c r="N8" t="str">
+        <x:v>caption</x:v>
+      </x:c>
+      <x:c r="O8" t="str">
+        <x:v>writeback</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>publish-lt-s01-iris-silence</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>lt-s01-iris-silence</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>情感錯頻情境</x:v>
+      </x:c>
+      <x:c r="G9" t="str">
+        <x:v>他沉默時，你最想聽見哪一句話？</x:v>
+      </x:c>
+      <x:c r="H9" t="str">
+        <x:v>youtube_shorts</x:v>
+      </x:c>
+      <x:c r="I9" t="str">
+        <x:v>YouTube Shorts</x:v>
+      </x:c>
+      <x:c r="J9" t="str">
+        <x:v>2026-06-15</x:v>
+      </x:c>
+      <x:c r="K9" t="str">
+        <x:v>20:30</x:v>
+      </x:c>
+      <x:c r="L9" t="str">
+        <x:v>Asia/Taipei</x:v>
+      </x:c>
+      <x:c r="M9" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_silence</x:v>
+      </x:c>
+      <x:c r="N9" t="str">
+        <x:v>你不是想聽甜言蜜語，你只是想確認自己有沒有被看見。
+完成 15 題測驗，找到你的情感守護者：https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_silence
+留言 A/B/C，或寫下一句你最想被說出口的話。
+#五種愛之語測驗 #情感守護者 #心語庭園 #錯頻修復 #LoveTypes</x:v>
+      </x:c>
+      <x:c r="O9" t="str">
+        <x:v>status=published, published_date, post_url, site_clicks, quiz_starts, quiz_completions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>publish-lt-s01-iris-silence</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>lt-s01-iris-silence</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>情感錯頻情境</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>他沉默時，你最想聽見哪一句話？</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>tiktok</x:v>
+      </x:c>
+      <x:c r="I10" t="str">
+        <x:v>TikTok</x:v>
+      </x:c>
+      <x:c r="J10" t="str">
+        <x:v>2026-06-15</x:v>
+      </x:c>
+      <x:c r="K10" t="str">
+        <x:v>21:00</x:v>
+      </x:c>
+      <x:c r="L10" t="str">
+        <x:v>Asia/Taipei</x:v>
+      </x:c>
+      <x:c r="M10" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_silence</x:v>
+      </x:c>
+      <x:c r="N10" t="str">
+        <x:v>你不是想聽甜言蜜語，你只是想確認自己有沒有被看見。
+首頁連結完成 15 題測驗：https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_silence
+留言 A/B/C，或寫下一句你最想被說出口的話。
+#五種愛之語測驗 #情感守護者 #心語庭園 #錯頻修復 #LoveTypes</x:v>
+      </x:c>
+      <x:c r="O10" t="str">
+        <x:v>status=published, published_date, post_url, site_clicks, quiz_starts, quiz_completions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>publish-lt-s01-iris-silence</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>lt-s01-iris-silence</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>情感錯頻情境</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>他沉默時，你最想聽見哪一句話？</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>instagram_reels</x:v>
+      </x:c>
+      <x:c r="I11" t="str">
+        <x:v>Instagram Reels</x:v>
+      </x:c>
+      <x:c r="J11" t="str">
+        <x:v>2026-06-15</x:v>
+      </x:c>
+      <x:c r="K11" t="str">
+        <x:v>21:30</x:v>
+      </x:c>
+      <x:c r="L11" t="str">
+        <x:v>Asia/Taipei</x:v>
+      </x:c>
+      <x:c r="M11" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_silence</x:v>
+      </x:c>
+      <x:c r="N11" t="str">
+        <x:v>你不是想聽甜言蜜語，你只是想確認自己有沒有被看見。
+個人檔案連結完成 15 題測驗：https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_silence
+留言 A/B/C，或寫下一句你最想被說出口的話。
+#五種愛之語測驗 #情感守護者 #心語庭園 #錯頻修復 #LoveTypes</x:v>
+      </x:c>
+      <x:c r="O11" t="str">
+        <x:v>status=published, published_date, post_url, site_clicks, quiz_starts, quiz_completions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>publish-lt-s02-iris-affirmation</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>lt-s02-iris-affirmation</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>守護者人格認同</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>哪一句肯定，會讓你瞬間安心？</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>youtube_shorts</x:v>
+      </x:c>
+      <x:c r="I12" t="str">
+        <x:v>YouTube Shorts</x:v>
+      </x:c>
+      <x:c r="J12" t="str">
+        <x:v>2026-06-17</x:v>
+      </x:c>
+      <x:c r="K12" t="str">
+        <x:v>20:30</x:v>
+      </x:c>
+      <x:c r="L12" t="str">
+        <x:v>Asia/Taipei</x:v>
+      </x:c>
+      <x:c r="M12" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_affirmation</x:v>
+      </x:c>
+      <x:c r="N12" t="str">
+        <x:v>真正的肯定，不是把你說得完美，而是讓你知道自己被看見。
+完成 15 題測驗，找到你的情感守護者：https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_affirmation
+留言你選的句子，艾莉絲會把它收進晨曦玻璃花園。
+#五種愛之語測驗 #情感守護者 #心語庭園 #錯頻修復 #LoveTypes</x:v>
+      </x:c>
+      <x:c r="O12" t="str">
+        <x:v>status=published, published_date, post_url, site_clicks, quiz_starts, quiz_completions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>publish-lt-s02-iris-affirmation</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>lt-s02-iris-affirmation</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>守護者人格認同</x:v>
+      </x:c>
+      <x:c r="G13" t="str">
+        <x:v>哪一句肯定，會讓你瞬間安心？</x:v>
+      </x:c>
+      <x:c r="H13" t="str">
+        <x:v>tiktok</x:v>
+      </x:c>
+      <x:c r="I13" t="str">
+        <x:v>TikTok</x:v>
+      </x:c>
+      <x:c r="J13" t="str">
+        <x:v>2026-06-17</x:v>
+      </x:c>
+      <x:c r="K13" t="str">
+        <x:v>21:00</x:v>
+      </x:c>
+      <x:c r="L13" t="str">
+        <x:v>Asia/Taipei</x:v>
+      </x:c>
+      <x:c r="M13" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_affirmation</x:v>
+      </x:c>
+      <x:c r="N13" t="str">
+        <x:v>真正的肯定，不是把你說得完美，而是讓你知道自己被看見。
+首頁連結完成 15 題測驗：https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_affirmation
+留言你選的句子，艾莉絲會把它收進晨曦玻璃花園。
+#五種愛之語測驗 #情感守護者 #心語庭園 #錯頻修復 #LoveTypes</x:v>
+      </x:c>
+      <x:c r="O13" t="str">
+        <x:v>status=published, published_date, post_url, site_clicks, quiz_starts, quiz_completions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>publish-lt-s02-iris-affirmation</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>lt-s02-iris-affirmation</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>守護者人格認同</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>哪一句肯定，會讓你瞬間安心？</x:v>
+      </x:c>
+      <x:c r="H14" t="str">
+        <x:v>instagram_reels</x:v>
+      </x:c>
+      <x:c r="I14" t="str">
+        <x:v>Instagram Reels</x:v>
+      </x:c>
+      <x:c r="J14" t="str">
+        <x:v>2026-06-17</x:v>
+      </x:c>
+      <x:c r="K14" t="str">
+        <x:v>21:30</x:v>
+      </x:c>
+      <x:c r="L14" t="str">
+        <x:v>Asia/Taipei</x:v>
+      </x:c>
+      <x:c r="M14" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_affirmation</x:v>
+      </x:c>
+      <x:c r="N14" t="str">
+        <x:v>真正的肯定，不是把你說得完美，而是讓你知道自己被看見。
+個人檔案連結完成 15 題測驗：https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_affirmation
+留言你選的句子，艾莉絲會把它收進晨曦玻璃花園。
+#五種愛之語測驗 #情感守護者 #心語庭園 #錯頻修復 #LoveTypes</x:v>
+      </x:c>
+      <x:c r="O14" t="str">
+        <x:v>status=published, published_date, post_url, site_clicks, quiz_starts, quiz_completions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>publish-lt-s03-iris-too-sensitive</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>lt-s03-iris-too-sensitive</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
+        <x:v>測驗入口</x:v>
+      </x:c>
+      <x:c r="G15" t="str">
+        <x:v>你真的太敏感嗎？還是你只是等一句清楚的話？</x:v>
+      </x:c>
+      <x:c r="H15" t="str">
+        <x:v>youtube_shorts</x:v>
+      </x:c>
+      <x:c r="I15" t="str">
+        <x:v>YouTube Shorts</x:v>
+      </x:c>
+      <x:c r="J15" t="str">
+        <x:v>2026-06-19</x:v>
+      </x:c>
+      <x:c r="K15" t="str">
+        <x:v>20:30</x:v>
+      </x:c>
+      <x:c r="L15" t="str">
+        <x:v>Asia/Taipei</x:v>
+      </x:c>
+      <x:c r="M15" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_too_sensitive</x:v>
+      </x:c>
+      <x:c r="N15" t="str">
+        <x:v>有時候你不是太敏感，你只是一直在替沉默找理由。
+完成 15 題測驗，找到你的情感守護者：https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_too_sensitive
+留言「我想被清楚回應」，或選 A：等話、B：等行動、C：等陪伴。
+#五種愛之語測驗 #情感守護者 #心語庭園 #錯頻修復 #LoveTypes</x:v>
+      </x:c>
+      <x:c r="O15" t="str">
+        <x:v>status=published, published_date, post_url, site_clicks, quiz_starts, quiz_completions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>publish-lt-s03-iris-too-sensitive</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>lt-s03-iris-too-sensitive</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="E16" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
+        <x:v>測驗入口</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>你真的太敏感嗎？還是你只是等一句清楚的話？</x:v>
+      </x:c>
+      <x:c r="H16" t="str">
+        <x:v>tiktok</x:v>
+      </x:c>
+      <x:c r="I16" t="str">
+        <x:v>TikTok</x:v>
+      </x:c>
+      <x:c r="J16" t="str">
+        <x:v>2026-06-19</x:v>
+      </x:c>
+      <x:c r="K16" t="str">
+        <x:v>21:00</x:v>
+      </x:c>
+      <x:c r="L16" t="str">
+        <x:v>Asia/Taipei</x:v>
+      </x:c>
+      <x:c r="M16" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_too_sensitive</x:v>
+      </x:c>
+      <x:c r="N16" t="str">
+        <x:v>有時候你不是太敏感，你只是一直在替沉默找理由。
+首頁連結完成 15 題測驗：https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_too_sensitive
+留言「我想被清楚回應」，或選 A：等話、B：等行動、C：等陪伴。
+#五種愛之語測驗 #情感守護者 #心語庭園 #錯頻修復 #LoveTypes</x:v>
+      </x:c>
+      <x:c r="O16" t="str">
+        <x:v>status=published, published_date, post_url, site_clicks, quiz_starts, quiz_completions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>publish-lt-s03-iris-too-sensitive</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>lt-s03-iris-too-sensitive</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="E17" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="F17" t="str">
+        <x:v>測驗入口</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>你真的太敏感嗎？還是你只是等一句清楚的話？</x:v>
+      </x:c>
+      <x:c r="H17" t="str">
+        <x:v>instagram_reels</x:v>
+      </x:c>
+      <x:c r="I17" t="str">
+        <x:v>Instagram Reels</x:v>
+      </x:c>
+      <x:c r="J17" t="str">
+        <x:v>2026-06-19</x:v>
+      </x:c>
+      <x:c r="K17" t="str">
+        <x:v>21:30</x:v>
+      </x:c>
+      <x:c r="L17" t="str">
+        <x:v>Asia/Taipei</x:v>
+      </x:c>
+      <x:c r="M17" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_too_sensitive</x:v>
+      </x:c>
+      <x:c r="N17" t="str">
+        <x:v>有時候你不是太敏感，你只是一直在替沉默找理由。
+個人檔案連結完成 15 題測驗：https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_too_sensitive
+留言「我想被清楚回應」，或選 A：等話、B：等行動、C：等陪伴。
+#五種愛之語測驗 #情感守護者 #心語庭園 #錯頻修復 #LoveTypes</x:v>
+      </x:c>
+      <x:c r="O17" t="str">
+        <x:v>status=published, published_date, post_url, site_clicks, quiz_starts, quiz_completions</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
+        <x:v>taskId</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>week</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>slot</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>guardianId</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
+        <x:v>guardianName</x:v>
+      </x:c>
+      <x:c r="F1" t="str">
+        <x:v>contentAngle</x:v>
+      </x:c>
+      <x:c r="G1" t="str">
+        <x:v>title</x:v>
+      </x:c>
+      <x:c r="H1" t="str">
+        <x:v>trackedUrl</x:v>
+      </x:c>
+      <x:c r="I1" t="str">
+        <x:v>primaryFreeItemId</x:v>
+      </x:c>
+      <x:c r="J1" t="str">
+        <x:v>ownedLeadItemId</x:v>
+      </x:c>
+      <x:c r="K1" t="str">
+        <x:v>supplyRoute</x:v>
+      </x:c>
+      <x:c r="L1" t="str">
+        <x:v>lunaScene</x:v>
+      </x:c>
+      <x:c r="M1" t="str">
+        <x:v>keepsake</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>publish-lt-s01-iris-silence</x:v>
+      </x:c>
+      <x:c r="B2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="E2" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="F2" t="str">
+        <x:v>情感錯頻情境</x:v>
+      </x:c>
+      <x:c r="G2" t="str">
+        <x:v>他沉默時，你最想聽見哪一句話？</x:v>
+      </x:c>
+      <x:c r="H2" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_silence</x:v>
+      </x:c>
+      <x:c r="I2" t="str">
+        <x:v>free-keepsake-iris</x:v>
+      </x:c>
+      <x:c r="J2" t="str">
+        <x:v>supply-wishlist-iris</x:v>
+      </x:c>
+      <x:c r="K2" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-iris</x:v>
+      </x:c>
+      <x:c r="L2" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-iris</x:v>
+      </x:c>
+      <x:c r="M2" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-iris</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>publish-lt-s02-iris-affirmation</x:v>
+      </x:c>
+      <x:c r="B3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="E3" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="F3" t="str">
+        <x:v>守護者人格認同</x:v>
+      </x:c>
+      <x:c r="G3" t="str">
+        <x:v>哪一句肯定，會讓你瞬間安心？</x:v>
+      </x:c>
+      <x:c r="H3" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_affirmation</x:v>
+      </x:c>
+      <x:c r="I3" t="str">
+        <x:v>free-keepsake-iris</x:v>
+      </x:c>
+      <x:c r="J3" t="str">
+        <x:v>supply-wishlist-iris</x:v>
+      </x:c>
+      <x:c r="K3" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-iris</x:v>
+      </x:c>
+      <x:c r="L3" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-iris</x:v>
+      </x:c>
+      <x:c r="M3" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-iris</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>publish-lt-s03-iris-too-sensitive</x:v>
+      </x:c>
+      <x:c r="B4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C4" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>測驗入口</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>你真的太敏感嗎？還是你只是等一句清楚的話？</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_too_sensitive</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>free-keepsake-iris</x:v>
+      </x:c>
+      <x:c r="J4" t="str">
+        <x:v>supply-wishlist-iris</x:v>
+      </x:c>
+      <x:c r="K4" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-iris</x:v>
+      </x:c>
+      <x:c r="L4" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-iris</x:v>
+      </x:c>
+      <x:c r="M4" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-iris</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
         <x:v>Field</x:v>
       </x:c>
       <x:c r="B1" t="str">
@@ -1465,41 +2418,57 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>free_keepsake_downloads</x:v>
+        <x:v>profile_clicks</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Guardian identity asset save or print intent.</x:v>
+        <x:v>Clicks on social Bio/Profile links before visitors reach LoveTypes.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>supply_lead_requests</x:v>
+        <x:v>profile_link_set_date</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Owned email/request demand for guardian supply assets.</x:v>
+        <x:v>Date the platform Bio/Profile tracked link was set live.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>luna_pack_clicks</x:v>
+        <x:v>free_keepsake_downloads</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>Luna Gumroad product exploration.</x:v>
+        <x:v>Guardian identity asset save or print intent.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>affiliate_book_clicks</x:v>
+        <x:v>supply_lead_requests</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>Affiliate book route exploration.</x:v>
+        <x:v>Owned email/request demand for guardian supply assets.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
+        <x:v>luna_pack_clicks</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>Luna Gumroad product exploration.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>affiliate_book_clicks</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>Affiliate book route exploration.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
         <x:v>contact_requests</x:v>
       </x:c>
-      <x:c r="B9" t="str">
+      <x:c r="B11" t="str">
         <x:v>High-intent contact or path-summary mailto request.</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Add weekly monetization decision gate
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R56df33bfb522424a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rc7532a120c39422f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="Rf58cf532355a44c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="4" r:id="R7a7be3db56884f32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="5" r:id="R255e0c797cce490c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="6" r:id="R7ace26f1d50444ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rfed0e5e58a604f43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R5d3e604823be4188"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R29923b31a2bb4534"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="4" r:id="R5c64e2d40b1040c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="5" r:id="Rbaa4c16cb1ee4a7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="6" r:id="R27ca93d7dc3a426e"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Add lead intake monetization playbook
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,12 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rfed0e5e58a604f43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R5d3e604823be4188"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R29923b31a2bb4534"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="4" r:id="R5c64e2d40b1040c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="5" r:id="Rbaa4c16cb1ee4a7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="6" r:id="R27ca93d7dc3a426e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R1cb4b1e28cd644b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R23ee90edfbe248d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R49e948f496724a51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R508ac3422f754746"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="5" r:id="R2b381e4b538541bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="6" r:id="R262a1059b9fb41ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="7" r:id="R513fca235f5a4020"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -244,51 +245,51 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>Week 1 profile gates pending</x:v>
+        <x:v>Lead intake template rows</x:v>
       </x:c>
       <x:c r="B7" t="n">
-        <x:v>3</x:v>
+        <x:v>15</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>Week 1 platform posts</x:v>
+        <x:v>Week 1 profile gates pending</x:v>
       </x:c>
       <x:c r="B8" t="n">
-        <x:v>9</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
+        <x:v>Week 1 platform posts</x:v>
+      </x:c>
+      <x:c r="B9" t="n">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
         <x:v>Empty data safety mode</x:v>
       </x:c>
-      <x:c r="B9" t="str">
+      <x:c r="B10" t="str">
         <x:v>YES</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" t="str"/>
-      <x:c r="B10" t="str"/>
-    </x:row>
     <x:row r="11">
-      <x:c r="A11" t="str">
-        <x:v>Metric</x:v>
-      </x:c>
-      <x:c r="B11" t="str">
-        <x:v>Value</x:v>
-      </x:c>
+      <x:c r="A11" t="str"/>
+      <x:c r="B11" t="str"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
-        <x:v>Views</x:v>
-      </x:c>
-      <x:c r="B12" t="n">
-        <x:v>0</x:v>
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>Value</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
-        <x:v>Site clicks</x:v>
+        <x:v>Views</x:v>
       </x:c>
       <x:c r="B13" t="n">
         <x:v>0</x:v>
@@ -296,7 +297,7 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
-        <x:v>Quiz starts</x:v>
+        <x:v>Site clicks</x:v>
       </x:c>
       <x:c r="B14" t="n">
         <x:v>0</x:v>
@@ -304,7 +305,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
-        <x:v>Quiz completions</x:v>
+        <x:v>Quiz starts</x:v>
       </x:c>
       <x:c r="B15" t="n">
         <x:v>0</x:v>
@@ -312,7 +313,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
-        <x:v>Route interest</x:v>
+        <x:v>Quiz completions</x:v>
       </x:c>
       <x:c r="B16" t="n">
         <x:v>0</x:v>
@@ -320,7 +321,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">
-        <x:v>Revenue intent</x:v>
+        <x:v>Route interest</x:v>
       </x:c>
       <x:c r="B17" t="n">
         <x:v>0</x:v>
@@ -328,36 +329,36 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="str">
-        <x:v>Lead intent</x:v>
+        <x:v>Revenue intent</x:v>
       </x:c>
       <x:c r="B18" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" t="str"/>
-      <x:c r="B19" t="str"/>
+      <x:c r="A19" t="str">
+        <x:v>Lead intent</x:v>
+      </x:c>
+      <x:c r="B19" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" t="str">
-        <x:v>Recommended actions</x:v>
-      </x:c>
+      <x:c r="A20" t="str"/>
       <x:c r="B20" t="str"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" t="str">
-        <x:v>high</x:v>
-      </x:c>
-      <x:c r="B21" t="str">
-        <x:v>發布 Week 1 前 3 支 Shorts，先取得測驗完成樣本。</x:v>
-      </x:c>
+        <x:v>Recommended actions</x:v>
+      </x:c>
+      <x:c r="B21" t="str"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="B22" t="str">
-        <x:v>發布後至少回填 post_url、site_clicks、quiz_starts、quiz_completions。</x:v>
+        <x:v>發布 Week 1 前 3 支 Shorts，先取得測驗完成樣本。</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -365,7 +366,7 @@
         <x:v>high</x:v>
       </x:c>
       <x:c r="B23" t="str">
-        <x:v>發布前同步完成 YouTube、TikTok、Instagram 的 Bio/Profile link，使用平台專屬 UTM。</x:v>
+        <x:v>發布後至少回填 post_url、site_clicks、quiz_starts、quiz_completions。</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -373,14 +374,22 @@
         <x:v>high</x:v>
       </x:c>
       <x:c r="B24" t="str">
-        <x:v>平台首頁設定後回填 platform-profile-tracker.csv 的 status、profile_link_set_date、profile_clicks、site_clicks、quiz_starts、quiz_completions。</x:v>
+        <x:v>發布前同步完成 YouTube、TikTok、Instagram 的 Bio/Profile link，使用平台專屬 UTM。</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>平台首頁設定後回填 platform-profile-tracker.csv 的 status、profile_link_set_date、profile_clicks、site_clicks、quiz_starts、quiz_completions。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="str">
         <x:v>medium</x:v>
       </x:c>
-      <x:c r="B25" t="str">
+      <x:c r="B26" t="str">
         <x:v>目前沒有回填數據，不調整商品、守護者優先序或付費 CTA。</x:v>
       </x:c>
     </x:row>
@@ -1509,6 +1518,773 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
+        <x:v>request_id</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>date</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>source</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>guardian_id</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
+        <x:v>guardian_name</x:v>
+      </x:c>
+      <x:c r="F1" t="str">
+        <x:v>intake_type</x:v>
+      </x:c>
+      <x:c r="G1" t="str">
+        <x:v>requested_asset</x:v>
+      </x:c>
+      <x:c r="H1" t="str">
+        <x:v>related_route</x:v>
+      </x:c>
+      <x:c r="I1" t="str">
+        <x:v>email_status</x:v>
+      </x:c>
+      <x:c r="J1" t="str">
+        <x:v>consent_status</x:v>
+      </x:c>
+      <x:c r="K1" t="str">
+        <x:v>priority</x:v>
+      </x:c>
+      <x:c r="L1" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="M1" t="str">
+        <x:v>first_response</x:v>
+      </x:c>
+      <x:c r="N1" t="str">
+        <x:v>next_action</x:v>
+      </x:c>
+      <x:c r="O1" t="str">
+        <x:v>follow_up_deadline</x:v>
+      </x:c>
+      <x:c r="P1" t="str">
+        <x:v>fulfillment_asset</x:v>
+      </x:c>
+      <x:c r="Q1" t="str">
+        <x:v>notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>template-iris-owned_asset_request</x:v>
+      </x:c>
+      <x:c r="B2" t="str"/>
+      <x:c r="C2" t="str">
+        <x:v>contact_or_waitlist</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="E2" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="F2" t="str">
+        <x:v>owned_asset_request</x:v>
+      </x:c>
+      <x:c r="G2" t="str">
+        <x:v>guardian PDF / wallpaper / short ritual</x:v>
+      </x:c>
+      <x:c r="H2" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-iris</x:v>
+      </x:c>
+      <x:c r="I2" t="str">
+        <x:v>not_received</x:v>
+      </x:c>
+      <x:c r="J2" t="str">
+        <x:v>not_applicable_until_user_contacts</x:v>
+      </x:c>
+      <x:c r="K2" t="str">
+        <x:v>medium</x:v>
+      </x:c>
+      <x:c r="L2" t="str">
+        <x:v>template</x:v>
+      </x:c>
+      <x:c r="M2" t="str">
+        <x:v>確認想收到的守護者素材，回覆預計製作方向與安全邊界。</x:v>
+      </x:c>
+      <x:c r="N2" t="str">
+        <x:v>累積同守護者重複需求後，排進 asset-build-backlog 的 build_owned_asset。</x:v>
+      </x:c>
+      <x:c r="O2" t="str"/>
+      <x:c r="P2" t="str"/>
+      <x:c r="Q2" t="str">
+        <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>template-iris-luna_scene_request</x:v>
+      </x:c>
+      <x:c r="B3" t="str"/>
+      <x:c r="C3" t="str">
+        <x:v>contact_or_waitlist</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="E3" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="F3" t="str">
+        <x:v>luna_scene_request</x:v>
+      </x:c>
+      <x:c r="G3" t="str">
+        <x:v>Luna bedtime / conflict cooldown / quiz aftercare pack</x:v>
+      </x:c>
+      <x:c r="H3" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-iris</x:v>
+      </x:c>
+      <x:c r="I3" t="str">
+        <x:v>not_received</x:v>
+      </x:c>
+      <x:c r="J3" t="str">
+        <x:v>not_applicable_until_user_contacts</x:v>
+      </x:c>
+      <x:c r="K3" t="str">
+        <x:v>medium</x:v>
+      </x:c>
+      <x:c r="L3" t="str">
+        <x:v>template</x:v>
+      </x:c>
+      <x:c r="M3" t="str">
+        <x:v>確認使用情境，不承諾療效，只提供夜間整理或冷卻素材方向。</x:v>
+      </x:c>
+      <x:c r="N3" t="str">
+        <x:v>若同守護者 Luna 需求重複，才測試結果後柔性商品承接。</x:v>
+      </x:c>
+      <x:c r="O3" t="str"/>
+      <x:c r="P3" t="str"/>
+      <x:c r="Q3" t="str">
+        <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>template-iris-repair_or_contact_request</x:v>
+      </x:c>
+      <x:c r="B4" t="str"/>
+      <x:c r="C4" t="str">
+        <x:v>contact_or_waitlist</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>repair_or_contact_request</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>relationship repair prompt / supply route guidance</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>not_received</x:v>
+      </x:c>
+      <x:c r="J4" t="str">
+        <x:v>not_applicable_until_user_contacts</x:v>
+      </x:c>
+      <x:c r="K4" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="L4" t="str">
+        <x:v>template</x:v>
+      </x:c>
+      <x:c r="M4" t="str">
+        <x:v>回覆可提供的網站路線與自助素材，不收集敏感個資，不取代諮商。</x:v>
+      </x:c>
+      <x:c r="N4" t="str">
+        <x:v>整理成 FAQ、修復計畫或 Contact 模板，不把個案內容公開。</x:v>
+      </x:c>
+      <x:c r="O4" t="str"/>
+      <x:c r="P4" t="str"/>
+      <x:c r="Q4" t="str">
+        <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>template-noah-owned_asset_request</x:v>
+      </x:c>
+      <x:c r="B5" t="str"/>
+      <x:c r="C5" t="str">
+        <x:v>contact_or_waitlist</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>noah</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>諾雅</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>owned_asset_request</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
+        <x:v>guardian PDF / wallpaper / short ritual</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-noah</x:v>
+      </x:c>
+      <x:c r="I5" t="str">
+        <x:v>not_received</x:v>
+      </x:c>
+      <x:c r="J5" t="str">
+        <x:v>not_applicable_until_user_contacts</x:v>
+      </x:c>
+      <x:c r="K5" t="str">
+        <x:v>medium</x:v>
+      </x:c>
+      <x:c r="L5" t="str">
+        <x:v>template</x:v>
+      </x:c>
+      <x:c r="M5" t="str">
+        <x:v>確認想收到的守護者素材，回覆預計製作方向與安全邊界。</x:v>
+      </x:c>
+      <x:c r="N5" t="str">
+        <x:v>累積同守護者重複需求後，排進 asset-build-backlog 的 build_owned_asset。</x:v>
+      </x:c>
+      <x:c r="O5" t="str"/>
+      <x:c r="P5" t="str"/>
+      <x:c r="Q5" t="str">
+        <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>template-noah-luna_scene_request</x:v>
+      </x:c>
+      <x:c r="B6" t="str"/>
+      <x:c r="C6" t="str">
+        <x:v>contact_or_waitlist</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>noah</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>諾雅</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>luna_scene_request</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>Luna bedtime / conflict cooldown / quiz aftercare pack</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-noah</x:v>
+      </x:c>
+      <x:c r="I6" t="str">
+        <x:v>not_received</x:v>
+      </x:c>
+      <x:c r="J6" t="str">
+        <x:v>not_applicable_until_user_contacts</x:v>
+      </x:c>
+      <x:c r="K6" t="str">
+        <x:v>medium</x:v>
+      </x:c>
+      <x:c r="L6" t="str">
+        <x:v>template</x:v>
+      </x:c>
+      <x:c r="M6" t="str">
+        <x:v>確認使用情境，不承諾療效，只提供夜間整理或冷卻素材方向。</x:v>
+      </x:c>
+      <x:c r="N6" t="str">
+        <x:v>若同守護者 Luna 需求重複，才測試結果後柔性商品承接。</x:v>
+      </x:c>
+      <x:c r="O6" t="str"/>
+      <x:c r="P6" t="str"/>
+      <x:c r="Q6" t="str">
+        <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>template-noah-repair_or_contact_request</x:v>
+      </x:c>
+      <x:c r="B7" t="str"/>
+      <x:c r="C7" t="str">
+        <x:v>contact_or_waitlist</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>noah</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>諾雅</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>repair_or_contact_request</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>relationship repair prompt / supply route guidance</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="I7" t="str">
+        <x:v>not_received</x:v>
+      </x:c>
+      <x:c r="J7" t="str">
+        <x:v>not_applicable_until_user_contacts</x:v>
+      </x:c>
+      <x:c r="K7" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="L7" t="str">
+        <x:v>template</x:v>
+      </x:c>
+      <x:c r="M7" t="str">
+        <x:v>回覆可提供的網站路線與自助素材，不收集敏感個資，不取代諮商。</x:v>
+      </x:c>
+      <x:c r="N7" t="str">
+        <x:v>整理成 FAQ、修復計畫或 Contact 模板，不把個案內容公開。</x:v>
+      </x:c>
+      <x:c r="O7" t="str"/>
+      <x:c r="P7" t="str"/>
+      <x:c r="Q7" t="str">
+        <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>template-vivian-owned_asset_request</x:v>
+      </x:c>
+      <x:c r="B8" t="str"/>
+      <x:c r="C8" t="str">
+        <x:v>contact_or_waitlist</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>vivian</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>薇薇安</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>owned_asset_request</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>guardian PDF / wallpaper / short ritual</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-vivian</x:v>
+      </x:c>
+      <x:c r="I8" t="str">
+        <x:v>not_received</x:v>
+      </x:c>
+      <x:c r="J8" t="str">
+        <x:v>not_applicable_until_user_contacts</x:v>
+      </x:c>
+      <x:c r="K8" t="str">
+        <x:v>medium</x:v>
+      </x:c>
+      <x:c r="L8" t="str">
+        <x:v>template</x:v>
+      </x:c>
+      <x:c r="M8" t="str">
+        <x:v>確認想收到的守護者素材，回覆預計製作方向與安全邊界。</x:v>
+      </x:c>
+      <x:c r="N8" t="str">
+        <x:v>累積同守護者重複需求後，排進 asset-build-backlog 的 build_owned_asset。</x:v>
+      </x:c>
+      <x:c r="O8" t="str"/>
+      <x:c r="P8" t="str"/>
+      <x:c r="Q8" t="str">
+        <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>template-vivian-luna_scene_request</x:v>
+      </x:c>
+      <x:c r="B9" t="str"/>
+      <x:c r="C9" t="str">
+        <x:v>contact_or_waitlist</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>vivian</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>薇薇安</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>luna_scene_request</x:v>
+      </x:c>
+      <x:c r="G9" t="str">
+        <x:v>Luna bedtime / conflict cooldown / quiz aftercare pack</x:v>
+      </x:c>
+      <x:c r="H9" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-vivian</x:v>
+      </x:c>
+      <x:c r="I9" t="str">
+        <x:v>not_received</x:v>
+      </x:c>
+      <x:c r="J9" t="str">
+        <x:v>not_applicable_until_user_contacts</x:v>
+      </x:c>
+      <x:c r="K9" t="str">
+        <x:v>medium</x:v>
+      </x:c>
+      <x:c r="L9" t="str">
+        <x:v>template</x:v>
+      </x:c>
+      <x:c r="M9" t="str">
+        <x:v>確認使用情境，不承諾療效，只提供夜間整理或冷卻素材方向。</x:v>
+      </x:c>
+      <x:c r="N9" t="str">
+        <x:v>若同守護者 Luna 需求重複，才測試結果後柔性商品承接。</x:v>
+      </x:c>
+      <x:c r="O9" t="str"/>
+      <x:c r="P9" t="str"/>
+      <x:c r="Q9" t="str">
+        <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>template-vivian-repair_or_contact_request</x:v>
+      </x:c>
+      <x:c r="B10" t="str"/>
+      <x:c r="C10" t="str">
+        <x:v>contact_or_waitlist</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>vivian</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>薇薇安</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>repair_or_contact_request</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>relationship repair prompt / supply route guidance</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="I10" t="str">
+        <x:v>not_received</x:v>
+      </x:c>
+      <x:c r="J10" t="str">
+        <x:v>not_applicable_until_user_contacts</x:v>
+      </x:c>
+      <x:c r="K10" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="L10" t="str">
+        <x:v>template</x:v>
+      </x:c>
+      <x:c r="M10" t="str">
+        <x:v>回覆可提供的網站路線與自助素材，不收集敏感個資，不取代諮商。</x:v>
+      </x:c>
+      <x:c r="N10" t="str">
+        <x:v>整理成 FAQ、修復計畫或 Contact 模板，不把個案內容公開。</x:v>
+      </x:c>
+      <x:c r="O10" t="str"/>
+      <x:c r="P10" t="str"/>
+      <x:c r="Q10" t="str">
+        <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>template-claire-owned_asset_request</x:v>
+      </x:c>
+      <x:c r="B11" t="str"/>
+      <x:c r="C11" t="str">
+        <x:v>contact_or_waitlist</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>claire</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>克萊兒</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>owned_asset_request</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>guardian PDF / wallpaper / short ritual</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-claire</x:v>
+      </x:c>
+      <x:c r="I11" t="str">
+        <x:v>not_received</x:v>
+      </x:c>
+      <x:c r="J11" t="str">
+        <x:v>not_applicable_until_user_contacts</x:v>
+      </x:c>
+      <x:c r="K11" t="str">
+        <x:v>medium</x:v>
+      </x:c>
+      <x:c r="L11" t="str">
+        <x:v>template</x:v>
+      </x:c>
+      <x:c r="M11" t="str">
+        <x:v>確認想收到的守護者素材，回覆預計製作方向與安全邊界。</x:v>
+      </x:c>
+      <x:c r="N11" t="str">
+        <x:v>累積同守護者重複需求後，排進 asset-build-backlog 的 build_owned_asset。</x:v>
+      </x:c>
+      <x:c r="O11" t="str"/>
+      <x:c r="P11" t="str"/>
+      <x:c r="Q11" t="str">
+        <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>template-claire-luna_scene_request</x:v>
+      </x:c>
+      <x:c r="B12" t="str"/>
+      <x:c r="C12" t="str">
+        <x:v>contact_or_waitlist</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>claire</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>克萊兒</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>luna_scene_request</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>Luna bedtime / conflict cooldown / quiz aftercare pack</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-claire</x:v>
+      </x:c>
+      <x:c r="I12" t="str">
+        <x:v>not_received</x:v>
+      </x:c>
+      <x:c r="J12" t="str">
+        <x:v>not_applicable_until_user_contacts</x:v>
+      </x:c>
+      <x:c r="K12" t="str">
+        <x:v>medium</x:v>
+      </x:c>
+      <x:c r="L12" t="str">
+        <x:v>template</x:v>
+      </x:c>
+      <x:c r="M12" t="str">
+        <x:v>確認使用情境，不承諾療效，只提供夜間整理或冷卻素材方向。</x:v>
+      </x:c>
+      <x:c r="N12" t="str">
+        <x:v>若同守護者 Luna 需求重複，才測試結果後柔性商品承接。</x:v>
+      </x:c>
+      <x:c r="O12" t="str"/>
+      <x:c r="P12" t="str"/>
+      <x:c r="Q12" t="str">
+        <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>template-claire-repair_or_contact_request</x:v>
+      </x:c>
+      <x:c r="B13" t="str"/>
+      <x:c r="C13" t="str">
+        <x:v>contact_or_waitlist</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>claire</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>克萊兒</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>repair_or_contact_request</x:v>
+      </x:c>
+      <x:c r="G13" t="str">
+        <x:v>relationship repair prompt / supply route guidance</x:v>
+      </x:c>
+      <x:c r="H13" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="I13" t="str">
+        <x:v>not_received</x:v>
+      </x:c>
+      <x:c r="J13" t="str">
+        <x:v>not_applicable_until_user_contacts</x:v>
+      </x:c>
+      <x:c r="K13" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="L13" t="str">
+        <x:v>template</x:v>
+      </x:c>
+      <x:c r="M13" t="str">
+        <x:v>回覆可提供的網站路線與自助素材，不收集敏感個資，不取代諮商。</x:v>
+      </x:c>
+      <x:c r="N13" t="str">
+        <x:v>整理成 FAQ、修復計畫或 Contact 模板，不把個案內容公開。</x:v>
+      </x:c>
+      <x:c r="O13" t="str"/>
+      <x:c r="P13" t="str"/>
+      <x:c r="Q13" t="str">
+        <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>template-dora-owned_asset_request</x:v>
+      </x:c>
+      <x:c r="B14" t="str"/>
+      <x:c r="C14" t="str">
+        <x:v>contact_or_waitlist</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>dora</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>朵拉</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>owned_asset_request</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>guardian PDF / wallpaper / short ritual</x:v>
+      </x:c>
+      <x:c r="H14" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-dora</x:v>
+      </x:c>
+      <x:c r="I14" t="str">
+        <x:v>not_received</x:v>
+      </x:c>
+      <x:c r="J14" t="str">
+        <x:v>not_applicable_until_user_contacts</x:v>
+      </x:c>
+      <x:c r="K14" t="str">
+        <x:v>medium</x:v>
+      </x:c>
+      <x:c r="L14" t="str">
+        <x:v>template</x:v>
+      </x:c>
+      <x:c r="M14" t="str">
+        <x:v>確認想收到的守護者素材，回覆預計製作方向與安全邊界。</x:v>
+      </x:c>
+      <x:c r="N14" t="str">
+        <x:v>累積同守護者重複需求後，排進 asset-build-backlog 的 build_owned_asset。</x:v>
+      </x:c>
+      <x:c r="O14" t="str"/>
+      <x:c r="P14" t="str"/>
+      <x:c r="Q14" t="str">
+        <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>template-dora-luna_scene_request</x:v>
+      </x:c>
+      <x:c r="B15" t="str"/>
+      <x:c r="C15" t="str">
+        <x:v>contact_or_waitlist</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>dora</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>朵拉</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
+        <x:v>luna_scene_request</x:v>
+      </x:c>
+      <x:c r="G15" t="str">
+        <x:v>Luna bedtime / conflict cooldown / quiz aftercare pack</x:v>
+      </x:c>
+      <x:c r="H15" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-dora</x:v>
+      </x:c>
+      <x:c r="I15" t="str">
+        <x:v>not_received</x:v>
+      </x:c>
+      <x:c r="J15" t="str">
+        <x:v>not_applicable_until_user_contacts</x:v>
+      </x:c>
+      <x:c r="K15" t="str">
+        <x:v>medium</x:v>
+      </x:c>
+      <x:c r="L15" t="str">
+        <x:v>template</x:v>
+      </x:c>
+      <x:c r="M15" t="str">
+        <x:v>確認使用情境，不承諾療效，只提供夜間整理或冷卻素材方向。</x:v>
+      </x:c>
+      <x:c r="N15" t="str">
+        <x:v>若同守護者 Luna 需求重複，才測試結果後柔性商品承接。</x:v>
+      </x:c>
+      <x:c r="O15" t="str"/>
+      <x:c r="P15" t="str"/>
+      <x:c r="Q15" t="str">
+        <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>template-dora-repair_or_contact_request</x:v>
+      </x:c>
+      <x:c r="B16" t="str"/>
+      <x:c r="C16" t="str">
+        <x:v>contact_or_waitlist</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>dora</x:v>
+      </x:c>
+      <x:c r="E16" t="str">
+        <x:v>朵拉</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
+        <x:v>repair_or_contact_request</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>relationship repair prompt / supply route guidance</x:v>
+      </x:c>
+      <x:c r="H16" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="I16" t="str">
+        <x:v>not_received</x:v>
+      </x:c>
+      <x:c r="J16" t="str">
+        <x:v>not_applicable_until_user_contacts</x:v>
+      </x:c>
+      <x:c r="K16" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="L16" t="str">
+        <x:v>template</x:v>
+      </x:c>
+      <x:c r="M16" t="str">
+        <x:v>回覆可提供的網站路線與自助素材，不收集敏感個資，不取代諮商。</x:v>
+      </x:c>
+      <x:c r="N16" t="str">
+        <x:v>整理成 FAQ、修復計畫或 Contact 模板，不把個案內容公開。</x:v>
+      </x:c>
+      <x:c r="O16" t="str"/>
+      <x:c r="P16" t="str"/>
+      <x:c r="Q16" t="str">
+        <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
         <x:v>Week 1 Profile Gates</x:v>
       </x:c>
       <x:c r="B1" t="str"/>
@@ -2207,7 +2983,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
@@ -2380,7 +3156,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
@@ -2472,6 +3248,14 @@
         <x:v>High-intent contact or path-summary mailto request.</x:v>
       </x:c>
     </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>lead-intake-tracker.csv</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>Template rows for real Contact, waitlist, Luna, or repair supply requests. Template rows are not user data.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Add guarded offer hypothesis board
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,13 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R1cb4b1e28cd644b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R23ee90edfbe248d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R49e948f496724a51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R508ac3422f754746"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="5" r:id="R2b381e4b538541bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="6" r:id="R262a1059b9fb41ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="7" r:id="R513fca235f5a4020"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc44d353e630f4409"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rf683b1a37b5544aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R690f9e28a0c64d52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R9281912d474a4865"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="R5ea5093c379a4803"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="6" r:id="R79ce6097fe544916"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="7" r:id="R4c94f09b95fc4254"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="8" r:id="Rba9f0397f88b4dff"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -253,51 +254,51 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>Week 1 profile gates pending</x:v>
+        <x:v>Offer hypothesis rows</x:v>
       </x:c>
       <x:c r="B8" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>Week 1 platform posts</x:v>
+        <x:v>Week 1 profile gates pending</x:v>
       </x:c>
       <x:c r="B9" t="n">
-        <x:v>9</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
+        <x:v>Week 1 platform posts</x:v>
+      </x:c>
+      <x:c r="B10" t="n">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
         <x:v>Empty data safety mode</x:v>
       </x:c>
-      <x:c r="B10" t="str">
+      <x:c r="B11" t="str">
         <x:v>YES</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" t="str"/>
-      <x:c r="B11" t="str"/>
-    </x:row>
     <x:row r="12">
-      <x:c r="A12" t="str">
-        <x:v>Metric</x:v>
-      </x:c>
-      <x:c r="B12" t="str">
-        <x:v>Value</x:v>
-      </x:c>
+      <x:c r="A12" t="str"/>
+      <x:c r="B12" t="str"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
-        <x:v>Views</x:v>
-      </x:c>
-      <x:c r="B13" t="n">
-        <x:v>0</x:v>
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>Value</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
-        <x:v>Site clicks</x:v>
+        <x:v>Views</x:v>
       </x:c>
       <x:c r="B14" t="n">
         <x:v>0</x:v>
@@ -305,7 +306,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
-        <x:v>Quiz starts</x:v>
+        <x:v>Site clicks</x:v>
       </x:c>
       <x:c r="B15" t="n">
         <x:v>0</x:v>
@@ -313,7 +314,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
-        <x:v>Quiz completions</x:v>
+        <x:v>Quiz starts</x:v>
       </x:c>
       <x:c r="B16" t="n">
         <x:v>0</x:v>
@@ -321,7 +322,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">
-        <x:v>Route interest</x:v>
+        <x:v>Quiz completions</x:v>
       </x:c>
       <x:c r="B17" t="n">
         <x:v>0</x:v>
@@ -329,7 +330,7 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="str">
-        <x:v>Revenue intent</x:v>
+        <x:v>Route interest</x:v>
       </x:c>
       <x:c r="B18" t="n">
         <x:v>0</x:v>
@@ -337,36 +338,36 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" t="str">
-        <x:v>Lead intent</x:v>
+        <x:v>Revenue intent</x:v>
       </x:c>
       <x:c r="B19" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" t="str"/>
-      <x:c r="B20" t="str"/>
+      <x:c r="A20" t="str">
+        <x:v>Lead intent</x:v>
+      </x:c>
+      <x:c r="B20" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" t="str">
-        <x:v>Recommended actions</x:v>
-      </x:c>
+      <x:c r="A21" t="str"/>
       <x:c r="B21" t="str"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" t="str">
-        <x:v>high</x:v>
-      </x:c>
-      <x:c r="B22" t="str">
-        <x:v>發布 Week 1 前 3 支 Shorts，先取得測驗完成樣本。</x:v>
-      </x:c>
+        <x:v>Recommended actions</x:v>
+      </x:c>
+      <x:c r="B22" t="str"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="B23" t="str">
-        <x:v>發布後至少回填 post_url、site_clicks、quiz_starts、quiz_completions。</x:v>
+        <x:v>發布 Week 1 前 3 支 Shorts，先取得測驗完成樣本。</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -374,7 +375,7 @@
         <x:v>high</x:v>
       </x:c>
       <x:c r="B24" t="str">
-        <x:v>發布前同步完成 YouTube、TikTok、Instagram 的 Bio/Profile link，使用平台專屬 UTM。</x:v>
+        <x:v>發布後至少回填 post_url、site_clicks、quiz_starts、quiz_completions。</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -382,14 +383,22 @@
         <x:v>high</x:v>
       </x:c>
       <x:c r="B25" t="str">
-        <x:v>平台首頁設定後回填 platform-profile-tracker.csv 的 status、profile_link_set_date、profile_clicks、site_clicks、quiz_starts、quiz_completions。</x:v>
+        <x:v>發布前同步完成 YouTube、TikTok、Instagram 的 Bio/Profile link，使用平台專屬 UTM。</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>平台首頁設定後回填 platform-profile-tracker.csv 的 status、profile_link_set_date、profile_clicks、site_clicks、quiz_starts、quiz_completions。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
         <x:v>medium</x:v>
       </x:c>
-      <x:c r="B26" t="str">
+      <x:c r="B27" t="str">
         <x:v>目前沒有回填數據，不調整商品、守護者優先序或付費 CTA。</x:v>
       </x:c>
     </x:row>
@@ -2285,6 +2294,243 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
+        <x:v>guardian_id</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>guardian_name</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>stage</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>offer_hypothesis</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
+        <x:v>free_asset</x:v>
+      </x:c>
+      <x:c r="F1" t="str">
+        <x:v>owned_asset</x:v>
+      </x:c>
+      <x:c r="G1" t="str">
+        <x:v>luna_test</x:v>
+      </x:c>
+      <x:c r="H1" t="str">
+        <x:v>affiliate_test</x:v>
+      </x:c>
+      <x:c r="I1" t="str">
+        <x:v>readiness</x:v>
+      </x:c>
+      <x:c r="J1" t="str">
+        <x:v>next_validation</x:v>
+      </x:c>
+      <x:c r="K1" t="str">
+        <x:v>target_url</x:v>
+      </x:c>
+      <x:c r="L1" t="str">
+        <x:v>safety_boundary</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>collect_signal</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
+        <x:v>目前只驗證測驗完成與守護者認同，不提出商品假設。</x:v>
+      </x:c>
+      <x:c r="E2" t="str">
+        <x:v>iris-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="F2" t="str">
+        <x:v>iris-email_lead_template</x:v>
+      </x:c>
+      <x:c r="G2" t="str">
+        <x:v>iris-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="H2" t="str">
+        <x:v>iris-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="I2" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="J2" t="str">
+        <x:v>先發布與回填 KPI；不新增付費 CTA，不改商品排序。</x:v>
+      </x:c>
+      <x:c r="K2" t="str">
+        <x:v>https://lovetypes.tw/start/</x:v>
+      </x:c>
+      <x:c r="L2" t="str">
+        <x:v>商品假設只能在測驗結果後或補給路線測試；不得承諾療效、診斷或必須購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>noah</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>諾雅</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>collect_signal</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>目前只驗證測驗完成與守護者認同，不提出商品假設。</x:v>
+      </x:c>
+      <x:c r="E3" t="str">
+        <x:v>noah-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="F3" t="str">
+        <x:v>noah-email_lead_template</x:v>
+      </x:c>
+      <x:c r="G3" t="str">
+        <x:v>noah-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="H3" t="str">
+        <x:v>noah-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="I3" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="J3" t="str">
+        <x:v>先發布與回填 KPI；不新增付費 CTA，不改商品排序。</x:v>
+      </x:c>
+      <x:c r="K3" t="str">
+        <x:v>https://lovetypes.tw/start/</x:v>
+      </x:c>
+      <x:c r="L3" t="str">
+        <x:v>商品假設只能在測驗結果後或補給路線測試；不得承諾療效、診斷或必須購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>vivian</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>薇薇安</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>collect_signal</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>目前只驗證測驗完成與守護者認同，不提出商品假設。</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>vivian-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>vivian-email_lead_template</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>vivian-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>vivian-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="J4" t="str">
+        <x:v>先發布與回填 KPI；不新增付費 CTA，不改商品排序。</x:v>
+      </x:c>
+      <x:c r="K4" t="str">
+        <x:v>https://lovetypes.tw/start/</x:v>
+      </x:c>
+      <x:c r="L4" t="str">
+        <x:v>商品假設只能在測驗結果後或補給路線測試；不得承諾療效、診斷或必須購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>claire</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>克萊兒</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>collect_signal</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>目前只驗證測驗完成與守護者認同，不提出商品假設。</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>claire-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>claire-email_lead_template</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
+        <x:v>claire-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
+        <x:v>claire-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="I5" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="J5" t="str">
+        <x:v>先發布與回填 KPI；不新增付費 CTA，不改商品排序。</x:v>
+      </x:c>
+      <x:c r="K5" t="str">
+        <x:v>https://lovetypes.tw/start/</x:v>
+      </x:c>
+      <x:c r="L5" t="str">
+        <x:v>商品假設只能在測驗結果後或補給路線測試；不得承諾療效、診斷或必須購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>dora</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>朵拉</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>collect_signal</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>目前只驗證測驗完成與守護者認同，不提出商品假設。</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>dora-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>dora-email_lead_template</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>dora-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>dora-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="I6" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="J6" t="str">
+        <x:v>先發布與回填 KPI；不新增付費 CTA，不改商品排序。</x:v>
+      </x:c>
+      <x:c r="K6" t="str">
+        <x:v>https://lovetypes.tw/start/</x:v>
+      </x:c>
+      <x:c r="L6" t="str">
+        <x:v>商品假設只能在測驗結果後或補給路線測試；不得承諾療效、診斷或必須購買。</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
         <x:v>Week 1 Profile Gates</x:v>
       </x:c>
       <x:c r="B1" t="str"/>
@@ -2983,7 +3229,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
@@ -3156,7 +3402,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
@@ -3256,6 +3502,14 @@
         <x:v>Template rows for real Contact, waitlist, Luna, or repair supply requests. Template rows are not user data.</x:v>
       </x:c>
     </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>offer-hypothesis-board.csv</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>Guardian-level offer hypotheses and readiness gates. HOLD rows must not change public paid CTA priority.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Add guarded offer experiment plan
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc44d353e630f4409"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rf683b1a37b5544aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R690f9e28a0c64d52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R9281912d474a4865"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="R5ea5093c379a4803"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="6" r:id="R79ce6097fe544916"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="7" r:id="R4c94f09b95fc4254"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="8" r:id="Rba9f0397f88b4dff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3124e247f7904cf3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R1761c80d5d734e26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R23e05850f75240fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R8299cfd16f7142f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="R34ddbf593f144d94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="R346a16c91af447e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="7" r:id="R1e5b3afaf1364b7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="8" r:id="Re36ed120752e4b28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="9" r:id="R185aa414bb3a4b7e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -262,51 +263,51 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>Week 1 profile gates pending</x:v>
+        <x:v>Offer experiment rows</x:v>
       </x:c>
       <x:c r="B9" t="n">
-        <x:v>3</x:v>
+        <x:v>20</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>Week 1 platform posts</x:v>
+        <x:v>Week 1 profile gates pending</x:v>
       </x:c>
       <x:c r="B10" t="n">
-        <x:v>9</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
+        <x:v>Week 1 platform posts</x:v>
+      </x:c>
+      <x:c r="B11" t="n">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
         <x:v>Empty data safety mode</x:v>
       </x:c>
-      <x:c r="B11" t="str">
+      <x:c r="B12" t="str">
         <x:v>YES</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" t="str"/>
-      <x:c r="B12" t="str"/>
-    </x:row>
     <x:row r="13">
-      <x:c r="A13" t="str">
-        <x:v>Metric</x:v>
-      </x:c>
-      <x:c r="B13" t="str">
-        <x:v>Value</x:v>
-      </x:c>
+      <x:c r="A13" t="str"/>
+      <x:c r="B13" t="str"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
-        <x:v>Views</x:v>
-      </x:c>
-      <x:c r="B14" t="n">
-        <x:v>0</x:v>
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>Value</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
-        <x:v>Site clicks</x:v>
+        <x:v>Views</x:v>
       </x:c>
       <x:c r="B15" t="n">
         <x:v>0</x:v>
@@ -314,7 +315,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
-        <x:v>Quiz starts</x:v>
+        <x:v>Site clicks</x:v>
       </x:c>
       <x:c r="B16" t="n">
         <x:v>0</x:v>
@@ -322,7 +323,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">
-        <x:v>Quiz completions</x:v>
+        <x:v>Quiz starts</x:v>
       </x:c>
       <x:c r="B17" t="n">
         <x:v>0</x:v>
@@ -330,7 +331,7 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="str">
-        <x:v>Route interest</x:v>
+        <x:v>Quiz completions</x:v>
       </x:c>
       <x:c r="B18" t="n">
         <x:v>0</x:v>
@@ -338,7 +339,7 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" t="str">
-        <x:v>Revenue intent</x:v>
+        <x:v>Route interest</x:v>
       </x:c>
       <x:c r="B19" t="n">
         <x:v>0</x:v>
@@ -346,36 +347,36 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" t="str">
+        <x:v>Revenue intent</x:v>
+      </x:c>
+      <x:c r="B20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
         <x:v>Lead intent</x:v>
       </x:c>
-      <x:c r="B20" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" t="str"/>
-      <x:c r="B21" t="str"/>
+      <x:c r="B21" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" t="str">
-        <x:v>Recommended actions</x:v>
-      </x:c>
+      <x:c r="A22" t="str"/>
       <x:c r="B22" t="str"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" t="str">
-        <x:v>high</x:v>
-      </x:c>
-      <x:c r="B23" t="str">
-        <x:v>發布 Week 1 前 3 支 Shorts，先取得測驗完成樣本。</x:v>
-      </x:c>
+        <x:v>Recommended actions</x:v>
+      </x:c>
+      <x:c r="B23" t="str"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="B24" t="str">
-        <x:v>發布後至少回填 post_url、site_clicks、quiz_starts、quiz_completions。</x:v>
+        <x:v>發布 Week 1 前 3 支 Shorts，先取得測驗完成樣本。</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -383,7 +384,7 @@
         <x:v>high</x:v>
       </x:c>
       <x:c r="B25" t="str">
-        <x:v>發布前同步完成 YouTube、TikTok、Instagram 的 Bio/Profile link，使用平台專屬 UTM。</x:v>
+        <x:v>發布後至少回填 post_url、site_clicks、quiz_starts、quiz_completions。</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -391,14 +392,22 @@
         <x:v>high</x:v>
       </x:c>
       <x:c r="B26" t="str">
-        <x:v>平台首頁設定後回填 platform-profile-tracker.csv 的 status、profile_link_set_date、profile_clicks、site_clicks、quiz_starts、quiz_completions。</x:v>
+        <x:v>發布前同步完成 YouTube、TikTok、Instagram 的 Bio/Profile link，使用平台專屬 UTM。</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>平台首頁設定後回填 platform-profile-tracker.csv 的 status、profile_link_set_date、profile_clicks、site_clicks、quiz_starts、quiz_completions。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
         <x:v>medium</x:v>
       </x:c>
-      <x:c r="B27" t="str">
+      <x:c r="B28" t="str">
         <x:v>目前沒有回填數據，不調整商品、守護者優先序或付費 CTA。</x:v>
       </x:c>
     </x:row>
@@ -2531,6 +2540,1128 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
+        <x:v>experiment_id</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>guardian_id</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>guardian_name</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>experiment_type</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="F1" t="str">
+        <x:v>hypothesis</x:v>
+      </x:c>
+      <x:c r="G1" t="str">
+        <x:v>primary_metric</x:v>
+      </x:c>
+      <x:c r="H1" t="str">
+        <x:v>primary_value</x:v>
+      </x:c>
+      <x:c r="I1" t="str">
+        <x:v>secondary_metric</x:v>
+      </x:c>
+      <x:c r="J1" t="str">
+        <x:v>secondary_value</x:v>
+      </x:c>
+      <x:c r="K1" t="str">
+        <x:v>minimum_signal</x:v>
+      </x:c>
+      <x:c r="L1" t="str">
+        <x:v>minimum_quiz_completions</x:v>
+      </x:c>
+      <x:c r="M1" t="str">
+        <x:v>quiz_completions</x:v>
+      </x:c>
+      <x:c r="N1" t="str">
+        <x:v>asset_id</x:v>
+      </x:c>
+      <x:c r="O1" t="str">
+        <x:v>target_url</x:v>
+      </x:c>
+      <x:c r="P1" t="str">
+        <x:v>next_action</x:v>
+      </x:c>
+      <x:c r="Q1" t="str">
+        <x:v>safety_boundary</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>iris-identity_save</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
+        <x:v>identity_save</x:v>
+      </x:c>
+      <x:c r="E2" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="F2" t="str">
+        <x:v>免費收藏物能提高守護者認同、保存與回訪。</x:v>
+      </x:c>
+      <x:c r="G2" t="str">
+        <x:v>free_keepsake_downloads</x:v>
+      </x:c>
+      <x:c r="H2" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I2" t="str">
+        <x:v>keepsake_clicks</x:v>
+      </x:c>
+      <x:c r="J2" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K2" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L2" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="M2" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N2" t="str">
+        <x:v>iris-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="O2" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-iris</x:v>
+      </x:c>
+      <x:c r="P2" t="str">
+        <x:v>先發布與回填 KPI；未達門檻前不製作或加強此商品假設。</x:v>
+      </x:c>
+      <x:c r="Q2" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>iris-owned_lead</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>owned_lead</x:v>
+      </x:c>
+      <x:c r="E3" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="F3" t="str">
+        <x:v>重複補給或 Contact 需求可轉成自有 Email 素材。</x:v>
+      </x:c>
+      <x:c r="G3" t="str">
+        <x:v>supply_lead_requests</x:v>
+      </x:c>
+      <x:c r="H3" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I3" t="str">
+        <x:v>contact_requests</x:v>
+      </x:c>
+      <x:c r="J3" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K3" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L3" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="M3" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N3" t="str">
+        <x:v>iris-email_lead_template</x:v>
+      </x:c>
+      <x:c r="O3" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="P3" t="str">
+        <x:v>先發布與回填 KPI；未達門檻前不製作或加強此商品假設。</x:v>
+      </x:c>
+      <x:c r="Q3" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>iris-luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>Luna 使用場景可在結果後路線承接夜間整理需求。</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>luna_pack_clicks</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>luna_clicks</x:v>
+      </x:c>
+      <x:c r="J4" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K4" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L4" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="M4" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N4" t="str">
+        <x:v>iris-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="O4" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-iris</x:v>
+      </x:c>
+      <x:c r="P4" t="str">
+        <x:v>先發布與回填 KPI；未達門檻前不製作或加強此商品假設。</x:v>
+      </x:c>
+      <x:c r="Q4" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>iris-affiliate_book</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>affiliate_book</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>延伸書卷可承接願意深讀的使用者，但不應取代免費路線。</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
+        <x:v>affiliate_book_clicks</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I5" t="str">
+        <x:v>resources_clicks</x:v>
+      </x:c>
+      <x:c r="J5" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K5" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L5" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="M5" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N5" t="str">
+        <x:v>iris-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="O5" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-iris</x:v>
+      </x:c>
+      <x:c r="P5" t="str">
+        <x:v>先發布與回填 KPI；未達門檻前不製作或加強此商品假設。</x:v>
+      </x:c>
+      <x:c r="Q5" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>noah-identity_save</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>noah</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>諾雅</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>identity_save</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>免費收藏物能提高守護者認同、保存與回訪。</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>free_keepsake_downloads</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I6" t="str">
+        <x:v>keepsake_clicks</x:v>
+      </x:c>
+      <x:c r="J6" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K6" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L6" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="M6" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N6" t="str">
+        <x:v>noah-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="O6" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-noah</x:v>
+      </x:c>
+      <x:c r="P6" t="str">
+        <x:v>先發布與回填 KPI；未達門檻前不製作或加強此商品假設。</x:v>
+      </x:c>
+      <x:c r="Q6" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>noah-owned_lead</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>noah</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>諾雅</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>owned_lead</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>重複補給或 Contact 需求可轉成自有 Email 素材。</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>supply_lead_requests</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I7" t="str">
+        <x:v>contact_requests</x:v>
+      </x:c>
+      <x:c r="J7" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K7" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L7" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="M7" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N7" t="str">
+        <x:v>noah-email_lead_template</x:v>
+      </x:c>
+      <x:c r="O7" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="P7" t="str">
+        <x:v>先發布與回填 KPI；未達門檻前不製作或加強此商品假設。</x:v>
+      </x:c>
+      <x:c r="Q7" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>noah-luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>noah</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>諾雅</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>Luna 使用場景可在結果後路線承接夜間整理需求。</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>luna_pack_clicks</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I8" t="str">
+        <x:v>luna_clicks</x:v>
+      </x:c>
+      <x:c r="J8" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K8" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L8" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="M8" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N8" t="str">
+        <x:v>noah-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="O8" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-noah</x:v>
+      </x:c>
+      <x:c r="P8" t="str">
+        <x:v>先發布與回填 KPI；未達門檻前不製作或加強此商品假設。</x:v>
+      </x:c>
+      <x:c r="Q8" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>noah-affiliate_book</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>noah</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>諾雅</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>affiliate_book</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>延伸書卷可承接願意深讀的使用者，但不應取代免費路線。</x:v>
+      </x:c>
+      <x:c r="G9" t="str">
+        <x:v>affiliate_book_clicks</x:v>
+      </x:c>
+      <x:c r="H9" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I9" t="str">
+        <x:v>resources_clicks</x:v>
+      </x:c>
+      <x:c r="J9" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K9" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L9" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="M9" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N9" t="str">
+        <x:v>noah-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="O9" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-noah</x:v>
+      </x:c>
+      <x:c r="P9" t="str">
+        <x:v>先發布與回填 KPI；未達門檻前不製作或加強此商品假設。</x:v>
+      </x:c>
+      <x:c r="Q9" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>vivian-identity_save</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>vivian</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>薇薇安</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>identity_save</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>免費收藏物能提高守護者認同、保存與回訪。</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>free_keepsake_downloads</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I10" t="str">
+        <x:v>keepsake_clicks</x:v>
+      </x:c>
+      <x:c r="J10" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K10" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L10" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="M10" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N10" t="str">
+        <x:v>vivian-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="O10" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-vivian</x:v>
+      </x:c>
+      <x:c r="P10" t="str">
+        <x:v>先發布與回填 KPI；未達門檻前不製作或加強此商品假設。</x:v>
+      </x:c>
+      <x:c r="Q10" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>vivian-owned_lead</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>vivian</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>薇薇安</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>owned_lead</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>重複補給或 Contact 需求可轉成自有 Email 素材。</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>supply_lead_requests</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I11" t="str">
+        <x:v>contact_requests</x:v>
+      </x:c>
+      <x:c r="J11" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K11" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L11" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="M11" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N11" t="str">
+        <x:v>vivian-email_lead_template</x:v>
+      </x:c>
+      <x:c r="O11" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="P11" t="str">
+        <x:v>先發布與回填 KPI；未達門檻前不製作或加強此商品假設。</x:v>
+      </x:c>
+      <x:c r="Q11" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>vivian-luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>vivian</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>薇薇安</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>Luna 使用場景可在結果後路線承接夜間整理需求。</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>luna_pack_clicks</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I12" t="str">
+        <x:v>luna_clicks</x:v>
+      </x:c>
+      <x:c r="J12" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K12" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L12" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="M12" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N12" t="str">
+        <x:v>vivian-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="O12" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-vivian</x:v>
+      </x:c>
+      <x:c r="P12" t="str">
+        <x:v>先發布與回填 KPI；未達門檻前不製作或加強此商品假設。</x:v>
+      </x:c>
+      <x:c r="Q12" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>vivian-affiliate_book</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>vivian</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>薇薇安</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>affiliate_book</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>延伸書卷可承接願意深讀的使用者，但不應取代免費路線。</x:v>
+      </x:c>
+      <x:c r="G13" t="str">
+        <x:v>affiliate_book_clicks</x:v>
+      </x:c>
+      <x:c r="H13" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I13" t="str">
+        <x:v>resources_clicks</x:v>
+      </x:c>
+      <x:c r="J13" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K13" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L13" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="M13" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N13" t="str">
+        <x:v>vivian-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="O13" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-vivian</x:v>
+      </x:c>
+      <x:c r="P13" t="str">
+        <x:v>先發布與回填 KPI；未達門檻前不製作或加強此商品假設。</x:v>
+      </x:c>
+      <x:c r="Q13" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>claire-identity_save</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>claire</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>克萊兒</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>identity_save</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>免費收藏物能提高守護者認同、保存與回訪。</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>free_keepsake_downloads</x:v>
+      </x:c>
+      <x:c r="H14" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I14" t="str">
+        <x:v>keepsake_clicks</x:v>
+      </x:c>
+      <x:c r="J14" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K14" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L14" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="M14" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N14" t="str">
+        <x:v>claire-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="O14" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-claire</x:v>
+      </x:c>
+      <x:c r="P14" t="str">
+        <x:v>先發布與回填 KPI；未達門檻前不製作或加強此商品假設。</x:v>
+      </x:c>
+      <x:c r="Q14" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>claire-owned_lead</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>claire</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>克萊兒</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>owned_lead</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
+        <x:v>重複補給或 Contact 需求可轉成自有 Email 素材。</x:v>
+      </x:c>
+      <x:c r="G15" t="str">
+        <x:v>supply_lead_requests</x:v>
+      </x:c>
+      <x:c r="H15" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I15" t="str">
+        <x:v>contact_requests</x:v>
+      </x:c>
+      <x:c r="J15" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K15" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L15" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="M15" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N15" t="str">
+        <x:v>claire-email_lead_template</x:v>
+      </x:c>
+      <x:c r="O15" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="P15" t="str">
+        <x:v>先發布與回填 KPI；未達門檻前不製作或加強此商品假設。</x:v>
+      </x:c>
+      <x:c r="Q15" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>claire-luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>claire</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>克萊兒</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="E16" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
+        <x:v>Luna 使用場景可在結果後路線承接夜間整理需求。</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>luna_pack_clicks</x:v>
+      </x:c>
+      <x:c r="H16" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I16" t="str">
+        <x:v>luna_clicks</x:v>
+      </x:c>
+      <x:c r="J16" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K16" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L16" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="M16" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N16" t="str">
+        <x:v>claire-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="O16" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-claire</x:v>
+      </x:c>
+      <x:c r="P16" t="str">
+        <x:v>先發布與回填 KPI；未達門檻前不製作或加強此商品假設。</x:v>
+      </x:c>
+      <x:c r="Q16" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>claire-affiliate_book</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>claire</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>克萊兒</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>affiliate_book</x:v>
+      </x:c>
+      <x:c r="E17" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="F17" t="str">
+        <x:v>延伸書卷可承接願意深讀的使用者，但不應取代免費路線。</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>affiliate_book_clicks</x:v>
+      </x:c>
+      <x:c r="H17" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I17" t="str">
+        <x:v>resources_clicks</x:v>
+      </x:c>
+      <x:c r="J17" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K17" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L17" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="M17" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N17" t="str">
+        <x:v>claire-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="O17" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-claire</x:v>
+      </x:c>
+      <x:c r="P17" t="str">
+        <x:v>先發布與回填 KPI；未達門檻前不製作或加強此商品假設。</x:v>
+      </x:c>
+      <x:c r="Q17" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>dora-identity_save</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>dora</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>朵拉</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>identity_save</x:v>
+      </x:c>
+      <x:c r="E18" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>免費收藏物能提高守護者認同、保存與回訪。</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>free_keepsake_downloads</x:v>
+      </x:c>
+      <x:c r="H18" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I18" t="str">
+        <x:v>keepsake_clicks</x:v>
+      </x:c>
+      <x:c r="J18" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K18" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L18" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="M18" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N18" t="str">
+        <x:v>dora-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="O18" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-dora</x:v>
+      </x:c>
+      <x:c r="P18" t="str">
+        <x:v>先發布與回填 KPI；未達門檻前不製作或加強此商品假設。</x:v>
+      </x:c>
+      <x:c r="Q18" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>dora-owned_lead</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>dora</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>朵拉</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>owned_lead</x:v>
+      </x:c>
+      <x:c r="E19" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="F19" t="str">
+        <x:v>重複補給或 Contact 需求可轉成自有 Email 素材。</x:v>
+      </x:c>
+      <x:c r="G19" t="str">
+        <x:v>supply_lead_requests</x:v>
+      </x:c>
+      <x:c r="H19" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I19" t="str">
+        <x:v>contact_requests</x:v>
+      </x:c>
+      <x:c r="J19" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K19" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L19" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="M19" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N19" t="str">
+        <x:v>dora-email_lead_template</x:v>
+      </x:c>
+      <x:c r="O19" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="P19" t="str">
+        <x:v>先發布與回填 KPI；未達門檻前不製作或加強此商品假設。</x:v>
+      </x:c>
+      <x:c r="Q19" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>dora-luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>dora</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>朵拉</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="E20" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="F20" t="str">
+        <x:v>Luna 使用場景可在結果後路線承接夜間整理需求。</x:v>
+      </x:c>
+      <x:c r="G20" t="str">
+        <x:v>luna_pack_clicks</x:v>
+      </x:c>
+      <x:c r="H20" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I20" t="str">
+        <x:v>luna_clicks</x:v>
+      </x:c>
+      <x:c r="J20" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K20" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L20" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="M20" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N20" t="str">
+        <x:v>dora-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="O20" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-dora</x:v>
+      </x:c>
+      <x:c r="P20" t="str">
+        <x:v>先發布與回填 KPI；未達門檻前不製作或加強此商品假設。</x:v>
+      </x:c>
+      <x:c r="Q20" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>dora-affiliate_book</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>dora</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>朵拉</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>affiliate_book</x:v>
+      </x:c>
+      <x:c r="E21" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="F21" t="str">
+        <x:v>延伸書卷可承接願意深讀的使用者，但不應取代免費路線。</x:v>
+      </x:c>
+      <x:c r="G21" t="str">
+        <x:v>affiliate_book_clicks</x:v>
+      </x:c>
+      <x:c r="H21" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I21" t="str">
+        <x:v>resources_clicks</x:v>
+      </x:c>
+      <x:c r="J21" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K21" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L21" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="M21" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N21" t="str">
+        <x:v>dora-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="O21" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-dora</x:v>
+      </x:c>
+      <x:c r="P21" t="str">
+        <x:v>先發布與回填 KPI；未達門檻前不製作或加強此商品假設。</x:v>
+      </x:c>
+      <x:c r="Q21" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
         <x:v>Week 1 Profile Gates</x:v>
       </x:c>
       <x:c r="B1" t="str"/>
@@ -3229,7 +4360,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
@@ -3402,7 +4533,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
@@ -3510,6 +4641,14 @@
         <x:v>Guardian-level offer hypotheses and readiness gates. HOLD rows must not change public paid CTA priority.</x:v>
       </x:c>
     </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>offer-experiment-plan.csv</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>Guarded product experiment thresholds for free assets, owned leads, Luna, and affiliate book tests.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Add offer experiment execution queue
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,15 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3124e247f7904cf3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R1761c80d5d734e26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R23e05850f75240fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R8299cfd16f7142f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="R34ddbf593f144d94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="R346a16c91af447e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="7" r:id="R1e5b3afaf1364b7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="8" r:id="Re36ed120752e4b28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="9" r:id="R185aa414bb3a4b7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3d479846c0554519"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R16a314dea9744d24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R64c42393f9104428"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="Rb7eeef88ef19449f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="Refa22eca0c3a461a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="Rbce1e3f47c7f410a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="Rc3802c0932594a1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="8" r:id="Ra1a35650123e4bcc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="9" r:id="R2ef0cd0c178b47f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="10" r:id="Ra865138427c340c5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -271,51 +272,51 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>Week 1 profile gates pending</x:v>
+        <x:v>Offer queue rows</x:v>
       </x:c>
       <x:c r="B10" t="n">
-        <x:v>3</x:v>
+        <x:v>80</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
-        <x:v>Week 1 platform posts</x:v>
+        <x:v>Week 1 profile gates pending</x:v>
       </x:c>
       <x:c r="B11" t="n">
-        <x:v>9</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
+        <x:v>Week 1 platform posts</x:v>
+      </x:c>
+      <x:c r="B12" t="n">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
         <x:v>Empty data safety mode</x:v>
       </x:c>
-      <x:c r="B12" t="str">
+      <x:c r="B13" t="str">
         <x:v>YES</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" t="str"/>
-      <x:c r="B13" t="str"/>
-    </x:row>
     <x:row r="14">
-      <x:c r="A14" t="str">
-        <x:v>Metric</x:v>
-      </x:c>
-      <x:c r="B14" t="str">
-        <x:v>Value</x:v>
-      </x:c>
+      <x:c r="A14" t="str"/>
+      <x:c r="B14" t="str"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
-        <x:v>Views</x:v>
-      </x:c>
-      <x:c r="B15" t="n">
-        <x:v>0</x:v>
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>Value</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
-        <x:v>Site clicks</x:v>
+        <x:v>Views</x:v>
       </x:c>
       <x:c r="B16" t="n">
         <x:v>0</x:v>
@@ -323,7 +324,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">
-        <x:v>Quiz starts</x:v>
+        <x:v>Site clicks</x:v>
       </x:c>
       <x:c r="B17" t="n">
         <x:v>0</x:v>
@@ -331,7 +332,7 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="str">
-        <x:v>Quiz completions</x:v>
+        <x:v>Quiz starts</x:v>
       </x:c>
       <x:c r="B18" t="n">
         <x:v>0</x:v>
@@ -339,7 +340,7 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" t="str">
-        <x:v>Route interest</x:v>
+        <x:v>Quiz completions</x:v>
       </x:c>
       <x:c r="B19" t="n">
         <x:v>0</x:v>
@@ -347,7 +348,7 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" t="str">
-        <x:v>Revenue intent</x:v>
+        <x:v>Route interest</x:v>
       </x:c>
       <x:c r="B20" t="n">
         <x:v>0</x:v>
@@ -355,36 +356,36 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" t="str">
-        <x:v>Lead intent</x:v>
+        <x:v>Revenue intent</x:v>
       </x:c>
       <x:c r="B21" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" t="str"/>
-      <x:c r="B22" t="str"/>
+      <x:c r="A22" t="str">
+        <x:v>Lead intent</x:v>
+      </x:c>
+      <x:c r="B22" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" t="str">
-        <x:v>Recommended actions</x:v>
-      </x:c>
+      <x:c r="A23" t="str"/>
       <x:c r="B23" t="str"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" t="str">
-        <x:v>high</x:v>
-      </x:c>
-      <x:c r="B24" t="str">
-        <x:v>發布 Week 1 前 3 支 Shorts，先取得測驗完成樣本。</x:v>
-      </x:c>
+        <x:v>Recommended actions</x:v>
+      </x:c>
+      <x:c r="B24" t="str"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="B25" t="str">
-        <x:v>發布後至少回填 post_url、site_clicks、quiz_starts、quiz_completions。</x:v>
+        <x:v>發布 Week 1 前 3 支 Shorts，先取得測驗完成樣本。</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -392,7 +393,7 @@
         <x:v>high</x:v>
       </x:c>
       <x:c r="B26" t="str">
-        <x:v>發布前同步完成 YouTube、TikTok、Instagram 的 Bio/Profile link，使用平台專屬 UTM。</x:v>
+        <x:v>發布後至少回填 post_url、site_clicks、quiz_starts、quiz_completions。</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -400,15 +401,152 @@
         <x:v>high</x:v>
       </x:c>
       <x:c r="B27" t="str">
-        <x:v>平台首頁設定後回填 platform-profile-tracker.csv 的 status、profile_link_set_date、profile_clicks、site_clicks、quiz_starts、quiz_completions。</x:v>
+        <x:v>發布前同步完成 YouTube、TikTok、Instagram 的 Bio/Profile link，使用平台專屬 UTM。</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>平台首頁設定後回填 platform-profile-tracker.csv 的 status、profile_link_set_date、profile_clicks、site_clicks、quiz_starts、quiz_completions。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
         <x:v>medium</x:v>
       </x:c>
-      <x:c r="B28" t="str">
+      <x:c r="B29" t="str">
         <x:v>目前沒有回填數據，不調整商品、守護者優先序或付費 CTA。</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
+        <x:v>Field</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>Meaning</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>site_clicks</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>Clicks from social profile/caption into LoveTypes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>quiz_starts</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>Sessions where the 15-question guardian quiz begins.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>quiz_completions</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>Completed quiz sessions; primary first-round KPI.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>profile_clicks</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>Clicks on social Bio/Profile links before visitors reach LoveTypes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>profile_link_set_date</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>Date the platform Bio/Profile tracked link was set live.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>free_keepsake_downloads</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>Guardian identity asset save or print intent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>supply_lead_requests</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>Owned email/request demand for guardian supply assets.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>luna_pack_clicks</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>Luna Gumroad product exploration.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>affiliate_book_clicks</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>Affiliate book route exploration.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>contact_requests</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>High-intent contact or path-summary mailto request.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>lead-intake-tracker.csv</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>Template rows for real Contact, waitlist, Luna, or repair supply requests. Template rows are not user data.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>offer-hypothesis-board.csv</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>Guardian-level offer hypotheses and readiness gates. HOLD rows must not change public paid CTA priority.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>offer-experiment-plan.csv</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>Guarded product experiment thresholds for free assets, owned leads, Luna, and affiliate book tests.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>offer-experiment-queue.csv</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>Execution queue for READY offer experiments. Blocked rows must not be produced as public assets.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3662,6 +3800,3579 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
+        <x:v>queue_id</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>experiment_id</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>guardian_id</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>guardian_name</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
+        <x:v>experiment_type</x:v>
+      </x:c>
+      <x:c r="F1" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="G1" t="str">
+        <x:v>step</x:v>
+      </x:c>
+      <x:c r="H1" t="str">
+        <x:v>deliverable</x:v>
+      </x:c>
+      <x:c r="I1" t="str">
+        <x:v>asset_id</x:v>
+      </x:c>
+      <x:c r="J1" t="str">
+        <x:v>target_url</x:v>
+      </x:c>
+      <x:c r="K1" t="str">
+        <x:v>owner</x:v>
+      </x:c>
+      <x:c r="L1" t="str">
+        <x:v>acceptance_check</x:v>
+      </x:c>
+      <x:c r="M1" t="str">
+        <x:v>writeback</x:v>
+      </x:c>
+      <x:c r="N1" t="str">
+        <x:v>safety_boundary</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>iris-identity_save-brief</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>iris-identity_save</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="E2" t="str">
+        <x:v>identity_save</x:v>
+      </x:c>
+      <x:c r="F2" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G2" t="str">
+        <x:v>brief</x:v>
+      </x:c>
+      <x:c r="H2" t="str">
+        <x:v>Write a one-page asset brief with guardian, scene, promise boundary, and CTA.</x:v>
+      </x:c>
+      <x:c r="I2" t="str">
+        <x:v>iris-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="J2" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-iris</x:v>
+      </x:c>
+      <x:c r="K2" t="str">
+        <x:v>content</x:v>
+      </x:c>
+      <x:c r="L2" t="str">
+        <x:v>Brief keeps the Shorts CTA as quiz and places offer only after result route.</x:v>
+      </x:c>
+      <x:c r="M2" t="str">
+        <x:v>Update offer-experiment-plan after KPI review.</x:v>
+      </x:c>
+      <x:c r="N2" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>iris-identity_save-asset</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>iris-identity_save</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="E3" t="str">
+        <x:v>identity_save</x:v>
+      </x:c>
+      <x:c r="F3" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G3" t="str">
+        <x:v>asset</x:v>
+      </x:c>
+      <x:c r="H3" t="str">
+        <x:v>Produce the smallest useful asset or route copy for the experiment.</x:v>
+      </x:c>
+      <x:c r="I3" t="str">
+        <x:v>iris-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="J3" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-iris</x:v>
+      </x:c>
+      <x:c r="K3" t="str">
+        <x:v>creative</x:v>
+      </x:c>
+      <x:c r="L3" t="str">
+        <x:v>Asset links to the existing target URL and does not claim diagnosis or therapeutic outcome.</x:v>
+      </x:c>
+      <x:c r="M3" t="str">
+        <x:v>Record fulfillment asset in lead-intake-tracker.csv when a real request exists.</x:v>
+      </x:c>
+      <x:c r="N3" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>iris-identity_save-qa</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>iris-identity_save</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>identity_save</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>qa</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>Check safety copy, route, tracking event, and mobile presentation before publish.</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>iris-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="J4" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-iris</x:v>
+      </x:c>
+      <x:c r="K4" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L4" t="str">
+        <x:v>Public smoke remains clean and no paid CTA is added before the experiment is READY.</x:v>
+      </x:c>
+      <x:c r="M4" t="str">
+        <x:v>Run predeploy_check.py before deploy.</x:v>
+      </x:c>
+      <x:c r="N4" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>iris-identity_save-measure</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>iris-identity_save</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>identity_save</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
+        <x:v>measure</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
+        <x:v>After the test window, backfill KPI fields and decide continue, revise, or stop.</x:v>
+      </x:c>
+      <x:c r="I5" t="str">
+        <x:v>iris-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="J5" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-iris</x:v>
+      </x:c>
+      <x:c r="K5" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L5" t="str">
+        <x:v>KPI row includes primary and secondary metric fields for the experiment.</x:v>
+      </x:c>
+      <x:c r="M5" t="str">
+        <x:v>Update kpi-tracker.csv, weekly-summary, decision gate, offer board, and experiment plan.</x:v>
+      </x:c>
+      <x:c r="N5" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>iris-owned_lead-brief</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>iris-owned_lead</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>owned_lead</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>brief</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>Write a one-page asset brief with guardian, scene, promise boundary, and CTA.</x:v>
+      </x:c>
+      <x:c r="I6" t="str">
+        <x:v>iris-email_lead_template</x:v>
+      </x:c>
+      <x:c r="J6" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="K6" t="str">
+        <x:v>content</x:v>
+      </x:c>
+      <x:c r="L6" t="str">
+        <x:v>Brief keeps the Shorts CTA as quiz and places offer only after result route.</x:v>
+      </x:c>
+      <x:c r="M6" t="str">
+        <x:v>Update offer-experiment-plan after KPI review.</x:v>
+      </x:c>
+      <x:c r="N6" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>iris-owned_lead-asset</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>iris-owned_lead</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>owned_lead</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>asset</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
+        <x:v>Produce the smallest useful asset or route copy for the experiment.</x:v>
+      </x:c>
+      <x:c r="I7" t="str">
+        <x:v>iris-email_lead_template</x:v>
+      </x:c>
+      <x:c r="J7" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="K7" t="str">
+        <x:v>creative</x:v>
+      </x:c>
+      <x:c r="L7" t="str">
+        <x:v>Asset links to the existing target URL and does not claim diagnosis or therapeutic outcome.</x:v>
+      </x:c>
+      <x:c r="M7" t="str">
+        <x:v>Record fulfillment asset in lead-intake-tracker.csv when a real request exists.</x:v>
+      </x:c>
+      <x:c r="N7" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>iris-owned_lead-qa</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>iris-owned_lead</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>owned_lead</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>qa</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>Check safety copy, route, tracking event, and mobile presentation before publish.</x:v>
+      </x:c>
+      <x:c r="I8" t="str">
+        <x:v>iris-email_lead_template</x:v>
+      </x:c>
+      <x:c r="J8" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="K8" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L8" t="str">
+        <x:v>Public smoke remains clean and no paid CTA is added before the experiment is READY.</x:v>
+      </x:c>
+      <x:c r="M8" t="str">
+        <x:v>Run predeploy_check.py before deploy.</x:v>
+      </x:c>
+      <x:c r="N8" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>iris-owned_lead-measure</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>iris-owned_lead</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>owned_lead</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G9" t="str">
+        <x:v>measure</x:v>
+      </x:c>
+      <x:c r="H9" t="str">
+        <x:v>After the test window, backfill KPI fields and decide continue, revise, or stop.</x:v>
+      </x:c>
+      <x:c r="I9" t="str">
+        <x:v>iris-email_lead_template</x:v>
+      </x:c>
+      <x:c r="J9" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="K9" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L9" t="str">
+        <x:v>KPI row includes primary and secondary metric fields for the experiment.</x:v>
+      </x:c>
+      <x:c r="M9" t="str">
+        <x:v>Update kpi-tracker.csv, weekly-summary, decision gate, offer board, and experiment plan.</x:v>
+      </x:c>
+      <x:c r="N9" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>iris-luna_soft_offer-brief</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>iris-luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>brief</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>Write a one-page asset brief with guardian, scene, promise boundary, and CTA.</x:v>
+      </x:c>
+      <x:c r="I10" t="str">
+        <x:v>iris-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="J10" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-iris</x:v>
+      </x:c>
+      <x:c r="K10" t="str">
+        <x:v>content</x:v>
+      </x:c>
+      <x:c r="L10" t="str">
+        <x:v>Brief keeps the Shorts CTA as quiz and places offer only after result route.</x:v>
+      </x:c>
+      <x:c r="M10" t="str">
+        <x:v>Update offer-experiment-plan after KPI review.</x:v>
+      </x:c>
+      <x:c r="N10" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>iris-luna_soft_offer-asset</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>iris-luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>asset</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>Produce the smallest useful asset or route copy for the experiment.</x:v>
+      </x:c>
+      <x:c r="I11" t="str">
+        <x:v>iris-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="J11" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-iris</x:v>
+      </x:c>
+      <x:c r="K11" t="str">
+        <x:v>creative</x:v>
+      </x:c>
+      <x:c r="L11" t="str">
+        <x:v>Asset links to the existing target URL and does not claim diagnosis or therapeutic outcome.</x:v>
+      </x:c>
+      <x:c r="M11" t="str">
+        <x:v>Record fulfillment asset in lead-intake-tracker.csv when a real request exists.</x:v>
+      </x:c>
+      <x:c r="N11" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>iris-luna_soft_offer-qa</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>iris-luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>qa</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>Check safety copy, route, tracking event, and mobile presentation before publish.</x:v>
+      </x:c>
+      <x:c r="I12" t="str">
+        <x:v>iris-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="J12" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-iris</x:v>
+      </x:c>
+      <x:c r="K12" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L12" t="str">
+        <x:v>Public smoke remains clean and no paid CTA is added before the experiment is READY.</x:v>
+      </x:c>
+      <x:c r="M12" t="str">
+        <x:v>Run predeploy_check.py before deploy.</x:v>
+      </x:c>
+      <x:c r="N12" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>iris-luna_soft_offer-measure</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>iris-luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G13" t="str">
+        <x:v>measure</x:v>
+      </x:c>
+      <x:c r="H13" t="str">
+        <x:v>After the test window, backfill KPI fields and decide continue, revise, or stop.</x:v>
+      </x:c>
+      <x:c r="I13" t="str">
+        <x:v>iris-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="J13" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-iris</x:v>
+      </x:c>
+      <x:c r="K13" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L13" t="str">
+        <x:v>KPI row includes primary and secondary metric fields for the experiment.</x:v>
+      </x:c>
+      <x:c r="M13" t="str">
+        <x:v>Update kpi-tracker.csv, weekly-summary, decision gate, offer board, and experiment plan.</x:v>
+      </x:c>
+      <x:c r="N13" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>iris-affiliate_book-brief</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>iris-affiliate_book</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>affiliate_book</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>brief</x:v>
+      </x:c>
+      <x:c r="H14" t="str">
+        <x:v>Write a one-page asset brief with guardian, scene, promise boundary, and CTA.</x:v>
+      </x:c>
+      <x:c r="I14" t="str">
+        <x:v>iris-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="J14" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-iris</x:v>
+      </x:c>
+      <x:c r="K14" t="str">
+        <x:v>content</x:v>
+      </x:c>
+      <x:c r="L14" t="str">
+        <x:v>Brief keeps the Shorts CTA as quiz and places offer only after result route.</x:v>
+      </x:c>
+      <x:c r="M14" t="str">
+        <x:v>Update offer-experiment-plan after KPI review.</x:v>
+      </x:c>
+      <x:c r="N14" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>iris-affiliate_book-asset</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>iris-affiliate_book</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>affiliate_book</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G15" t="str">
+        <x:v>asset</x:v>
+      </x:c>
+      <x:c r="H15" t="str">
+        <x:v>Produce the smallest useful asset or route copy for the experiment.</x:v>
+      </x:c>
+      <x:c r="I15" t="str">
+        <x:v>iris-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="J15" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-iris</x:v>
+      </x:c>
+      <x:c r="K15" t="str">
+        <x:v>creative</x:v>
+      </x:c>
+      <x:c r="L15" t="str">
+        <x:v>Asset links to the existing target URL and does not claim diagnosis or therapeutic outcome.</x:v>
+      </x:c>
+      <x:c r="M15" t="str">
+        <x:v>Record fulfillment asset in lead-intake-tracker.csv when a real request exists.</x:v>
+      </x:c>
+      <x:c r="N15" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>iris-affiliate_book-qa</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>iris-affiliate_book</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="E16" t="str">
+        <x:v>affiliate_book</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>qa</x:v>
+      </x:c>
+      <x:c r="H16" t="str">
+        <x:v>Check safety copy, route, tracking event, and mobile presentation before publish.</x:v>
+      </x:c>
+      <x:c r="I16" t="str">
+        <x:v>iris-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="J16" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-iris</x:v>
+      </x:c>
+      <x:c r="K16" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L16" t="str">
+        <x:v>Public smoke remains clean and no paid CTA is added before the experiment is READY.</x:v>
+      </x:c>
+      <x:c r="M16" t="str">
+        <x:v>Run predeploy_check.py before deploy.</x:v>
+      </x:c>
+      <x:c r="N16" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>iris-affiliate_book-measure</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>iris-affiliate_book</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="E17" t="str">
+        <x:v>affiliate_book</x:v>
+      </x:c>
+      <x:c r="F17" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>measure</x:v>
+      </x:c>
+      <x:c r="H17" t="str">
+        <x:v>After the test window, backfill KPI fields and decide continue, revise, or stop.</x:v>
+      </x:c>
+      <x:c r="I17" t="str">
+        <x:v>iris-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="J17" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-iris</x:v>
+      </x:c>
+      <x:c r="K17" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L17" t="str">
+        <x:v>KPI row includes primary and secondary metric fields for the experiment.</x:v>
+      </x:c>
+      <x:c r="M17" t="str">
+        <x:v>Update kpi-tracker.csv, weekly-summary, decision gate, offer board, and experiment plan.</x:v>
+      </x:c>
+      <x:c r="N17" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>noah-identity_save-brief</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>noah-identity_save</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>noah</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>諾雅</x:v>
+      </x:c>
+      <x:c r="E18" t="str">
+        <x:v>identity_save</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>brief</x:v>
+      </x:c>
+      <x:c r="H18" t="str">
+        <x:v>Write a one-page asset brief with guardian, scene, promise boundary, and CTA.</x:v>
+      </x:c>
+      <x:c r="I18" t="str">
+        <x:v>noah-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="J18" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-noah</x:v>
+      </x:c>
+      <x:c r="K18" t="str">
+        <x:v>content</x:v>
+      </x:c>
+      <x:c r="L18" t="str">
+        <x:v>Brief keeps the Shorts CTA as quiz and places offer only after result route.</x:v>
+      </x:c>
+      <x:c r="M18" t="str">
+        <x:v>Update offer-experiment-plan after KPI review.</x:v>
+      </x:c>
+      <x:c r="N18" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>noah-identity_save-asset</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>noah-identity_save</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>noah</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>諾雅</x:v>
+      </x:c>
+      <x:c r="E19" t="str">
+        <x:v>identity_save</x:v>
+      </x:c>
+      <x:c r="F19" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G19" t="str">
+        <x:v>asset</x:v>
+      </x:c>
+      <x:c r="H19" t="str">
+        <x:v>Produce the smallest useful asset or route copy for the experiment.</x:v>
+      </x:c>
+      <x:c r="I19" t="str">
+        <x:v>noah-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="J19" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-noah</x:v>
+      </x:c>
+      <x:c r="K19" t="str">
+        <x:v>creative</x:v>
+      </x:c>
+      <x:c r="L19" t="str">
+        <x:v>Asset links to the existing target URL and does not claim diagnosis or therapeutic outcome.</x:v>
+      </x:c>
+      <x:c r="M19" t="str">
+        <x:v>Record fulfillment asset in lead-intake-tracker.csv when a real request exists.</x:v>
+      </x:c>
+      <x:c r="N19" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>noah-identity_save-qa</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>noah-identity_save</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>noah</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>諾雅</x:v>
+      </x:c>
+      <x:c r="E20" t="str">
+        <x:v>identity_save</x:v>
+      </x:c>
+      <x:c r="F20" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G20" t="str">
+        <x:v>qa</x:v>
+      </x:c>
+      <x:c r="H20" t="str">
+        <x:v>Check safety copy, route, tracking event, and mobile presentation before publish.</x:v>
+      </x:c>
+      <x:c r="I20" t="str">
+        <x:v>noah-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="J20" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-noah</x:v>
+      </x:c>
+      <x:c r="K20" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L20" t="str">
+        <x:v>Public smoke remains clean and no paid CTA is added before the experiment is READY.</x:v>
+      </x:c>
+      <x:c r="M20" t="str">
+        <x:v>Run predeploy_check.py before deploy.</x:v>
+      </x:c>
+      <x:c r="N20" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>noah-identity_save-measure</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>noah-identity_save</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>noah</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>諾雅</x:v>
+      </x:c>
+      <x:c r="E21" t="str">
+        <x:v>identity_save</x:v>
+      </x:c>
+      <x:c r="F21" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G21" t="str">
+        <x:v>measure</x:v>
+      </x:c>
+      <x:c r="H21" t="str">
+        <x:v>After the test window, backfill KPI fields and decide continue, revise, or stop.</x:v>
+      </x:c>
+      <x:c r="I21" t="str">
+        <x:v>noah-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="J21" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-noah</x:v>
+      </x:c>
+      <x:c r="K21" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L21" t="str">
+        <x:v>KPI row includes primary and secondary metric fields for the experiment.</x:v>
+      </x:c>
+      <x:c r="M21" t="str">
+        <x:v>Update kpi-tracker.csv, weekly-summary, decision gate, offer board, and experiment plan.</x:v>
+      </x:c>
+      <x:c r="N21" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>noah-owned_lead-brief</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>noah-owned_lead</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>noah</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>諾雅</x:v>
+      </x:c>
+      <x:c r="E22" t="str">
+        <x:v>owned_lead</x:v>
+      </x:c>
+      <x:c r="F22" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G22" t="str">
+        <x:v>brief</x:v>
+      </x:c>
+      <x:c r="H22" t="str">
+        <x:v>Write a one-page asset brief with guardian, scene, promise boundary, and CTA.</x:v>
+      </x:c>
+      <x:c r="I22" t="str">
+        <x:v>noah-email_lead_template</x:v>
+      </x:c>
+      <x:c r="J22" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="K22" t="str">
+        <x:v>content</x:v>
+      </x:c>
+      <x:c r="L22" t="str">
+        <x:v>Brief keeps the Shorts CTA as quiz and places offer only after result route.</x:v>
+      </x:c>
+      <x:c r="M22" t="str">
+        <x:v>Update offer-experiment-plan after KPI review.</x:v>
+      </x:c>
+      <x:c r="N22" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>noah-owned_lead-asset</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>noah-owned_lead</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>noah</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
+        <x:v>諾雅</x:v>
+      </x:c>
+      <x:c r="E23" t="str">
+        <x:v>owned_lead</x:v>
+      </x:c>
+      <x:c r="F23" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G23" t="str">
+        <x:v>asset</x:v>
+      </x:c>
+      <x:c r="H23" t="str">
+        <x:v>Produce the smallest useful asset or route copy for the experiment.</x:v>
+      </x:c>
+      <x:c r="I23" t="str">
+        <x:v>noah-email_lead_template</x:v>
+      </x:c>
+      <x:c r="J23" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="K23" t="str">
+        <x:v>creative</x:v>
+      </x:c>
+      <x:c r="L23" t="str">
+        <x:v>Asset links to the existing target URL and does not claim diagnosis or therapeutic outcome.</x:v>
+      </x:c>
+      <x:c r="M23" t="str">
+        <x:v>Record fulfillment asset in lead-intake-tracker.csv when a real request exists.</x:v>
+      </x:c>
+      <x:c r="N23" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>noah-owned_lead-qa</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>noah-owned_lead</x:v>
+      </x:c>
+      <x:c r="C24" t="str">
+        <x:v>noah</x:v>
+      </x:c>
+      <x:c r="D24" t="str">
+        <x:v>諾雅</x:v>
+      </x:c>
+      <x:c r="E24" t="str">
+        <x:v>owned_lead</x:v>
+      </x:c>
+      <x:c r="F24" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G24" t="str">
+        <x:v>qa</x:v>
+      </x:c>
+      <x:c r="H24" t="str">
+        <x:v>Check safety copy, route, tracking event, and mobile presentation before publish.</x:v>
+      </x:c>
+      <x:c r="I24" t="str">
+        <x:v>noah-email_lead_template</x:v>
+      </x:c>
+      <x:c r="J24" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="K24" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L24" t="str">
+        <x:v>Public smoke remains clean and no paid CTA is added before the experiment is READY.</x:v>
+      </x:c>
+      <x:c r="M24" t="str">
+        <x:v>Run predeploy_check.py before deploy.</x:v>
+      </x:c>
+      <x:c r="N24" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="str">
+        <x:v>noah-owned_lead-measure</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>noah-owned_lead</x:v>
+      </x:c>
+      <x:c r="C25" t="str">
+        <x:v>noah</x:v>
+      </x:c>
+      <x:c r="D25" t="str">
+        <x:v>諾雅</x:v>
+      </x:c>
+      <x:c r="E25" t="str">
+        <x:v>owned_lead</x:v>
+      </x:c>
+      <x:c r="F25" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G25" t="str">
+        <x:v>measure</x:v>
+      </x:c>
+      <x:c r="H25" t="str">
+        <x:v>After the test window, backfill KPI fields and decide continue, revise, or stop.</x:v>
+      </x:c>
+      <x:c r="I25" t="str">
+        <x:v>noah-email_lead_template</x:v>
+      </x:c>
+      <x:c r="J25" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="K25" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L25" t="str">
+        <x:v>KPI row includes primary and secondary metric fields for the experiment.</x:v>
+      </x:c>
+      <x:c r="M25" t="str">
+        <x:v>Update kpi-tracker.csv, weekly-summary, decision gate, offer board, and experiment plan.</x:v>
+      </x:c>
+      <x:c r="N25" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="str">
+        <x:v>noah-luna_soft_offer-brief</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>noah-luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="C26" t="str">
+        <x:v>noah</x:v>
+      </x:c>
+      <x:c r="D26" t="str">
+        <x:v>諾雅</x:v>
+      </x:c>
+      <x:c r="E26" t="str">
+        <x:v>luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="F26" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G26" t="str">
+        <x:v>brief</x:v>
+      </x:c>
+      <x:c r="H26" t="str">
+        <x:v>Write a one-page asset brief with guardian, scene, promise boundary, and CTA.</x:v>
+      </x:c>
+      <x:c r="I26" t="str">
+        <x:v>noah-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="J26" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-noah</x:v>
+      </x:c>
+      <x:c r="K26" t="str">
+        <x:v>content</x:v>
+      </x:c>
+      <x:c r="L26" t="str">
+        <x:v>Brief keeps the Shorts CTA as quiz and places offer only after result route.</x:v>
+      </x:c>
+      <x:c r="M26" t="str">
+        <x:v>Update offer-experiment-plan after KPI review.</x:v>
+      </x:c>
+      <x:c r="N26" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>noah-luna_soft_offer-asset</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>noah-luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>noah</x:v>
+      </x:c>
+      <x:c r="D27" t="str">
+        <x:v>諾雅</x:v>
+      </x:c>
+      <x:c r="E27" t="str">
+        <x:v>luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="F27" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G27" t="str">
+        <x:v>asset</x:v>
+      </x:c>
+      <x:c r="H27" t="str">
+        <x:v>Produce the smallest useful asset or route copy for the experiment.</x:v>
+      </x:c>
+      <x:c r="I27" t="str">
+        <x:v>noah-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="J27" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-noah</x:v>
+      </x:c>
+      <x:c r="K27" t="str">
+        <x:v>creative</x:v>
+      </x:c>
+      <x:c r="L27" t="str">
+        <x:v>Asset links to the existing target URL and does not claim diagnosis or therapeutic outcome.</x:v>
+      </x:c>
+      <x:c r="M27" t="str">
+        <x:v>Record fulfillment asset in lead-intake-tracker.csv when a real request exists.</x:v>
+      </x:c>
+      <x:c r="N27" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>noah-luna_soft_offer-qa</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>noah-luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="C28" t="str">
+        <x:v>noah</x:v>
+      </x:c>
+      <x:c r="D28" t="str">
+        <x:v>諾雅</x:v>
+      </x:c>
+      <x:c r="E28" t="str">
+        <x:v>luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="F28" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G28" t="str">
+        <x:v>qa</x:v>
+      </x:c>
+      <x:c r="H28" t="str">
+        <x:v>Check safety copy, route, tracking event, and mobile presentation before publish.</x:v>
+      </x:c>
+      <x:c r="I28" t="str">
+        <x:v>noah-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="J28" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-noah</x:v>
+      </x:c>
+      <x:c r="K28" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L28" t="str">
+        <x:v>Public smoke remains clean and no paid CTA is added before the experiment is READY.</x:v>
+      </x:c>
+      <x:c r="M28" t="str">
+        <x:v>Run predeploy_check.py before deploy.</x:v>
+      </x:c>
+      <x:c r="N28" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
+        <x:v>noah-luna_soft_offer-measure</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>noah-luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="C29" t="str">
+        <x:v>noah</x:v>
+      </x:c>
+      <x:c r="D29" t="str">
+        <x:v>諾雅</x:v>
+      </x:c>
+      <x:c r="E29" t="str">
+        <x:v>luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="F29" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G29" t="str">
+        <x:v>measure</x:v>
+      </x:c>
+      <x:c r="H29" t="str">
+        <x:v>After the test window, backfill KPI fields and decide continue, revise, or stop.</x:v>
+      </x:c>
+      <x:c r="I29" t="str">
+        <x:v>noah-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="J29" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-noah</x:v>
+      </x:c>
+      <x:c r="K29" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L29" t="str">
+        <x:v>KPI row includes primary and secondary metric fields for the experiment.</x:v>
+      </x:c>
+      <x:c r="M29" t="str">
+        <x:v>Update kpi-tracker.csv, weekly-summary, decision gate, offer board, and experiment plan.</x:v>
+      </x:c>
+      <x:c r="N29" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="str">
+        <x:v>noah-affiliate_book-brief</x:v>
+      </x:c>
+      <x:c r="B30" t="str">
+        <x:v>noah-affiliate_book</x:v>
+      </x:c>
+      <x:c r="C30" t="str">
+        <x:v>noah</x:v>
+      </x:c>
+      <x:c r="D30" t="str">
+        <x:v>諾雅</x:v>
+      </x:c>
+      <x:c r="E30" t="str">
+        <x:v>affiliate_book</x:v>
+      </x:c>
+      <x:c r="F30" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G30" t="str">
+        <x:v>brief</x:v>
+      </x:c>
+      <x:c r="H30" t="str">
+        <x:v>Write a one-page asset brief with guardian, scene, promise boundary, and CTA.</x:v>
+      </x:c>
+      <x:c r="I30" t="str">
+        <x:v>noah-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="J30" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-noah</x:v>
+      </x:c>
+      <x:c r="K30" t="str">
+        <x:v>content</x:v>
+      </x:c>
+      <x:c r="L30" t="str">
+        <x:v>Brief keeps the Shorts CTA as quiz and places offer only after result route.</x:v>
+      </x:c>
+      <x:c r="M30" t="str">
+        <x:v>Update offer-experiment-plan after KPI review.</x:v>
+      </x:c>
+      <x:c r="N30" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" t="str">
+        <x:v>noah-affiliate_book-asset</x:v>
+      </x:c>
+      <x:c r="B31" t="str">
+        <x:v>noah-affiliate_book</x:v>
+      </x:c>
+      <x:c r="C31" t="str">
+        <x:v>noah</x:v>
+      </x:c>
+      <x:c r="D31" t="str">
+        <x:v>諾雅</x:v>
+      </x:c>
+      <x:c r="E31" t="str">
+        <x:v>affiliate_book</x:v>
+      </x:c>
+      <x:c r="F31" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G31" t="str">
+        <x:v>asset</x:v>
+      </x:c>
+      <x:c r="H31" t="str">
+        <x:v>Produce the smallest useful asset or route copy for the experiment.</x:v>
+      </x:c>
+      <x:c r="I31" t="str">
+        <x:v>noah-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="J31" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-noah</x:v>
+      </x:c>
+      <x:c r="K31" t="str">
+        <x:v>creative</x:v>
+      </x:c>
+      <x:c r="L31" t="str">
+        <x:v>Asset links to the existing target URL and does not claim diagnosis or therapeutic outcome.</x:v>
+      </x:c>
+      <x:c r="M31" t="str">
+        <x:v>Record fulfillment asset in lead-intake-tracker.csv when a real request exists.</x:v>
+      </x:c>
+      <x:c r="N31" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" t="str">
+        <x:v>noah-affiliate_book-qa</x:v>
+      </x:c>
+      <x:c r="B32" t="str">
+        <x:v>noah-affiliate_book</x:v>
+      </x:c>
+      <x:c r="C32" t="str">
+        <x:v>noah</x:v>
+      </x:c>
+      <x:c r="D32" t="str">
+        <x:v>諾雅</x:v>
+      </x:c>
+      <x:c r="E32" t="str">
+        <x:v>affiliate_book</x:v>
+      </x:c>
+      <x:c r="F32" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G32" t="str">
+        <x:v>qa</x:v>
+      </x:c>
+      <x:c r="H32" t="str">
+        <x:v>Check safety copy, route, tracking event, and mobile presentation before publish.</x:v>
+      </x:c>
+      <x:c r="I32" t="str">
+        <x:v>noah-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="J32" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-noah</x:v>
+      </x:c>
+      <x:c r="K32" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L32" t="str">
+        <x:v>Public smoke remains clean and no paid CTA is added before the experiment is READY.</x:v>
+      </x:c>
+      <x:c r="M32" t="str">
+        <x:v>Run predeploy_check.py before deploy.</x:v>
+      </x:c>
+      <x:c r="N32" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" t="str">
+        <x:v>noah-affiliate_book-measure</x:v>
+      </x:c>
+      <x:c r="B33" t="str">
+        <x:v>noah-affiliate_book</x:v>
+      </x:c>
+      <x:c r="C33" t="str">
+        <x:v>noah</x:v>
+      </x:c>
+      <x:c r="D33" t="str">
+        <x:v>諾雅</x:v>
+      </x:c>
+      <x:c r="E33" t="str">
+        <x:v>affiliate_book</x:v>
+      </x:c>
+      <x:c r="F33" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G33" t="str">
+        <x:v>measure</x:v>
+      </x:c>
+      <x:c r="H33" t="str">
+        <x:v>After the test window, backfill KPI fields and decide continue, revise, or stop.</x:v>
+      </x:c>
+      <x:c r="I33" t="str">
+        <x:v>noah-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="J33" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-noah</x:v>
+      </x:c>
+      <x:c r="K33" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L33" t="str">
+        <x:v>KPI row includes primary and secondary metric fields for the experiment.</x:v>
+      </x:c>
+      <x:c r="M33" t="str">
+        <x:v>Update kpi-tracker.csv, weekly-summary, decision gate, offer board, and experiment plan.</x:v>
+      </x:c>
+      <x:c r="N33" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" t="str">
+        <x:v>vivian-identity_save-brief</x:v>
+      </x:c>
+      <x:c r="B34" t="str">
+        <x:v>vivian-identity_save</x:v>
+      </x:c>
+      <x:c r="C34" t="str">
+        <x:v>vivian</x:v>
+      </x:c>
+      <x:c r="D34" t="str">
+        <x:v>薇薇安</x:v>
+      </x:c>
+      <x:c r="E34" t="str">
+        <x:v>identity_save</x:v>
+      </x:c>
+      <x:c r="F34" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G34" t="str">
+        <x:v>brief</x:v>
+      </x:c>
+      <x:c r="H34" t="str">
+        <x:v>Write a one-page asset brief with guardian, scene, promise boundary, and CTA.</x:v>
+      </x:c>
+      <x:c r="I34" t="str">
+        <x:v>vivian-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="J34" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-vivian</x:v>
+      </x:c>
+      <x:c r="K34" t="str">
+        <x:v>content</x:v>
+      </x:c>
+      <x:c r="L34" t="str">
+        <x:v>Brief keeps the Shorts CTA as quiz and places offer only after result route.</x:v>
+      </x:c>
+      <x:c r="M34" t="str">
+        <x:v>Update offer-experiment-plan after KPI review.</x:v>
+      </x:c>
+      <x:c r="N34" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" t="str">
+        <x:v>vivian-identity_save-asset</x:v>
+      </x:c>
+      <x:c r="B35" t="str">
+        <x:v>vivian-identity_save</x:v>
+      </x:c>
+      <x:c r="C35" t="str">
+        <x:v>vivian</x:v>
+      </x:c>
+      <x:c r="D35" t="str">
+        <x:v>薇薇安</x:v>
+      </x:c>
+      <x:c r="E35" t="str">
+        <x:v>identity_save</x:v>
+      </x:c>
+      <x:c r="F35" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G35" t="str">
+        <x:v>asset</x:v>
+      </x:c>
+      <x:c r="H35" t="str">
+        <x:v>Produce the smallest useful asset or route copy for the experiment.</x:v>
+      </x:c>
+      <x:c r="I35" t="str">
+        <x:v>vivian-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="J35" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-vivian</x:v>
+      </x:c>
+      <x:c r="K35" t="str">
+        <x:v>creative</x:v>
+      </x:c>
+      <x:c r="L35" t="str">
+        <x:v>Asset links to the existing target URL and does not claim diagnosis or therapeutic outcome.</x:v>
+      </x:c>
+      <x:c r="M35" t="str">
+        <x:v>Record fulfillment asset in lead-intake-tracker.csv when a real request exists.</x:v>
+      </x:c>
+      <x:c r="N35" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" t="str">
+        <x:v>vivian-identity_save-qa</x:v>
+      </x:c>
+      <x:c r="B36" t="str">
+        <x:v>vivian-identity_save</x:v>
+      </x:c>
+      <x:c r="C36" t="str">
+        <x:v>vivian</x:v>
+      </x:c>
+      <x:c r="D36" t="str">
+        <x:v>薇薇安</x:v>
+      </x:c>
+      <x:c r="E36" t="str">
+        <x:v>identity_save</x:v>
+      </x:c>
+      <x:c r="F36" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G36" t="str">
+        <x:v>qa</x:v>
+      </x:c>
+      <x:c r="H36" t="str">
+        <x:v>Check safety copy, route, tracking event, and mobile presentation before publish.</x:v>
+      </x:c>
+      <x:c r="I36" t="str">
+        <x:v>vivian-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="J36" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-vivian</x:v>
+      </x:c>
+      <x:c r="K36" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L36" t="str">
+        <x:v>Public smoke remains clean and no paid CTA is added before the experiment is READY.</x:v>
+      </x:c>
+      <x:c r="M36" t="str">
+        <x:v>Run predeploy_check.py before deploy.</x:v>
+      </x:c>
+      <x:c r="N36" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="str">
+        <x:v>vivian-identity_save-measure</x:v>
+      </x:c>
+      <x:c r="B37" t="str">
+        <x:v>vivian-identity_save</x:v>
+      </x:c>
+      <x:c r="C37" t="str">
+        <x:v>vivian</x:v>
+      </x:c>
+      <x:c r="D37" t="str">
+        <x:v>薇薇安</x:v>
+      </x:c>
+      <x:c r="E37" t="str">
+        <x:v>identity_save</x:v>
+      </x:c>
+      <x:c r="F37" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G37" t="str">
+        <x:v>measure</x:v>
+      </x:c>
+      <x:c r="H37" t="str">
+        <x:v>After the test window, backfill KPI fields and decide continue, revise, or stop.</x:v>
+      </x:c>
+      <x:c r="I37" t="str">
+        <x:v>vivian-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="J37" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-vivian</x:v>
+      </x:c>
+      <x:c r="K37" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L37" t="str">
+        <x:v>KPI row includes primary and secondary metric fields for the experiment.</x:v>
+      </x:c>
+      <x:c r="M37" t="str">
+        <x:v>Update kpi-tracker.csv, weekly-summary, decision gate, offer board, and experiment plan.</x:v>
+      </x:c>
+      <x:c r="N37" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" t="str">
+        <x:v>vivian-owned_lead-brief</x:v>
+      </x:c>
+      <x:c r="B38" t="str">
+        <x:v>vivian-owned_lead</x:v>
+      </x:c>
+      <x:c r="C38" t="str">
+        <x:v>vivian</x:v>
+      </x:c>
+      <x:c r="D38" t="str">
+        <x:v>薇薇安</x:v>
+      </x:c>
+      <x:c r="E38" t="str">
+        <x:v>owned_lead</x:v>
+      </x:c>
+      <x:c r="F38" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G38" t="str">
+        <x:v>brief</x:v>
+      </x:c>
+      <x:c r="H38" t="str">
+        <x:v>Write a one-page asset brief with guardian, scene, promise boundary, and CTA.</x:v>
+      </x:c>
+      <x:c r="I38" t="str">
+        <x:v>vivian-email_lead_template</x:v>
+      </x:c>
+      <x:c r="J38" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="K38" t="str">
+        <x:v>content</x:v>
+      </x:c>
+      <x:c r="L38" t="str">
+        <x:v>Brief keeps the Shorts CTA as quiz and places offer only after result route.</x:v>
+      </x:c>
+      <x:c r="M38" t="str">
+        <x:v>Update offer-experiment-plan after KPI review.</x:v>
+      </x:c>
+      <x:c r="N38" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" t="str">
+        <x:v>vivian-owned_lead-asset</x:v>
+      </x:c>
+      <x:c r="B39" t="str">
+        <x:v>vivian-owned_lead</x:v>
+      </x:c>
+      <x:c r="C39" t="str">
+        <x:v>vivian</x:v>
+      </x:c>
+      <x:c r="D39" t="str">
+        <x:v>薇薇安</x:v>
+      </x:c>
+      <x:c r="E39" t="str">
+        <x:v>owned_lead</x:v>
+      </x:c>
+      <x:c r="F39" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G39" t="str">
+        <x:v>asset</x:v>
+      </x:c>
+      <x:c r="H39" t="str">
+        <x:v>Produce the smallest useful asset or route copy for the experiment.</x:v>
+      </x:c>
+      <x:c r="I39" t="str">
+        <x:v>vivian-email_lead_template</x:v>
+      </x:c>
+      <x:c r="J39" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="K39" t="str">
+        <x:v>creative</x:v>
+      </x:c>
+      <x:c r="L39" t="str">
+        <x:v>Asset links to the existing target URL and does not claim diagnosis or therapeutic outcome.</x:v>
+      </x:c>
+      <x:c r="M39" t="str">
+        <x:v>Record fulfillment asset in lead-intake-tracker.csv when a real request exists.</x:v>
+      </x:c>
+      <x:c r="N39" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" t="str">
+        <x:v>vivian-owned_lead-qa</x:v>
+      </x:c>
+      <x:c r="B40" t="str">
+        <x:v>vivian-owned_lead</x:v>
+      </x:c>
+      <x:c r="C40" t="str">
+        <x:v>vivian</x:v>
+      </x:c>
+      <x:c r="D40" t="str">
+        <x:v>薇薇安</x:v>
+      </x:c>
+      <x:c r="E40" t="str">
+        <x:v>owned_lead</x:v>
+      </x:c>
+      <x:c r="F40" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G40" t="str">
+        <x:v>qa</x:v>
+      </x:c>
+      <x:c r="H40" t="str">
+        <x:v>Check safety copy, route, tracking event, and mobile presentation before publish.</x:v>
+      </x:c>
+      <x:c r="I40" t="str">
+        <x:v>vivian-email_lead_template</x:v>
+      </x:c>
+      <x:c r="J40" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="K40" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L40" t="str">
+        <x:v>Public smoke remains clean and no paid CTA is added before the experiment is READY.</x:v>
+      </x:c>
+      <x:c r="M40" t="str">
+        <x:v>Run predeploy_check.py before deploy.</x:v>
+      </x:c>
+      <x:c r="N40" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" t="str">
+        <x:v>vivian-owned_lead-measure</x:v>
+      </x:c>
+      <x:c r="B41" t="str">
+        <x:v>vivian-owned_lead</x:v>
+      </x:c>
+      <x:c r="C41" t="str">
+        <x:v>vivian</x:v>
+      </x:c>
+      <x:c r="D41" t="str">
+        <x:v>薇薇安</x:v>
+      </x:c>
+      <x:c r="E41" t="str">
+        <x:v>owned_lead</x:v>
+      </x:c>
+      <x:c r="F41" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G41" t="str">
+        <x:v>measure</x:v>
+      </x:c>
+      <x:c r="H41" t="str">
+        <x:v>After the test window, backfill KPI fields and decide continue, revise, or stop.</x:v>
+      </x:c>
+      <x:c r="I41" t="str">
+        <x:v>vivian-email_lead_template</x:v>
+      </x:c>
+      <x:c r="J41" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="K41" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L41" t="str">
+        <x:v>KPI row includes primary and secondary metric fields for the experiment.</x:v>
+      </x:c>
+      <x:c r="M41" t="str">
+        <x:v>Update kpi-tracker.csv, weekly-summary, decision gate, offer board, and experiment plan.</x:v>
+      </x:c>
+      <x:c r="N41" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" t="str">
+        <x:v>vivian-luna_soft_offer-brief</x:v>
+      </x:c>
+      <x:c r="B42" t="str">
+        <x:v>vivian-luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="C42" t="str">
+        <x:v>vivian</x:v>
+      </x:c>
+      <x:c r="D42" t="str">
+        <x:v>薇薇安</x:v>
+      </x:c>
+      <x:c r="E42" t="str">
+        <x:v>luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="F42" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G42" t="str">
+        <x:v>brief</x:v>
+      </x:c>
+      <x:c r="H42" t="str">
+        <x:v>Write a one-page asset brief with guardian, scene, promise boundary, and CTA.</x:v>
+      </x:c>
+      <x:c r="I42" t="str">
+        <x:v>vivian-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="J42" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-vivian</x:v>
+      </x:c>
+      <x:c r="K42" t="str">
+        <x:v>content</x:v>
+      </x:c>
+      <x:c r="L42" t="str">
+        <x:v>Brief keeps the Shorts CTA as quiz and places offer only after result route.</x:v>
+      </x:c>
+      <x:c r="M42" t="str">
+        <x:v>Update offer-experiment-plan after KPI review.</x:v>
+      </x:c>
+      <x:c r="N42" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" t="str">
+        <x:v>vivian-luna_soft_offer-asset</x:v>
+      </x:c>
+      <x:c r="B43" t="str">
+        <x:v>vivian-luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="C43" t="str">
+        <x:v>vivian</x:v>
+      </x:c>
+      <x:c r="D43" t="str">
+        <x:v>薇薇安</x:v>
+      </x:c>
+      <x:c r="E43" t="str">
+        <x:v>luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="F43" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G43" t="str">
+        <x:v>asset</x:v>
+      </x:c>
+      <x:c r="H43" t="str">
+        <x:v>Produce the smallest useful asset or route copy for the experiment.</x:v>
+      </x:c>
+      <x:c r="I43" t="str">
+        <x:v>vivian-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="J43" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-vivian</x:v>
+      </x:c>
+      <x:c r="K43" t="str">
+        <x:v>creative</x:v>
+      </x:c>
+      <x:c r="L43" t="str">
+        <x:v>Asset links to the existing target URL and does not claim diagnosis or therapeutic outcome.</x:v>
+      </x:c>
+      <x:c r="M43" t="str">
+        <x:v>Record fulfillment asset in lead-intake-tracker.csv when a real request exists.</x:v>
+      </x:c>
+      <x:c r="N43" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" t="str">
+        <x:v>vivian-luna_soft_offer-qa</x:v>
+      </x:c>
+      <x:c r="B44" t="str">
+        <x:v>vivian-luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="C44" t="str">
+        <x:v>vivian</x:v>
+      </x:c>
+      <x:c r="D44" t="str">
+        <x:v>薇薇安</x:v>
+      </x:c>
+      <x:c r="E44" t="str">
+        <x:v>luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="F44" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G44" t="str">
+        <x:v>qa</x:v>
+      </x:c>
+      <x:c r="H44" t="str">
+        <x:v>Check safety copy, route, tracking event, and mobile presentation before publish.</x:v>
+      </x:c>
+      <x:c r="I44" t="str">
+        <x:v>vivian-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="J44" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-vivian</x:v>
+      </x:c>
+      <x:c r="K44" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L44" t="str">
+        <x:v>Public smoke remains clean and no paid CTA is added before the experiment is READY.</x:v>
+      </x:c>
+      <x:c r="M44" t="str">
+        <x:v>Run predeploy_check.py before deploy.</x:v>
+      </x:c>
+      <x:c r="N44" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" t="str">
+        <x:v>vivian-luna_soft_offer-measure</x:v>
+      </x:c>
+      <x:c r="B45" t="str">
+        <x:v>vivian-luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="C45" t="str">
+        <x:v>vivian</x:v>
+      </x:c>
+      <x:c r="D45" t="str">
+        <x:v>薇薇安</x:v>
+      </x:c>
+      <x:c r="E45" t="str">
+        <x:v>luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="F45" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G45" t="str">
+        <x:v>measure</x:v>
+      </x:c>
+      <x:c r="H45" t="str">
+        <x:v>After the test window, backfill KPI fields and decide continue, revise, or stop.</x:v>
+      </x:c>
+      <x:c r="I45" t="str">
+        <x:v>vivian-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="J45" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-vivian</x:v>
+      </x:c>
+      <x:c r="K45" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L45" t="str">
+        <x:v>KPI row includes primary and secondary metric fields for the experiment.</x:v>
+      </x:c>
+      <x:c r="M45" t="str">
+        <x:v>Update kpi-tracker.csv, weekly-summary, decision gate, offer board, and experiment plan.</x:v>
+      </x:c>
+      <x:c r="N45" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" t="str">
+        <x:v>vivian-affiliate_book-brief</x:v>
+      </x:c>
+      <x:c r="B46" t="str">
+        <x:v>vivian-affiliate_book</x:v>
+      </x:c>
+      <x:c r="C46" t="str">
+        <x:v>vivian</x:v>
+      </x:c>
+      <x:c r="D46" t="str">
+        <x:v>薇薇安</x:v>
+      </x:c>
+      <x:c r="E46" t="str">
+        <x:v>affiliate_book</x:v>
+      </x:c>
+      <x:c r="F46" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G46" t="str">
+        <x:v>brief</x:v>
+      </x:c>
+      <x:c r="H46" t="str">
+        <x:v>Write a one-page asset brief with guardian, scene, promise boundary, and CTA.</x:v>
+      </x:c>
+      <x:c r="I46" t="str">
+        <x:v>vivian-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="J46" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-vivian</x:v>
+      </x:c>
+      <x:c r="K46" t="str">
+        <x:v>content</x:v>
+      </x:c>
+      <x:c r="L46" t="str">
+        <x:v>Brief keeps the Shorts CTA as quiz and places offer only after result route.</x:v>
+      </x:c>
+      <x:c r="M46" t="str">
+        <x:v>Update offer-experiment-plan after KPI review.</x:v>
+      </x:c>
+      <x:c r="N46" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" t="str">
+        <x:v>vivian-affiliate_book-asset</x:v>
+      </x:c>
+      <x:c r="B47" t="str">
+        <x:v>vivian-affiliate_book</x:v>
+      </x:c>
+      <x:c r="C47" t="str">
+        <x:v>vivian</x:v>
+      </x:c>
+      <x:c r="D47" t="str">
+        <x:v>薇薇安</x:v>
+      </x:c>
+      <x:c r="E47" t="str">
+        <x:v>affiliate_book</x:v>
+      </x:c>
+      <x:c r="F47" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G47" t="str">
+        <x:v>asset</x:v>
+      </x:c>
+      <x:c r="H47" t="str">
+        <x:v>Produce the smallest useful asset or route copy for the experiment.</x:v>
+      </x:c>
+      <x:c r="I47" t="str">
+        <x:v>vivian-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="J47" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-vivian</x:v>
+      </x:c>
+      <x:c r="K47" t="str">
+        <x:v>creative</x:v>
+      </x:c>
+      <x:c r="L47" t="str">
+        <x:v>Asset links to the existing target URL and does not claim diagnosis or therapeutic outcome.</x:v>
+      </x:c>
+      <x:c r="M47" t="str">
+        <x:v>Record fulfillment asset in lead-intake-tracker.csv when a real request exists.</x:v>
+      </x:c>
+      <x:c r="N47" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" t="str">
+        <x:v>vivian-affiliate_book-qa</x:v>
+      </x:c>
+      <x:c r="B48" t="str">
+        <x:v>vivian-affiliate_book</x:v>
+      </x:c>
+      <x:c r="C48" t="str">
+        <x:v>vivian</x:v>
+      </x:c>
+      <x:c r="D48" t="str">
+        <x:v>薇薇安</x:v>
+      </x:c>
+      <x:c r="E48" t="str">
+        <x:v>affiliate_book</x:v>
+      </x:c>
+      <x:c r="F48" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G48" t="str">
+        <x:v>qa</x:v>
+      </x:c>
+      <x:c r="H48" t="str">
+        <x:v>Check safety copy, route, tracking event, and mobile presentation before publish.</x:v>
+      </x:c>
+      <x:c r="I48" t="str">
+        <x:v>vivian-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="J48" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-vivian</x:v>
+      </x:c>
+      <x:c r="K48" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L48" t="str">
+        <x:v>Public smoke remains clean and no paid CTA is added before the experiment is READY.</x:v>
+      </x:c>
+      <x:c r="M48" t="str">
+        <x:v>Run predeploy_check.py before deploy.</x:v>
+      </x:c>
+      <x:c r="N48" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" t="str">
+        <x:v>vivian-affiliate_book-measure</x:v>
+      </x:c>
+      <x:c r="B49" t="str">
+        <x:v>vivian-affiliate_book</x:v>
+      </x:c>
+      <x:c r="C49" t="str">
+        <x:v>vivian</x:v>
+      </x:c>
+      <x:c r="D49" t="str">
+        <x:v>薇薇安</x:v>
+      </x:c>
+      <x:c r="E49" t="str">
+        <x:v>affiliate_book</x:v>
+      </x:c>
+      <x:c r="F49" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G49" t="str">
+        <x:v>measure</x:v>
+      </x:c>
+      <x:c r="H49" t="str">
+        <x:v>After the test window, backfill KPI fields and decide continue, revise, or stop.</x:v>
+      </x:c>
+      <x:c r="I49" t="str">
+        <x:v>vivian-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="J49" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-vivian</x:v>
+      </x:c>
+      <x:c r="K49" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L49" t="str">
+        <x:v>KPI row includes primary and secondary metric fields for the experiment.</x:v>
+      </x:c>
+      <x:c r="M49" t="str">
+        <x:v>Update kpi-tracker.csv, weekly-summary, decision gate, offer board, and experiment plan.</x:v>
+      </x:c>
+      <x:c r="N49" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" t="str">
+        <x:v>claire-identity_save-brief</x:v>
+      </x:c>
+      <x:c r="B50" t="str">
+        <x:v>claire-identity_save</x:v>
+      </x:c>
+      <x:c r="C50" t="str">
+        <x:v>claire</x:v>
+      </x:c>
+      <x:c r="D50" t="str">
+        <x:v>克萊兒</x:v>
+      </x:c>
+      <x:c r="E50" t="str">
+        <x:v>identity_save</x:v>
+      </x:c>
+      <x:c r="F50" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G50" t="str">
+        <x:v>brief</x:v>
+      </x:c>
+      <x:c r="H50" t="str">
+        <x:v>Write a one-page asset brief with guardian, scene, promise boundary, and CTA.</x:v>
+      </x:c>
+      <x:c r="I50" t="str">
+        <x:v>claire-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="J50" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-claire</x:v>
+      </x:c>
+      <x:c r="K50" t="str">
+        <x:v>content</x:v>
+      </x:c>
+      <x:c r="L50" t="str">
+        <x:v>Brief keeps the Shorts CTA as quiz and places offer only after result route.</x:v>
+      </x:c>
+      <x:c r="M50" t="str">
+        <x:v>Update offer-experiment-plan after KPI review.</x:v>
+      </x:c>
+      <x:c r="N50" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" t="str">
+        <x:v>claire-identity_save-asset</x:v>
+      </x:c>
+      <x:c r="B51" t="str">
+        <x:v>claire-identity_save</x:v>
+      </x:c>
+      <x:c r="C51" t="str">
+        <x:v>claire</x:v>
+      </x:c>
+      <x:c r="D51" t="str">
+        <x:v>克萊兒</x:v>
+      </x:c>
+      <x:c r="E51" t="str">
+        <x:v>identity_save</x:v>
+      </x:c>
+      <x:c r="F51" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G51" t="str">
+        <x:v>asset</x:v>
+      </x:c>
+      <x:c r="H51" t="str">
+        <x:v>Produce the smallest useful asset or route copy for the experiment.</x:v>
+      </x:c>
+      <x:c r="I51" t="str">
+        <x:v>claire-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="J51" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-claire</x:v>
+      </x:c>
+      <x:c r="K51" t="str">
+        <x:v>creative</x:v>
+      </x:c>
+      <x:c r="L51" t="str">
+        <x:v>Asset links to the existing target URL and does not claim diagnosis or therapeutic outcome.</x:v>
+      </x:c>
+      <x:c r="M51" t="str">
+        <x:v>Record fulfillment asset in lead-intake-tracker.csv when a real request exists.</x:v>
+      </x:c>
+      <x:c r="N51" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" t="str">
+        <x:v>claire-identity_save-qa</x:v>
+      </x:c>
+      <x:c r="B52" t="str">
+        <x:v>claire-identity_save</x:v>
+      </x:c>
+      <x:c r="C52" t="str">
+        <x:v>claire</x:v>
+      </x:c>
+      <x:c r="D52" t="str">
+        <x:v>克萊兒</x:v>
+      </x:c>
+      <x:c r="E52" t="str">
+        <x:v>identity_save</x:v>
+      </x:c>
+      <x:c r="F52" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G52" t="str">
+        <x:v>qa</x:v>
+      </x:c>
+      <x:c r="H52" t="str">
+        <x:v>Check safety copy, route, tracking event, and mobile presentation before publish.</x:v>
+      </x:c>
+      <x:c r="I52" t="str">
+        <x:v>claire-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="J52" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-claire</x:v>
+      </x:c>
+      <x:c r="K52" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L52" t="str">
+        <x:v>Public smoke remains clean and no paid CTA is added before the experiment is READY.</x:v>
+      </x:c>
+      <x:c r="M52" t="str">
+        <x:v>Run predeploy_check.py before deploy.</x:v>
+      </x:c>
+      <x:c r="N52" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" t="str">
+        <x:v>claire-identity_save-measure</x:v>
+      </x:c>
+      <x:c r="B53" t="str">
+        <x:v>claire-identity_save</x:v>
+      </x:c>
+      <x:c r="C53" t="str">
+        <x:v>claire</x:v>
+      </x:c>
+      <x:c r="D53" t="str">
+        <x:v>克萊兒</x:v>
+      </x:c>
+      <x:c r="E53" t="str">
+        <x:v>identity_save</x:v>
+      </x:c>
+      <x:c r="F53" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G53" t="str">
+        <x:v>measure</x:v>
+      </x:c>
+      <x:c r="H53" t="str">
+        <x:v>After the test window, backfill KPI fields and decide continue, revise, or stop.</x:v>
+      </x:c>
+      <x:c r="I53" t="str">
+        <x:v>claire-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="J53" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-claire</x:v>
+      </x:c>
+      <x:c r="K53" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L53" t="str">
+        <x:v>KPI row includes primary and secondary metric fields for the experiment.</x:v>
+      </x:c>
+      <x:c r="M53" t="str">
+        <x:v>Update kpi-tracker.csv, weekly-summary, decision gate, offer board, and experiment plan.</x:v>
+      </x:c>
+      <x:c r="N53" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" t="str">
+        <x:v>claire-owned_lead-brief</x:v>
+      </x:c>
+      <x:c r="B54" t="str">
+        <x:v>claire-owned_lead</x:v>
+      </x:c>
+      <x:c r="C54" t="str">
+        <x:v>claire</x:v>
+      </x:c>
+      <x:c r="D54" t="str">
+        <x:v>克萊兒</x:v>
+      </x:c>
+      <x:c r="E54" t="str">
+        <x:v>owned_lead</x:v>
+      </x:c>
+      <x:c r="F54" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G54" t="str">
+        <x:v>brief</x:v>
+      </x:c>
+      <x:c r="H54" t="str">
+        <x:v>Write a one-page asset brief with guardian, scene, promise boundary, and CTA.</x:v>
+      </x:c>
+      <x:c r="I54" t="str">
+        <x:v>claire-email_lead_template</x:v>
+      </x:c>
+      <x:c r="J54" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="K54" t="str">
+        <x:v>content</x:v>
+      </x:c>
+      <x:c r="L54" t="str">
+        <x:v>Brief keeps the Shorts CTA as quiz and places offer only after result route.</x:v>
+      </x:c>
+      <x:c r="M54" t="str">
+        <x:v>Update offer-experiment-plan after KPI review.</x:v>
+      </x:c>
+      <x:c r="N54" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" t="str">
+        <x:v>claire-owned_lead-asset</x:v>
+      </x:c>
+      <x:c r="B55" t="str">
+        <x:v>claire-owned_lead</x:v>
+      </x:c>
+      <x:c r="C55" t="str">
+        <x:v>claire</x:v>
+      </x:c>
+      <x:c r="D55" t="str">
+        <x:v>克萊兒</x:v>
+      </x:c>
+      <x:c r="E55" t="str">
+        <x:v>owned_lead</x:v>
+      </x:c>
+      <x:c r="F55" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G55" t="str">
+        <x:v>asset</x:v>
+      </x:c>
+      <x:c r="H55" t="str">
+        <x:v>Produce the smallest useful asset or route copy for the experiment.</x:v>
+      </x:c>
+      <x:c r="I55" t="str">
+        <x:v>claire-email_lead_template</x:v>
+      </x:c>
+      <x:c r="J55" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="K55" t="str">
+        <x:v>creative</x:v>
+      </x:c>
+      <x:c r="L55" t="str">
+        <x:v>Asset links to the existing target URL and does not claim diagnosis or therapeutic outcome.</x:v>
+      </x:c>
+      <x:c r="M55" t="str">
+        <x:v>Record fulfillment asset in lead-intake-tracker.csv when a real request exists.</x:v>
+      </x:c>
+      <x:c r="N55" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" t="str">
+        <x:v>claire-owned_lead-qa</x:v>
+      </x:c>
+      <x:c r="B56" t="str">
+        <x:v>claire-owned_lead</x:v>
+      </x:c>
+      <x:c r="C56" t="str">
+        <x:v>claire</x:v>
+      </x:c>
+      <x:c r="D56" t="str">
+        <x:v>克萊兒</x:v>
+      </x:c>
+      <x:c r="E56" t="str">
+        <x:v>owned_lead</x:v>
+      </x:c>
+      <x:c r="F56" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G56" t="str">
+        <x:v>qa</x:v>
+      </x:c>
+      <x:c r="H56" t="str">
+        <x:v>Check safety copy, route, tracking event, and mobile presentation before publish.</x:v>
+      </x:c>
+      <x:c r="I56" t="str">
+        <x:v>claire-email_lead_template</x:v>
+      </x:c>
+      <x:c r="J56" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="K56" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L56" t="str">
+        <x:v>Public smoke remains clean and no paid CTA is added before the experiment is READY.</x:v>
+      </x:c>
+      <x:c r="M56" t="str">
+        <x:v>Run predeploy_check.py before deploy.</x:v>
+      </x:c>
+      <x:c r="N56" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" t="str">
+        <x:v>claire-owned_lead-measure</x:v>
+      </x:c>
+      <x:c r="B57" t="str">
+        <x:v>claire-owned_lead</x:v>
+      </x:c>
+      <x:c r="C57" t="str">
+        <x:v>claire</x:v>
+      </x:c>
+      <x:c r="D57" t="str">
+        <x:v>克萊兒</x:v>
+      </x:c>
+      <x:c r="E57" t="str">
+        <x:v>owned_lead</x:v>
+      </x:c>
+      <x:c r="F57" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G57" t="str">
+        <x:v>measure</x:v>
+      </x:c>
+      <x:c r="H57" t="str">
+        <x:v>After the test window, backfill KPI fields and decide continue, revise, or stop.</x:v>
+      </x:c>
+      <x:c r="I57" t="str">
+        <x:v>claire-email_lead_template</x:v>
+      </x:c>
+      <x:c r="J57" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="K57" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L57" t="str">
+        <x:v>KPI row includes primary and secondary metric fields for the experiment.</x:v>
+      </x:c>
+      <x:c r="M57" t="str">
+        <x:v>Update kpi-tracker.csv, weekly-summary, decision gate, offer board, and experiment plan.</x:v>
+      </x:c>
+      <x:c r="N57" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" t="str">
+        <x:v>claire-luna_soft_offer-brief</x:v>
+      </x:c>
+      <x:c r="B58" t="str">
+        <x:v>claire-luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="C58" t="str">
+        <x:v>claire</x:v>
+      </x:c>
+      <x:c r="D58" t="str">
+        <x:v>克萊兒</x:v>
+      </x:c>
+      <x:c r="E58" t="str">
+        <x:v>luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="F58" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G58" t="str">
+        <x:v>brief</x:v>
+      </x:c>
+      <x:c r="H58" t="str">
+        <x:v>Write a one-page asset brief with guardian, scene, promise boundary, and CTA.</x:v>
+      </x:c>
+      <x:c r="I58" t="str">
+        <x:v>claire-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="J58" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-claire</x:v>
+      </x:c>
+      <x:c r="K58" t="str">
+        <x:v>content</x:v>
+      </x:c>
+      <x:c r="L58" t="str">
+        <x:v>Brief keeps the Shorts CTA as quiz and places offer only after result route.</x:v>
+      </x:c>
+      <x:c r="M58" t="str">
+        <x:v>Update offer-experiment-plan after KPI review.</x:v>
+      </x:c>
+      <x:c r="N58" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" t="str">
+        <x:v>claire-luna_soft_offer-asset</x:v>
+      </x:c>
+      <x:c r="B59" t="str">
+        <x:v>claire-luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="C59" t="str">
+        <x:v>claire</x:v>
+      </x:c>
+      <x:c r="D59" t="str">
+        <x:v>克萊兒</x:v>
+      </x:c>
+      <x:c r="E59" t="str">
+        <x:v>luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="F59" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G59" t="str">
+        <x:v>asset</x:v>
+      </x:c>
+      <x:c r="H59" t="str">
+        <x:v>Produce the smallest useful asset or route copy for the experiment.</x:v>
+      </x:c>
+      <x:c r="I59" t="str">
+        <x:v>claire-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="J59" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-claire</x:v>
+      </x:c>
+      <x:c r="K59" t="str">
+        <x:v>creative</x:v>
+      </x:c>
+      <x:c r="L59" t="str">
+        <x:v>Asset links to the existing target URL and does not claim diagnosis or therapeutic outcome.</x:v>
+      </x:c>
+      <x:c r="M59" t="str">
+        <x:v>Record fulfillment asset in lead-intake-tracker.csv when a real request exists.</x:v>
+      </x:c>
+      <x:c r="N59" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" t="str">
+        <x:v>claire-luna_soft_offer-qa</x:v>
+      </x:c>
+      <x:c r="B60" t="str">
+        <x:v>claire-luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="C60" t="str">
+        <x:v>claire</x:v>
+      </x:c>
+      <x:c r="D60" t="str">
+        <x:v>克萊兒</x:v>
+      </x:c>
+      <x:c r="E60" t="str">
+        <x:v>luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="F60" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G60" t="str">
+        <x:v>qa</x:v>
+      </x:c>
+      <x:c r="H60" t="str">
+        <x:v>Check safety copy, route, tracking event, and mobile presentation before publish.</x:v>
+      </x:c>
+      <x:c r="I60" t="str">
+        <x:v>claire-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="J60" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-claire</x:v>
+      </x:c>
+      <x:c r="K60" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L60" t="str">
+        <x:v>Public smoke remains clean and no paid CTA is added before the experiment is READY.</x:v>
+      </x:c>
+      <x:c r="M60" t="str">
+        <x:v>Run predeploy_check.py before deploy.</x:v>
+      </x:c>
+      <x:c r="N60" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" t="str">
+        <x:v>claire-luna_soft_offer-measure</x:v>
+      </x:c>
+      <x:c r="B61" t="str">
+        <x:v>claire-luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="C61" t="str">
+        <x:v>claire</x:v>
+      </x:c>
+      <x:c r="D61" t="str">
+        <x:v>克萊兒</x:v>
+      </x:c>
+      <x:c r="E61" t="str">
+        <x:v>luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="F61" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G61" t="str">
+        <x:v>measure</x:v>
+      </x:c>
+      <x:c r="H61" t="str">
+        <x:v>After the test window, backfill KPI fields and decide continue, revise, or stop.</x:v>
+      </x:c>
+      <x:c r="I61" t="str">
+        <x:v>claire-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="J61" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-claire</x:v>
+      </x:c>
+      <x:c r="K61" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L61" t="str">
+        <x:v>KPI row includes primary and secondary metric fields for the experiment.</x:v>
+      </x:c>
+      <x:c r="M61" t="str">
+        <x:v>Update kpi-tracker.csv, weekly-summary, decision gate, offer board, and experiment plan.</x:v>
+      </x:c>
+      <x:c r="N61" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" t="str">
+        <x:v>claire-affiliate_book-brief</x:v>
+      </x:c>
+      <x:c r="B62" t="str">
+        <x:v>claire-affiliate_book</x:v>
+      </x:c>
+      <x:c r="C62" t="str">
+        <x:v>claire</x:v>
+      </x:c>
+      <x:c r="D62" t="str">
+        <x:v>克萊兒</x:v>
+      </x:c>
+      <x:c r="E62" t="str">
+        <x:v>affiliate_book</x:v>
+      </x:c>
+      <x:c r="F62" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G62" t="str">
+        <x:v>brief</x:v>
+      </x:c>
+      <x:c r="H62" t="str">
+        <x:v>Write a one-page asset brief with guardian, scene, promise boundary, and CTA.</x:v>
+      </x:c>
+      <x:c r="I62" t="str">
+        <x:v>claire-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="J62" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-claire</x:v>
+      </x:c>
+      <x:c r="K62" t="str">
+        <x:v>content</x:v>
+      </x:c>
+      <x:c r="L62" t="str">
+        <x:v>Brief keeps the Shorts CTA as quiz and places offer only after result route.</x:v>
+      </x:c>
+      <x:c r="M62" t="str">
+        <x:v>Update offer-experiment-plan after KPI review.</x:v>
+      </x:c>
+      <x:c r="N62" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" t="str">
+        <x:v>claire-affiliate_book-asset</x:v>
+      </x:c>
+      <x:c r="B63" t="str">
+        <x:v>claire-affiliate_book</x:v>
+      </x:c>
+      <x:c r="C63" t="str">
+        <x:v>claire</x:v>
+      </x:c>
+      <x:c r="D63" t="str">
+        <x:v>克萊兒</x:v>
+      </x:c>
+      <x:c r="E63" t="str">
+        <x:v>affiliate_book</x:v>
+      </x:c>
+      <x:c r="F63" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G63" t="str">
+        <x:v>asset</x:v>
+      </x:c>
+      <x:c r="H63" t="str">
+        <x:v>Produce the smallest useful asset or route copy for the experiment.</x:v>
+      </x:c>
+      <x:c r="I63" t="str">
+        <x:v>claire-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="J63" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-claire</x:v>
+      </x:c>
+      <x:c r="K63" t="str">
+        <x:v>creative</x:v>
+      </x:c>
+      <x:c r="L63" t="str">
+        <x:v>Asset links to the existing target URL and does not claim diagnosis or therapeutic outcome.</x:v>
+      </x:c>
+      <x:c r="M63" t="str">
+        <x:v>Record fulfillment asset in lead-intake-tracker.csv when a real request exists.</x:v>
+      </x:c>
+      <x:c r="N63" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" t="str">
+        <x:v>claire-affiliate_book-qa</x:v>
+      </x:c>
+      <x:c r="B64" t="str">
+        <x:v>claire-affiliate_book</x:v>
+      </x:c>
+      <x:c r="C64" t="str">
+        <x:v>claire</x:v>
+      </x:c>
+      <x:c r="D64" t="str">
+        <x:v>克萊兒</x:v>
+      </x:c>
+      <x:c r="E64" t="str">
+        <x:v>affiliate_book</x:v>
+      </x:c>
+      <x:c r="F64" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G64" t="str">
+        <x:v>qa</x:v>
+      </x:c>
+      <x:c r="H64" t="str">
+        <x:v>Check safety copy, route, tracking event, and mobile presentation before publish.</x:v>
+      </x:c>
+      <x:c r="I64" t="str">
+        <x:v>claire-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="J64" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-claire</x:v>
+      </x:c>
+      <x:c r="K64" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L64" t="str">
+        <x:v>Public smoke remains clean and no paid CTA is added before the experiment is READY.</x:v>
+      </x:c>
+      <x:c r="M64" t="str">
+        <x:v>Run predeploy_check.py before deploy.</x:v>
+      </x:c>
+      <x:c r="N64" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" t="str">
+        <x:v>claire-affiliate_book-measure</x:v>
+      </x:c>
+      <x:c r="B65" t="str">
+        <x:v>claire-affiliate_book</x:v>
+      </x:c>
+      <x:c r="C65" t="str">
+        <x:v>claire</x:v>
+      </x:c>
+      <x:c r="D65" t="str">
+        <x:v>克萊兒</x:v>
+      </x:c>
+      <x:c r="E65" t="str">
+        <x:v>affiliate_book</x:v>
+      </x:c>
+      <x:c r="F65" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G65" t="str">
+        <x:v>measure</x:v>
+      </x:c>
+      <x:c r="H65" t="str">
+        <x:v>After the test window, backfill KPI fields and decide continue, revise, or stop.</x:v>
+      </x:c>
+      <x:c r="I65" t="str">
+        <x:v>claire-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="J65" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-claire</x:v>
+      </x:c>
+      <x:c r="K65" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L65" t="str">
+        <x:v>KPI row includes primary and secondary metric fields for the experiment.</x:v>
+      </x:c>
+      <x:c r="M65" t="str">
+        <x:v>Update kpi-tracker.csv, weekly-summary, decision gate, offer board, and experiment plan.</x:v>
+      </x:c>
+      <x:c r="N65" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" t="str">
+        <x:v>dora-identity_save-brief</x:v>
+      </x:c>
+      <x:c r="B66" t="str">
+        <x:v>dora-identity_save</x:v>
+      </x:c>
+      <x:c r="C66" t="str">
+        <x:v>dora</x:v>
+      </x:c>
+      <x:c r="D66" t="str">
+        <x:v>朵拉</x:v>
+      </x:c>
+      <x:c r="E66" t="str">
+        <x:v>identity_save</x:v>
+      </x:c>
+      <x:c r="F66" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G66" t="str">
+        <x:v>brief</x:v>
+      </x:c>
+      <x:c r="H66" t="str">
+        <x:v>Write a one-page asset brief with guardian, scene, promise boundary, and CTA.</x:v>
+      </x:c>
+      <x:c r="I66" t="str">
+        <x:v>dora-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="J66" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-dora</x:v>
+      </x:c>
+      <x:c r="K66" t="str">
+        <x:v>content</x:v>
+      </x:c>
+      <x:c r="L66" t="str">
+        <x:v>Brief keeps the Shorts CTA as quiz and places offer only after result route.</x:v>
+      </x:c>
+      <x:c r="M66" t="str">
+        <x:v>Update offer-experiment-plan after KPI review.</x:v>
+      </x:c>
+      <x:c r="N66" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" t="str">
+        <x:v>dora-identity_save-asset</x:v>
+      </x:c>
+      <x:c r="B67" t="str">
+        <x:v>dora-identity_save</x:v>
+      </x:c>
+      <x:c r="C67" t="str">
+        <x:v>dora</x:v>
+      </x:c>
+      <x:c r="D67" t="str">
+        <x:v>朵拉</x:v>
+      </x:c>
+      <x:c r="E67" t="str">
+        <x:v>identity_save</x:v>
+      </x:c>
+      <x:c r="F67" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G67" t="str">
+        <x:v>asset</x:v>
+      </x:c>
+      <x:c r="H67" t="str">
+        <x:v>Produce the smallest useful asset or route copy for the experiment.</x:v>
+      </x:c>
+      <x:c r="I67" t="str">
+        <x:v>dora-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="J67" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-dora</x:v>
+      </x:c>
+      <x:c r="K67" t="str">
+        <x:v>creative</x:v>
+      </x:c>
+      <x:c r="L67" t="str">
+        <x:v>Asset links to the existing target URL and does not claim diagnosis or therapeutic outcome.</x:v>
+      </x:c>
+      <x:c r="M67" t="str">
+        <x:v>Record fulfillment asset in lead-intake-tracker.csv when a real request exists.</x:v>
+      </x:c>
+      <x:c r="N67" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" t="str">
+        <x:v>dora-identity_save-qa</x:v>
+      </x:c>
+      <x:c r="B68" t="str">
+        <x:v>dora-identity_save</x:v>
+      </x:c>
+      <x:c r="C68" t="str">
+        <x:v>dora</x:v>
+      </x:c>
+      <x:c r="D68" t="str">
+        <x:v>朵拉</x:v>
+      </x:c>
+      <x:c r="E68" t="str">
+        <x:v>identity_save</x:v>
+      </x:c>
+      <x:c r="F68" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G68" t="str">
+        <x:v>qa</x:v>
+      </x:c>
+      <x:c r="H68" t="str">
+        <x:v>Check safety copy, route, tracking event, and mobile presentation before publish.</x:v>
+      </x:c>
+      <x:c r="I68" t="str">
+        <x:v>dora-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="J68" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-dora</x:v>
+      </x:c>
+      <x:c r="K68" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L68" t="str">
+        <x:v>Public smoke remains clean and no paid CTA is added before the experiment is READY.</x:v>
+      </x:c>
+      <x:c r="M68" t="str">
+        <x:v>Run predeploy_check.py before deploy.</x:v>
+      </x:c>
+      <x:c r="N68" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" t="str">
+        <x:v>dora-identity_save-measure</x:v>
+      </x:c>
+      <x:c r="B69" t="str">
+        <x:v>dora-identity_save</x:v>
+      </x:c>
+      <x:c r="C69" t="str">
+        <x:v>dora</x:v>
+      </x:c>
+      <x:c r="D69" t="str">
+        <x:v>朵拉</x:v>
+      </x:c>
+      <x:c r="E69" t="str">
+        <x:v>identity_save</x:v>
+      </x:c>
+      <x:c r="F69" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G69" t="str">
+        <x:v>measure</x:v>
+      </x:c>
+      <x:c r="H69" t="str">
+        <x:v>After the test window, backfill KPI fields and decide continue, revise, or stop.</x:v>
+      </x:c>
+      <x:c r="I69" t="str">
+        <x:v>dora-free_story_card_upgrade</x:v>
+      </x:c>
+      <x:c r="J69" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-dora</x:v>
+      </x:c>
+      <x:c r="K69" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L69" t="str">
+        <x:v>KPI row includes primary and secondary metric fields for the experiment.</x:v>
+      </x:c>
+      <x:c r="M69" t="str">
+        <x:v>Update kpi-tracker.csv, weekly-summary, decision gate, offer board, and experiment plan.</x:v>
+      </x:c>
+      <x:c r="N69" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" t="str">
+        <x:v>dora-owned_lead-brief</x:v>
+      </x:c>
+      <x:c r="B70" t="str">
+        <x:v>dora-owned_lead</x:v>
+      </x:c>
+      <x:c r="C70" t="str">
+        <x:v>dora</x:v>
+      </x:c>
+      <x:c r="D70" t="str">
+        <x:v>朵拉</x:v>
+      </x:c>
+      <x:c r="E70" t="str">
+        <x:v>owned_lead</x:v>
+      </x:c>
+      <x:c r="F70" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G70" t="str">
+        <x:v>brief</x:v>
+      </x:c>
+      <x:c r="H70" t="str">
+        <x:v>Write a one-page asset brief with guardian, scene, promise boundary, and CTA.</x:v>
+      </x:c>
+      <x:c r="I70" t="str">
+        <x:v>dora-email_lead_template</x:v>
+      </x:c>
+      <x:c r="J70" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="K70" t="str">
+        <x:v>content</x:v>
+      </x:c>
+      <x:c r="L70" t="str">
+        <x:v>Brief keeps the Shorts CTA as quiz and places offer only after result route.</x:v>
+      </x:c>
+      <x:c r="M70" t="str">
+        <x:v>Update offer-experiment-plan after KPI review.</x:v>
+      </x:c>
+      <x:c r="N70" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" t="str">
+        <x:v>dora-owned_lead-asset</x:v>
+      </x:c>
+      <x:c r="B71" t="str">
+        <x:v>dora-owned_lead</x:v>
+      </x:c>
+      <x:c r="C71" t="str">
+        <x:v>dora</x:v>
+      </x:c>
+      <x:c r="D71" t="str">
+        <x:v>朵拉</x:v>
+      </x:c>
+      <x:c r="E71" t="str">
+        <x:v>owned_lead</x:v>
+      </x:c>
+      <x:c r="F71" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G71" t="str">
+        <x:v>asset</x:v>
+      </x:c>
+      <x:c r="H71" t="str">
+        <x:v>Produce the smallest useful asset or route copy for the experiment.</x:v>
+      </x:c>
+      <x:c r="I71" t="str">
+        <x:v>dora-email_lead_template</x:v>
+      </x:c>
+      <x:c r="J71" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="K71" t="str">
+        <x:v>creative</x:v>
+      </x:c>
+      <x:c r="L71" t="str">
+        <x:v>Asset links to the existing target URL and does not claim diagnosis or therapeutic outcome.</x:v>
+      </x:c>
+      <x:c r="M71" t="str">
+        <x:v>Record fulfillment asset in lead-intake-tracker.csv when a real request exists.</x:v>
+      </x:c>
+      <x:c r="N71" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" t="str">
+        <x:v>dora-owned_lead-qa</x:v>
+      </x:c>
+      <x:c r="B72" t="str">
+        <x:v>dora-owned_lead</x:v>
+      </x:c>
+      <x:c r="C72" t="str">
+        <x:v>dora</x:v>
+      </x:c>
+      <x:c r="D72" t="str">
+        <x:v>朵拉</x:v>
+      </x:c>
+      <x:c r="E72" t="str">
+        <x:v>owned_lead</x:v>
+      </x:c>
+      <x:c r="F72" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G72" t="str">
+        <x:v>qa</x:v>
+      </x:c>
+      <x:c r="H72" t="str">
+        <x:v>Check safety copy, route, tracking event, and mobile presentation before publish.</x:v>
+      </x:c>
+      <x:c r="I72" t="str">
+        <x:v>dora-email_lead_template</x:v>
+      </x:c>
+      <x:c r="J72" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="K72" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L72" t="str">
+        <x:v>Public smoke remains clean and no paid CTA is added before the experiment is READY.</x:v>
+      </x:c>
+      <x:c r="M72" t="str">
+        <x:v>Run predeploy_check.py before deploy.</x:v>
+      </x:c>
+      <x:c r="N72" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" t="str">
+        <x:v>dora-owned_lead-measure</x:v>
+      </x:c>
+      <x:c r="B73" t="str">
+        <x:v>dora-owned_lead</x:v>
+      </x:c>
+      <x:c r="C73" t="str">
+        <x:v>dora</x:v>
+      </x:c>
+      <x:c r="D73" t="str">
+        <x:v>朵拉</x:v>
+      </x:c>
+      <x:c r="E73" t="str">
+        <x:v>owned_lead</x:v>
+      </x:c>
+      <x:c r="F73" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G73" t="str">
+        <x:v>measure</x:v>
+      </x:c>
+      <x:c r="H73" t="str">
+        <x:v>After the test window, backfill KPI fields and decide continue, revise, or stop.</x:v>
+      </x:c>
+      <x:c r="I73" t="str">
+        <x:v>dora-email_lead_template</x:v>
+      </x:c>
+      <x:c r="J73" t="str">
+        <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
+      </x:c>
+      <x:c r="K73" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L73" t="str">
+        <x:v>KPI row includes primary and secondary metric fields for the experiment.</x:v>
+      </x:c>
+      <x:c r="M73" t="str">
+        <x:v>Update kpi-tracker.csv, weekly-summary, decision gate, offer board, and experiment plan.</x:v>
+      </x:c>
+      <x:c r="N73" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" t="str">
+        <x:v>dora-luna_soft_offer-brief</x:v>
+      </x:c>
+      <x:c r="B74" t="str">
+        <x:v>dora-luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="C74" t="str">
+        <x:v>dora</x:v>
+      </x:c>
+      <x:c r="D74" t="str">
+        <x:v>朵拉</x:v>
+      </x:c>
+      <x:c r="E74" t="str">
+        <x:v>luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="F74" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G74" t="str">
+        <x:v>brief</x:v>
+      </x:c>
+      <x:c r="H74" t="str">
+        <x:v>Write a one-page asset brief with guardian, scene, promise boundary, and CTA.</x:v>
+      </x:c>
+      <x:c r="I74" t="str">
+        <x:v>dora-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="J74" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-dora</x:v>
+      </x:c>
+      <x:c r="K74" t="str">
+        <x:v>content</x:v>
+      </x:c>
+      <x:c r="L74" t="str">
+        <x:v>Brief keeps the Shorts CTA as quiz and places offer only after result route.</x:v>
+      </x:c>
+      <x:c r="M74" t="str">
+        <x:v>Update offer-experiment-plan after KPI review.</x:v>
+      </x:c>
+      <x:c r="N74" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" t="str">
+        <x:v>dora-luna_soft_offer-asset</x:v>
+      </x:c>
+      <x:c r="B75" t="str">
+        <x:v>dora-luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="C75" t="str">
+        <x:v>dora</x:v>
+      </x:c>
+      <x:c r="D75" t="str">
+        <x:v>朵拉</x:v>
+      </x:c>
+      <x:c r="E75" t="str">
+        <x:v>luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="F75" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G75" t="str">
+        <x:v>asset</x:v>
+      </x:c>
+      <x:c r="H75" t="str">
+        <x:v>Produce the smallest useful asset or route copy for the experiment.</x:v>
+      </x:c>
+      <x:c r="I75" t="str">
+        <x:v>dora-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="J75" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-dora</x:v>
+      </x:c>
+      <x:c r="K75" t="str">
+        <x:v>creative</x:v>
+      </x:c>
+      <x:c r="L75" t="str">
+        <x:v>Asset links to the existing target URL and does not claim diagnosis or therapeutic outcome.</x:v>
+      </x:c>
+      <x:c r="M75" t="str">
+        <x:v>Record fulfillment asset in lead-intake-tracker.csv when a real request exists.</x:v>
+      </x:c>
+      <x:c r="N75" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" t="str">
+        <x:v>dora-luna_soft_offer-qa</x:v>
+      </x:c>
+      <x:c r="B76" t="str">
+        <x:v>dora-luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="C76" t="str">
+        <x:v>dora</x:v>
+      </x:c>
+      <x:c r="D76" t="str">
+        <x:v>朵拉</x:v>
+      </x:c>
+      <x:c r="E76" t="str">
+        <x:v>luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="F76" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G76" t="str">
+        <x:v>qa</x:v>
+      </x:c>
+      <x:c r="H76" t="str">
+        <x:v>Check safety copy, route, tracking event, and mobile presentation before publish.</x:v>
+      </x:c>
+      <x:c r="I76" t="str">
+        <x:v>dora-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="J76" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-dora</x:v>
+      </x:c>
+      <x:c r="K76" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L76" t="str">
+        <x:v>Public smoke remains clean and no paid CTA is added before the experiment is READY.</x:v>
+      </x:c>
+      <x:c r="M76" t="str">
+        <x:v>Run predeploy_check.py before deploy.</x:v>
+      </x:c>
+      <x:c r="N76" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" t="str">
+        <x:v>dora-luna_soft_offer-measure</x:v>
+      </x:c>
+      <x:c r="B77" t="str">
+        <x:v>dora-luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="C77" t="str">
+        <x:v>dora</x:v>
+      </x:c>
+      <x:c r="D77" t="str">
+        <x:v>朵拉</x:v>
+      </x:c>
+      <x:c r="E77" t="str">
+        <x:v>luna_soft_offer</x:v>
+      </x:c>
+      <x:c r="F77" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G77" t="str">
+        <x:v>measure</x:v>
+      </x:c>
+      <x:c r="H77" t="str">
+        <x:v>After the test window, backfill KPI fields and decide continue, revise, or stop.</x:v>
+      </x:c>
+      <x:c r="I77" t="str">
+        <x:v>dora-luna_scene_cta</x:v>
+      </x:c>
+      <x:c r="J77" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-dora</x:v>
+      </x:c>
+      <x:c r="K77" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L77" t="str">
+        <x:v>KPI row includes primary and secondary metric fields for the experiment.</x:v>
+      </x:c>
+      <x:c r="M77" t="str">
+        <x:v>Update kpi-tracker.csv, weekly-summary, decision gate, offer board, and experiment plan.</x:v>
+      </x:c>
+      <x:c r="N77" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" t="str">
+        <x:v>dora-affiliate_book-brief</x:v>
+      </x:c>
+      <x:c r="B78" t="str">
+        <x:v>dora-affiliate_book</x:v>
+      </x:c>
+      <x:c r="C78" t="str">
+        <x:v>dora</x:v>
+      </x:c>
+      <x:c r="D78" t="str">
+        <x:v>朵拉</x:v>
+      </x:c>
+      <x:c r="E78" t="str">
+        <x:v>affiliate_book</x:v>
+      </x:c>
+      <x:c r="F78" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G78" t="str">
+        <x:v>brief</x:v>
+      </x:c>
+      <x:c r="H78" t="str">
+        <x:v>Write a one-page asset brief with guardian, scene, promise boundary, and CTA.</x:v>
+      </x:c>
+      <x:c r="I78" t="str">
+        <x:v>dora-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="J78" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-dora</x:v>
+      </x:c>
+      <x:c r="K78" t="str">
+        <x:v>content</x:v>
+      </x:c>
+      <x:c r="L78" t="str">
+        <x:v>Brief keeps the Shorts CTA as quiz and places offer only after result route.</x:v>
+      </x:c>
+      <x:c r="M78" t="str">
+        <x:v>Update offer-experiment-plan after KPI review.</x:v>
+      </x:c>
+      <x:c r="N78" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" t="str">
+        <x:v>dora-affiliate_book-asset</x:v>
+      </x:c>
+      <x:c r="B79" t="str">
+        <x:v>dora-affiliate_book</x:v>
+      </x:c>
+      <x:c r="C79" t="str">
+        <x:v>dora</x:v>
+      </x:c>
+      <x:c r="D79" t="str">
+        <x:v>朵拉</x:v>
+      </x:c>
+      <x:c r="E79" t="str">
+        <x:v>affiliate_book</x:v>
+      </x:c>
+      <x:c r="F79" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G79" t="str">
+        <x:v>asset</x:v>
+      </x:c>
+      <x:c r="H79" t="str">
+        <x:v>Produce the smallest useful asset or route copy for the experiment.</x:v>
+      </x:c>
+      <x:c r="I79" t="str">
+        <x:v>dora-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="J79" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-dora</x:v>
+      </x:c>
+      <x:c r="K79" t="str">
+        <x:v>creative</x:v>
+      </x:c>
+      <x:c r="L79" t="str">
+        <x:v>Asset links to the existing target URL and does not claim diagnosis or therapeutic outcome.</x:v>
+      </x:c>
+      <x:c r="M79" t="str">
+        <x:v>Record fulfillment asset in lead-intake-tracker.csv when a real request exists.</x:v>
+      </x:c>
+      <x:c r="N79" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" t="str">
+        <x:v>dora-affiliate_book-qa</x:v>
+      </x:c>
+      <x:c r="B80" t="str">
+        <x:v>dora-affiliate_book</x:v>
+      </x:c>
+      <x:c r="C80" t="str">
+        <x:v>dora</x:v>
+      </x:c>
+      <x:c r="D80" t="str">
+        <x:v>朵拉</x:v>
+      </x:c>
+      <x:c r="E80" t="str">
+        <x:v>affiliate_book</x:v>
+      </x:c>
+      <x:c r="F80" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G80" t="str">
+        <x:v>qa</x:v>
+      </x:c>
+      <x:c r="H80" t="str">
+        <x:v>Check safety copy, route, tracking event, and mobile presentation before publish.</x:v>
+      </x:c>
+      <x:c r="I80" t="str">
+        <x:v>dora-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="J80" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-dora</x:v>
+      </x:c>
+      <x:c r="K80" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L80" t="str">
+        <x:v>Public smoke remains clean and no paid CTA is added before the experiment is READY.</x:v>
+      </x:c>
+      <x:c r="M80" t="str">
+        <x:v>Run predeploy_check.py before deploy.</x:v>
+      </x:c>
+      <x:c r="N80" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" t="str">
+        <x:v>dora-affiliate_book-measure</x:v>
+      </x:c>
+      <x:c r="B81" t="str">
+        <x:v>dora-affiliate_book</x:v>
+      </x:c>
+      <x:c r="C81" t="str">
+        <x:v>dora</x:v>
+      </x:c>
+      <x:c r="D81" t="str">
+        <x:v>朵拉</x:v>
+      </x:c>
+      <x:c r="E81" t="str">
+        <x:v>affiliate_book</x:v>
+      </x:c>
+      <x:c r="F81" t="str">
+        <x:v>blocked_by_gate</x:v>
+      </x:c>
+      <x:c r="G81" t="str">
+        <x:v>measure</x:v>
+      </x:c>
+      <x:c r="H81" t="str">
+        <x:v>After the test window, backfill KPI fields and decide continue, revise, or stop.</x:v>
+      </x:c>
+      <x:c r="I81" t="str">
+        <x:v>dora-affiliate_book_bundle</x:v>
+      </x:c>
+      <x:c r="J81" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-dora</x:v>
+      </x:c>
+      <x:c r="K81" t="str">
+        <x:v>ops</x:v>
+      </x:c>
+      <x:c r="L81" t="str">
+        <x:v>KPI row includes primary and secondary metric fields for the experiment.</x:v>
+      </x:c>
+      <x:c r="M81" t="str">
+        <x:v>Update kpi-tracker.csv, weekly-summary, decision gate, offer board, and experiment plan.</x:v>
+      </x:c>
+      <x:c r="N81" t="str">
+        <x:v>只在結果後、旅人補給、Luna 或 Contact 路線測試；不診斷、不承諾療效、不要求購買。</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
         <x:v>Week 1 Profile Gates</x:v>
       </x:c>
       <x:c r="B1" t="str"/>
@@ -4360,7 +8071,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
@@ -4531,125 +8242,4 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" t="str">
-        <x:v>Field</x:v>
-      </x:c>
-      <x:c r="B1" t="str">
-        <x:v>Meaning</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" t="str">
-        <x:v>site_clicks</x:v>
-      </x:c>
-      <x:c r="B2" t="str">
-        <x:v>Clicks from social profile/caption into LoveTypes.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" t="str">
-        <x:v>quiz_starts</x:v>
-      </x:c>
-      <x:c r="B3" t="str">
-        <x:v>Sessions where the 15-question guardian quiz begins.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" t="str">
-        <x:v>quiz_completions</x:v>
-      </x:c>
-      <x:c r="B4" t="str">
-        <x:v>Completed quiz sessions; primary first-round KPI.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" t="str">
-        <x:v>profile_clicks</x:v>
-      </x:c>
-      <x:c r="B5" t="str">
-        <x:v>Clicks on social Bio/Profile links before visitors reach LoveTypes.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" t="str">
-        <x:v>profile_link_set_date</x:v>
-      </x:c>
-      <x:c r="B6" t="str">
-        <x:v>Date the platform Bio/Profile tracked link was set live.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" t="str">
-        <x:v>free_keepsake_downloads</x:v>
-      </x:c>
-      <x:c r="B7" t="str">
-        <x:v>Guardian identity asset save or print intent.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" t="str">
-        <x:v>supply_lead_requests</x:v>
-      </x:c>
-      <x:c r="B8" t="str">
-        <x:v>Owned email/request demand for guardian supply assets.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" t="str">
-        <x:v>luna_pack_clicks</x:v>
-      </x:c>
-      <x:c r="B9" t="str">
-        <x:v>Luna Gumroad product exploration.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" t="str">
-        <x:v>affiliate_book_clicks</x:v>
-      </x:c>
-      <x:c r="B10" t="str">
-        <x:v>Affiliate book route exploration.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" t="str">
-        <x:v>contact_requests</x:v>
-      </x:c>
-      <x:c r="B11" t="str">
-        <x:v>High-intent contact or path-summary mailto request.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" t="str">
-        <x:v>lead-intake-tracker.csv</x:v>
-      </x:c>
-      <x:c r="B12" t="str">
-        <x:v>Template rows for real Contact, waitlist, Luna, or repair supply requests. Template rows are not user data.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" t="str">
-        <x:v>offer-hypothesis-board.csv</x:v>
-      </x:c>
-      <x:c r="B13" t="str">
-        <x:v>Guardian-level offer hypotheses and readiness gates. HOLD rows must not change public paid CTA priority.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" t="str">
-        <x:v>offer-experiment-plan.csv</x:v>
-      </x:c>
-      <x:c r="B14" t="str">
-        <x:v>Guarded product experiment thresholds for free assets, owned leads, Luna, and affiliate book tests.</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add promotion launch command center
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,16 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3d479846c0554519"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R16a314dea9744d24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R64c42393f9104428"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="Rb7eeef88ef19449f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="Refa22eca0c3a461a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="Rbce1e3f47c7f410a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="Rc3802c0932594a1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="8" r:id="Ra1a35650123e4bcc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="9" r:id="R2ef0cd0c178b47f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="10" r:id="Ra865138427c340c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R75b9cfccbcf84696"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R2c76153eee054350"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R12d2bd2376574a9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R5c861a12aac44df7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="R7d5de031636c44d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="R7b3b549dac914ec4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="R9c3e424ac65540bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="Ra2a9aee467334bf7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="Ra6ae868120ef4219"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="R1017824211a4425c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="R7f594d6e68b74b49"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -280,51 +281,51 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
-        <x:v>Week 1 profile gates pending</x:v>
+        <x:v>Launch command rows</x:v>
       </x:c>
       <x:c r="B11" t="n">
-        <x:v>3</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
-        <x:v>Week 1 platform posts</x:v>
+        <x:v>Week 1 profile gates pending</x:v>
       </x:c>
       <x:c r="B12" t="n">
-        <x:v>9</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
+        <x:v>Week 1 platform posts</x:v>
+      </x:c>
+      <x:c r="B13" t="n">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
         <x:v>Empty data safety mode</x:v>
       </x:c>
-      <x:c r="B13" t="str">
+      <x:c r="B14" t="str">
         <x:v>YES</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" t="str"/>
-      <x:c r="B14" t="str"/>
-    </x:row>
     <x:row r="15">
-      <x:c r="A15" t="str">
-        <x:v>Metric</x:v>
-      </x:c>
-      <x:c r="B15" t="str">
-        <x:v>Value</x:v>
-      </x:c>
+      <x:c r="A15" t="str"/>
+      <x:c r="B15" t="str"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
-        <x:v>Views</x:v>
-      </x:c>
-      <x:c r="B16" t="n">
-        <x:v>0</x:v>
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>Value</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">
-        <x:v>Site clicks</x:v>
+        <x:v>Views</x:v>
       </x:c>
       <x:c r="B17" t="n">
         <x:v>0</x:v>
@@ -332,7 +333,7 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="str">
-        <x:v>Quiz starts</x:v>
+        <x:v>Site clicks</x:v>
       </x:c>
       <x:c r="B18" t="n">
         <x:v>0</x:v>
@@ -340,7 +341,7 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" t="str">
-        <x:v>Quiz completions</x:v>
+        <x:v>Quiz starts</x:v>
       </x:c>
       <x:c r="B19" t="n">
         <x:v>0</x:v>
@@ -348,7 +349,7 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" t="str">
-        <x:v>Route interest</x:v>
+        <x:v>Quiz completions</x:v>
       </x:c>
       <x:c r="B20" t="n">
         <x:v>0</x:v>
@@ -356,7 +357,7 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" t="str">
-        <x:v>Revenue intent</x:v>
+        <x:v>Route interest</x:v>
       </x:c>
       <x:c r="B21" t="n">
         <x:v>0</x:v>
@@ -364,36 +365,36 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" t="str">
-        <x:v>Lead intent</x:v>
+        <x:v>Revenue intent</x:v>
       </x:c>
       <x:c r="B22" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" t="str"/>
-      <x:c r="B23" t="str"/>
+      <x:c r="A23" t="str">
+        <x:v>Lead intent</x:v>
+      </x:c>
+      <x:c r="B23" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" t="str">
-        <x:v>Recommended actions</x:v>
-      </x:c>
+      <x:c r="A24" t="str"/>
       <x:c r="B24" t="str"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" t="str">
-        <x:v>high</x:v>
-      </x:c>
-      <x:c r="B25" t="str">
-        <x:v>發布 Week 1 前 3 支 Shorts，先取得測驗完成樣本。</x:v>
-      </x:c>
+        <x:v>Recommended actions</x:v>
+      </x:c>
+      <x:c r="B25" t="str"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" t="str">
         <x:v>high</x:v>
       </x:c>
       <x:c r="B26" t="str">
-        <x:v>發布後至少回填 post_url、site_clicks、quiz_starts、quiz_completions。</x:v>
+        <x:v>發布 Week 1 前 3 支 Shorts，先取得測驗完成樣本。</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -401,7 +402,7 @@
         <x:v>high</x:v>
       </x:c>
       <x:c r="B27" t="str">
-        <x:v>發布前同步完成 YouTube、TikTok、Instagram 的 Bio/Profile link，使用平台專屬 UTM。</x:v>
+        <x:v>發布後至少回填 post_url、site_clicks、quiz_starts、quiz_completions。</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -409,14 +410,22 @@
         <x:v>high</x:v>
       </x:c>
       <x:c r="B28" t="str">
-        <x:v>平台首頁設定後回填 platform-profile-tracker.csv 的 status、profile_link_set_date、profile_clicks、site_clicks、quiz_starts、quiz_completions。</x:v>
+        <x:v>發布前同步完成 YouTube、TikTok、Instagram 的 Bio/Profile link，使用平台專屬 UTM。</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>平台首頁設定後回填 platform-profile-tracker.csv 的 status、profile_link_set_date、profile_clicks、site_clicks、quiz_starts、quiz_completions。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="str">
         <x:v>medium</x:v>
       </x:c>
-      <x:c r="B29" t="str">
+      <x:c r="B30" t="str">
         <x:v>目前沒有回填數據，不調整商品、守護者優先序或付費 CTA。</x:v>
       </x:c>
     </x:row>
@@ -431,6 +440,179 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
+        <x:v>taskId</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>week</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>slot</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>guardianId</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
+        <x:v>guardianName</x:v>
+      </x:c>
+      <x:c r="F1" t="str">
+        <x:v>contentAngle</x:v>
+      </x:c>
+      <x:c r="G1" t="str">
+        <x:v>title</x:v>
+      </x:c>
+      <x:c r="H1" t="str">
+        <x:v>trackedUrl</x:v>
+      </x:c>
+      <x:c r="I1" t="str">
+        <x:v>primaryFreeItemId</x:v>
+      </x:c>
+      <x:c r="J1" t="str">
+        <x:v>ownedLeadItemId</x:v>
+      </x:c>
+      <x:c r="K1" t="str">
+        <x:v>supplyRoute</x:v>
+      </x:c>
+      <x:c r="L1" t="str">
+        <x:v>lunaScene</x:v>
+      </x:c>
+      <x:c r="M1" t="str">
+        <x:v>keepsake</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>publish-lt-s01-iris-silence</x:v>
+      </x:c>
+      <x:c r="B2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="E2" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="F2" t="str">
+        <x:v>情感錯頻情境</x:v>
+      </x:c>
+      <x:c r="G2" t="str">
+        <x:v>他沉默時，你最想聽見哪一句話？</x:v>
+      </x:c>
+      <x:c r="H2" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_silence</x:v>
+      </x:c>
+      <x:c r="I2" t="str">
+        <x:v>free-keepsake-iris</x:v>
+      </x:c>
+      <x:c r="J2" t="str">
+        <x:v>supply-wishlist-iris</x:v>
+      </x:c>
+      <x:c r="K2" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-iris</x:v>
+      </x:c>
+      <x:c r="L2" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-iris</x:v>
+      </x:c>
+      <x:c r="M2" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-iris</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>publish-lt-s02-iris-affirmation</x:v>
+      </x:c>
+      <x:c r="B3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="E3" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="F3" t="str">
+        <x:v>守護者人格認同</x:v>
+      </x:c>
+      <x:c r="G3" t="str">
+        <x:v>哪一句肯定，會讓你瞬間安心？</x:v>
+      </x:c>
+      <x:c r="H3" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_affirmation</x:v>
+      </x:c>
+      <x:c r="I3" t="str">
+        <x:v>free-keepsake-iris</x:v>
+      </x:c>
+      <x:c r="J3" t="str">
+        <x:v>supply-wishlist-iris</x:v>
+      </x:c>
+      <x:c r="K3" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-iris</x:v>
+      </x:c>
+      <x:c r="L3" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-iris</x:v>
+      </x:c>
+      <x:c r="M3" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-iris</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>publish-lt-s03-iris-too-sensitive</x:v>
+      </x:c>
+      <x:c r="B4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C4" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>測驗入口</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>你真的太敏感嗎？還是你只是等一句清楚的話？</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_too_sensitive</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>free-keepsake-iris</x:v>
+      </x:c>
+      <x:c r="J4" t="str">
+        <x:v>supply-wishlist-iris</x:v>
+      </x:c>
+      <x:c r="K4" t="str">
+        <x:v>https://lovetypes.tw/resources/#supply-iris</x:v>
+      </x:c>
+      <x:c r="L4" t="str">
+        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-iris</x:v>
+      </x:c>
+      <x:c r="M4" t="str">
+        <x:v>https://lovetypes.tw/keepsakes/#keepsake-iris</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
         <x:v>Field</x:v>
       </x:c>
       <x:c r="B1" t="str">
@@ -547,6 +729,14 @@
       </x:c>
       <x:c r="B15" t="str">
         <x:v>Execution queue for READY offer experiments. Blocked rows must not be produced as public assets.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>launch-command-center.csv</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>Daily execution command board for profile setup, asset checks, Week 1 publishing, and KPI writeback.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7373,6 +7563,1286 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
+        <x:v>sequence</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>phase</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>priority</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
+        <x:v>platform</x:v>
+      </x:c>
+      <x:c r="F1" t="str">
+        <x:v>task_id</x:v>
+      </x:c>
+      <x:c r="G1" t="str">
+        <x:v>script_id</x:v>
+      </x:c>
+      <x:c r="H1" t="str">
+        <x:v>guardian_id</x:v>
+      </x:c>
+      <x:c r="I1" t="str">
+        <x:v>guardian_name</x:v>
+      </x:c>
+      <x:c r="J1" t="str">
+        <x:v>title</x:v>
+      </x:c>
+      <x:c r="K1" t="str">
+        <x:v>scheduled_date</x:v>
+      </x:c>
+      <x:c r="L1" t="str">
+        <x:v>scheduled_time</x:v>
+      </x:c>
+      <x:c r="M1" t="str">
+        <x:v>tracked_url</x:v>
+      </x:c>
+      <x:c r="N1" t="str">
+        <x:v>action</x:v>
+      </x:c>
+      <x:c r="O1" t="str">
+        <x:v>writeback</x:v>
+      </x:c>
+      <x:c r="P1" t="str">
+        <x:v>blocked_by</x:v>
+      </x:c>
+      <x:c r="Q1" t="str">
+        <x:v>safety_note</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>profile_setup</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="E2" t="str">
+        <x:v>youtube_shorts</x:v>
+      </x:c>
+      <x:c r="F2" t="str">
+        <x:v>profile-youtube_shorts</x:v>
+      </x:c>
+      <x:c r="G2" t="str"/>
+      <x:c r="H2" t="str"/>
+      <x:c r="I2" t="str"/>
+      <x:c r="J2" t="str">
+        <x:v>設定 YouTube Shorts 個人頁入口</x:v>
+      </x:c>
+      <x:c r="K2" t="str"/>
+      <x:c r="L2" t="str"/>
+      <x:c r="M2" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=youtube&amp;utm_medium=social_profile&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=youtube_shorts_bio</x:v>
+      </x:c>
+      <x:c r="N2" t="str">
+        <x:v>把 Bio/Profile link 設為 Channel description / video description，並放上置頂留言。</x:v>
+      </x:c>
+      <x:c r="O2" t="str">
+        <x:v>status=set/live, profile_link_set_date, profile_clicks, site_clicks, quiz_starts, quiz_completions</x:v>
+      </x:c>
+      <x:c r="P2" t="str"/>
+      <x:c r="Q2" t="str">
+        <x:v>入口只導向 15 題測驗，不導購、不承諾療效。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>profile_setup</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="E3" t="str">
+        <x:v>tiktok</x:v>
+      </x:c>
+      <x:c r="F3" t="str">
+        <x:v>profile-tiktok</x:v>
+      </x:c>
+      <x:c r="G3" t="str"/>
+      <x:c r="H3" t="str"/>
+      <x:c r="I3" t="str"/>
+      <x:c r="J3" t="str">
+        <x:v>設定 TikTok 個人頁入口</x:v>
+      </x:c>
+      <x:c r="K3" t="str"/>
+      <x:c r="L3" t="str"/>
+      <x:c r="M3" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=tiktok&amp;utm_medium=social_profile&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=tiktok_bio</x:v>
+      </x:c>
+      <x:c r="N3" t="str">
+        <x:v>把 Bio/Profile link 設為 Profile website link，並放上置頂留言。</x:v>
+      </x:c>
+      <x:c r="O3" t="str">
+        <x:v>status=set/live, profile_link_set_date, profile_clicks, site_clicks, quiz_starts, quiz_completions</x:v>
+      </x:c>
+      <x:c r="P3" t="str"/>
+      <x:c r="Q3" t="str">
+        <x:v>入口只導向 15 題測驗，不導購、不承諾療效。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>profile_setup</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>instagram_reels</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>profile-instagram_reels</x:v>
+      </x:c>
+      <x:c r="G4" t="str"/>
+      <x:c r="H4" t="str"/>
+      <x:c r="I4" t="str"/>
+      <x:c r="J4" t="str">
+        <x:v>設定 Instagram Reels 個人頁入口</x:v>
+      </x:c>
+      <x:c r="K4" t="str"/>
+      <x:c r="L4" t="str"/>
+      <x:c r="M4" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=instagram&amp;utm_medium=social_profile&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=instagram_reels_bio</x:v>
+      </x:c>
+      <x:c r="N4" t="str">
+        <x:v>把 Bio/Profile link 設為 Profile link in bio，並放上置頂留言。</x:v>
+      </x:c>
+      <x:c r="O4" t="str">
+        <x:v>status=set/live, profile_link_set_date, profile_clicks, site_clicks, quiz_starts, quiz_completions</x:v>
+      </x:c>
+      <x:c r="P4" t="str"/>
+      <x:c r="Q4" t="str">
+        <x:v>入口只導向 15 題測驗，不導購、不承諾療效。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>asset_ready_check</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>all</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>publish-lt-s01-iris-silence</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
+        <x:v>lt-s01-iris-silence</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="I5" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="J5" t="str">
+        <x:v>他沉默時，你最想聽見哪一句話？</x:v>
+      </x:c>
+      <x:c r="K5" t="str"/>
+      <x:c r="L5" t="str"/>
+      <x:c r="M5" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_silence</x:v>
+      </x:c>
+      <x:c r="N5" t="str">
+        <x:v>確認直式影片、字幕、封面或首幀、caption、留言 CTA 與安全邊界都可發布。</x:v>
+      </x:c>
+      <x:c r="O5" t="str">
+        <x:v>mark asset ready before platform posting</x:v>
+      </x:c>
+      <x:c r="P5" t="str"/>
+      <x:c r="Q5" t="str">
+        <x:v>短片 CTA 維持測驗入口，不把素材改成直接購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>asset_ready_check</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>all</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>publish-lt-s02-iris-affirmation</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>lt-s02-iris-affirmation</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="I6" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="J6" t="str">
+        <x:v>哪一句肯定，會讓你瞬間安心？</x:v>
+      </x:c>
+      <x:c r="K6" t="str"/>
+      <x:c r="L6" t="str"/>
+      <x:c r="M6" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_affirmation</x:v>
+      </x:c>
+      <x:c r="N6" t="str">
+        <x:v>確認直式影片、字幕、封面或首幀、caption、留言 CTA 與安全邊界都可發布。</x:v>
+      </x:c>
+      <x:c r="O6" t="str">
+        <x:v>mark asset ready before platform posting</x:v>
+      </x:c>
+      <x:c r="P6" t="str"/>
+      <x:c r="Q6" t="str">
+        <x:v>短片 CTA 維持測驗入口，不把素材改成直接購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>asset_ready_check</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>ready</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>all</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>publish-lt-s03-iris-too-sensitive</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>lt-s03-iris-too-sensitive</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="I7" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="J7" t="str">
+        <x:v>你真的太敏感嗎？還是你只是等一句清楚的話？</x:v>
+      </x:c>
+      <x:c r="K7" t="str"/>
+      <x:c r="L7" t="str"/>
+      <x:c r="M7" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_too_sensitive</x:v>
+      </x:c>
+      <x:c r="N7" t="str">
+        <x:v>確認直式影片、字幕、封面或首幀、caption、留言 CTA 與安全邊界都可發布。</x:v>
+      </x:c>
+      <x:c r="O7" t="str">
+        <x:v>mark asset ready before platform posting</x:v>
+      </x:c>
+      <x:c r="P7" t="str"/>
+      <x:c r="Q7" t="str">
+        <x:v>短片 CTA 維持測驗入口，不把素材改成直接購買。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>publish_post</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>blocked_until_ready</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>youtube_shorts</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>publish-lt-s01-iris-silence</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>lt-s01-iris-silence</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="I8" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="J8" t="str">
+        <x:v>他沉默時，你最想聽見哪一句話？</x:v>
+      </x:c>
+      <x:c r="K8" t="str">
+        <x:v>2026-06-15</x:v>
+      </x:c>
+      <x:c r="L8" t="str">
+        <x:v>20:30</x:v>
+      </x:c>
+      <x:c r="M8" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_silence</x:v>
+      </x:c>
+      <x:c r="N8" t="str">
+        <x:v>依 YouTube Shorts caption 發布，確認連結與 UTM 未被改寫。</x:v>
+      </x:c>
+      <x:c r="O8" t="str">
+        <x:v>posting-queue.csv: status=published, published_date, post_url</x:v>
+      </x:c>
+      <x:c r="P8" t="str">
+        <x:v>profile_setup, asset_ready_check</x:v>
+      </x:c>
+      <x:c r="Q8" t="str">
+        <x:v>只使用單一 CTA：完成 15 題測驗，找到你的情感守護者。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>kpi_backfill</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>blocked_until_published</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>youtube_shorts</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>publish-lt-s01-iris-silence</x:v>
+      </x:c>
+      <x:c r="G9" t="str">
+        <x:v>lt-s01-iris-silence</x:v>
+      </x:c>
+      <x:c r="H9" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="I9" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="J9" t="str">
+        <x:v>他沉默時，你最想聽見哪一句話？</x:v>
+      </x:c>
+      <x:c r="K9" t="str">
+        <x:v>2026-06-15</x:v>
+      </x:c>
+      <x:c r="L9" t="str">
+        <x:v>20:30</x:v>
+      </x:c>
+      <x:c r="M9" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_silence</x:v>
+      </x:c>
+      <x:c r="N9" t="str">
+        <x:v>發布後回填貼文 URL 與最小 KPI：site_clicks、quiz_starts、quiz_completions。</x:v>
+      </x:c>
+      <x:c r="O9" t="str">
+        <x:v>kpi-tracker.csv: platform, post_url, site_clicks, quiz_starts, quiz_completions</x:v>
+      </x:c>
+      <x:c r="P9" t="str">
+        <x:v>post_url</x:v>
+      </x:c>
+      <x:c r="Q9" t="str">
+        <x:v>只使用單一 CTA：完成 15 題測驗，找到你的情感守護者。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>publish_post</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>blocked_until_ready</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>tiktok</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>publish-lt-s01-iris-silence</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>lt-s01-iris-silence</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="I10" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="J10" t="str">
+        <x:v>他沉默時，你最想聽見哪一句話？</x:v>
+      </x:c>
+      <x:c r="K10" t="str">
+        <x:v>2026-06-15</x:v>
+      </x:c>
+      <x:c r="L10" t="str">
+        <x:v>21:00</x:v>
+      </x:c>
+      <x:c r="M10" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_silence</x:v>
+      </x:c>
+      <x:c r="N10" t="str">
+        <x:v>依 TikTok caption 發布，確認連結與 UTM 未被改寫。</x:v>
+      </x:c>
+      <x:c r="O10" t="str">
+        <x:v>posting-queue.csv: status=published, published_date, post_url</x:v>
+      </x:c>
+      <x:c r="P10" t="str">
+        <x:v>profile_setup, asset_ready_check</x:v>
+      </x:c>
+      <x:c r="Q10" t="str">
+        <x:v>只使用單一 CTA：完成 15 題測驗，找到你的情感守護者。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>kpi_backfill</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>blocked_until_published</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>tiktok</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>publish-lt-s01-iris-silence</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>lt-s01-iris-silence</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="I11" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="J11" t="str">
+        <x:v>他沉默時，你最想聽見哪一句話？</x:v>
+      </x:c>
+      <x:c r="K11" t="str">
+        <x:v>2026-06-15</x:v>
+      </x:c>
+      <x:c r="L11" t="str">
+        <x:v>21:00</x:v>
+      </x:c>
+      <x:c r="M11" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_silence</x:v>
+      </x:c>
+      <x:c r="N11" t="str">
+        <x:v>發布後回填貼文 URL 與最小 KPI：site_clicks、quiz_starts、quiz_completions。</x:v>
+      </x:c>
+      <x:c r="O11" t="str">
+        <x:v>kpi-tracker.csv: platform, post_url, site_clicks, quiz_starts, quiz_completions</x:v>
+      </x:c>
+      <x:c r="P11" t="str">
+        <x:v>post_url</x:v>
+      </x:c>
+      <x:c r="Q11" t="str">
+        <x:v>只使用單一 CTA：完成 15 題測驗，找到你的情感守護者。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>publish_post</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>blocked_until_ready</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>instagram_reels</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>publish-lt-s01-iris-silence</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>lt-s01-iris-silence</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="I12" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="J12" t="str">
+        <x:v>他沉默時，你最想聽見哪一句話？</x:v>
+      </x:c>
+      <x:c r="K12" t="str">
+        <x:v>2026-06-15</x:v>
+      </x:c>
+      <x:c r="L12" t="str">
+        <x:v>21:30</x:v>
+      </x:c>
+      <x:c r="M12" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_silence</x:v>
+      </x:c>
+      <x:c r="N12" t="str">
+        <x:v>依 Instagram Reels caption 發布，確認連結與 UTM 未被改寫。</x:v>
+      </x:c>
+      <x:c r="O12" t="str">
+        <x:v>posting-queue.csv: status=published, published_date, post_url</x:v>
+      </x:c>
+      <x:c r="P12" t="str">
+        <x:v>profile_setup, asset_ready_check</x:v>
+      </x:c>
+      <x:c r="Q12" t="str">
+        <x:v>只使用單一 CTA：完成 15 題測驗，找到你的情感守護者。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>kpi_backfill</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>blocked_until_published</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>instagram_reels</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>publish-lt-s01-iris-silence</x:v>
+      </x:c>
+      <x:c r="G13" t="str">
+        <x:v>lt-s01-iris-silence</x:v>
+      </x:c>
+      <x:c r="H13" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="I13" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="J13" t="str">
+        <x:v>他沉默時，你最想聽見哪一句話？</x:v>
+      </x:c>
+      <x:c r="K13" t="str">
+        <x:v>2026-06-15</x:v>
+      </x:c>
+      <x:c r="L13" t="str">
+        <x:v>21:30</x:v>
+      </x:c>
+      <x:c r="M13" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_silence</x:v>
+      </x:c>
+      <x:c r="N13" t="str">
+        <x:v>發布後回填貼文 URL 與最小 KPI：site_clicks、quiz_starts、quiz_completions。</x:v>
+      </x:c>
+      <x:c r="O13" t="str">
+        <x:v>kpi-tracker.csv: platform, post_url, site_clicks, quiz_starts, quiz_completions</x:v>
+      </x:c>
+      <x:c r="P13" t="str">
+        <x:v>post_url</x:v>
+      </x:c>
+      <x:c r="Q13" t="str">
+        <x:v>只使用單一 CTA：完成 15 題測驗，找到你的情感守護者。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>publish_post</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>blocked_until_ready</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>youtube_shorts</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>publish-lt-s02-iris-affirmation</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>lt-s02-iris-affirmation</x:v>
+      </x:c>
+      <x:c r="H14" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="I14" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="J14" t="str">
+        <x:v>哪一句肯定，會讓你瞬間安心？</x:v>
+      </x:c>
+      <x:c r="K14" t="str">
+        <x:v>2026-06-17</x:v>
+      </x:c>
+      <x:c r="L14" t="str">
+        <x:v>20:30</x:v>
+      </x:c>
+      <x:c r="M14" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_affirmation</x:v>
+      </x:c>
+      <x:c r="N14" t="str">
+        <x:v>依 YouTube Shorts caption 發布，確認連結與 UTM 未被改寫。</x:v>
+      </x:c>
+      <x:c r="O14" t="str">
+        <x:v>posting-queue.csv: status=published, published_date, post_url</x:v>
+      </x:c>
+      <x:c r="P14" t="str">
+        <x:v>profile_setup, asset_ready_check</x:v>
+      </x:c>
+      <x:c r="Q14" t="str">
+        <x:v>只使用單一 CTA：完成 15 題測驗，找到你的情感守護者。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>kpi_backfill</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>blocked_until_published</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>youtube_shorts</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
+        <x:v>publish-lt-s02-iris-affirmation</x:v>
+      </x:c>
+      <x:c r="G15" t="str">
+        <x:v>lt-s02-iris-affirmation</x:v>
+      </x:c>
+      <x:c r="H15" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="I15" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="J15" t="str">
+        <x:v>哪一句肯定，會讓你瞬間安心？</x:v>
+      </x:c>
+      <x:c r="K15" t="str">
+        <x:v>2026-06-17</x:v>
+      </x:c>
+      <x:c r="L15" t="str">
+        <x:v>20:30</x:v>
+      </x:c>
+      <x:c r="M15" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_affirmation</x:v>
+      </x:c>
+      <x:c r="N15" t="str">
+        <x:v>發布後回填貼文 URL 與最小 KPI：site_clicks、quiz_starts、quiz_completions。</x:v>
+      </x:c>
+      <x:c r="O15" t="str">
+        <x:v>kpi-tracker.csv: platform, post_url, site_clicks, quiz_starts, quiz_completions</x:v>
+      </x:c>
+      <x:c r="P15" t="str">
+        <x:v>post_url</x:v>
+      </x:c>
+      <x:c r="Q15" t="str">
+        <x:v>只使用單一 CTA：完成 15 題測驗，找到你的情感守護者。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>publish_post</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>blocked_until_ready</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="E16" t="str">
+        <x:v>tiktok</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
+        <x:v>publish-lt-s02-iris-affirmation</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>lt-s02-iris-affirmation</x:v>
+      </x:c>
+      <x:c r="H16" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="I16" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="J16" t="str">
+        <x:v>哪一句肯定，會讓你瞬間安心？</x:v>
+      </x:c>
+      <x:c r="K16" t="str">
+        <x:v>2026-06-17</x:v>
+      </x:c>
+      <x:c r="L16" t="str">
+        <x:v>21:00</x:v>
+      </x:c>
+      <x:c r="M16" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_affirmation</x:v>
+      </x:c>
+      <x:c r="N16" t="str">
+        <x:v>依 TikTok caption 發布，確認連結與 UTM 未被改寫。</x:v>
+      </x:c>
+      <x:c r="O16" t="str">
+        <x:v>posting-queue.csv: status=published, published_date, post_url</x:v>
+      </x:c>
+      <x:c r="P16" t="str">
+        <x:v>profile_setup, asset_ready_check</x:v>
+      </x:c>
+      <x:c r="Q16" t="str">
+        <x:v>只使用單一 CTA：完成 15 題測驗，找到你的情感守護者。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>kpi_backfill</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>blocked_until_published</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="E17" t="str">
+        <x:v>tiktok</x:v>
+      </x:c>
+      <x:c r="F17" t="str">
+        <x:v>publish-lt-s02-iris-affirmation</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>lt-s02-iris-affirmation</x:v>
+      </x:c>
+      <x:c r="H17" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="I17" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="J17" t="str">
+        <x:v>哪一句肯定，會讓你瞬間安心？</x:v>
+      </x:c>
+      <x:c r="K17" t="str">
+        <x:v>2026-06-17</x:v>
+      </x:c>
+      <x:c r="L17" t="str">
+        <x:v>21:00</x:v>
+      </x:c>
+      <x:c r="M17" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_affirmation</x:v>
+      </x:c>
+      <x:c r="N17" t="str">
+        <x:v>發布後回填貼文 URL 與最小 KPI：site_clicks、quiz_starts、quiz_completions。</x:v>
+      </x:c>
+      <x:c r="O17" t="str">
+        <x:v>kpi-tracker.csv: platform, post_url, site_clicks, quiz_starts, quiz_completions</x:v>
+      </x:c>
+      <x:c r="P17" t="str">
+        <x:v>post_url</x:v>
+      </x:c>
+      <x:c r="Q17" t="str">
+        <x:v>只使用單一 CTA：完成 15 題測驗，找到你的情感守護者。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>publish_post</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>blocked_until_ready</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="E18" t="str">
+        <x:v>instagram_reels</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>publish-lt-s02-iris-affirmation</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>lt-s02-iris-affirmation</x:v>
+      </x:c>
+      <x:c r="H18" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="I18" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="J18" t="str">
+        <x:v>哪一句肯定，會讓你瞬間安心？</x:v>
+      </x:c>
+      <x:c r="K18" t="str">
+        <x:v>2026-06-17</x:v>
+      </x:c>
+      <x:c r="L18" t="str">
+        <x:v>21:30</x:v>
+      </x:c>
+      <x:c r="M18" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_affirmation</x:v>
+      </x:c>
+      <x:c r="N18" t="str">
+        <x:v>依 Instagram Reels caption 發布，確認連結與 UTM 未被改寫。</x:v>
+      </x:c>
+      <x:c r="O18" t="str">
+        <x:v>posting-queue.csv: status=published, published_date, post_url</x:v>
+      </x:c>
+      <x:c r="P18" t="str">
+        <x:v>profile_setup, asset_ready_check</x:v>
+      </x:c>
+      <x:c r="Q18" t="str">
+        <x:v>只使用單一 CTA：完成 15 題測驗，找到你的情感守護者。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>kpi_backfill</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>blocked_until_published</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="E19" t="str">
+        <x:v>instagram_reels</x:v>
+      </x:c>
+      <x:c r="F19" t="str">
+        <x:v>publish-lt-s02-iris-affirmation</x:v>
+      </x:c>
+      <x:c r="G19" t="str">
+        <x:v>lt-s02-iris-affirmation</x:v>
+      </x:c>
+      <x:c r="H19" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="I19" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="J19" t="str">
+        <x:v>哪一句肯定，會讓你瞬間安心？</x:v>
+      </x:c>
+      <x:c r="K19" t="str">
+        <x:v>2026-06-17</x:v>
+      </x:c>
+      <x:c r="L19" t="str">
+        <x:v>21:30</x:v>
+      </x:c>
+      <x:c r="M19" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_affirmation</x:v>
+      </x:c>
+      <x:c r="N19" t="str">
+        <x:v>發布後回填貼文 URL 與最小 KPI：site_clicks、quiz_starts、quiz_completions。</x:v>
+      </x:c>
+      <x:c r="O19" t="str">
+        <x:v>kpi-tracker.csv: platform, post_url, site_clicks, quiz_starts, quiz_completions</x:v>
+      </x:c>
+      <x:c r="P19" t="str">
+        <x:v>post_url</x:v>
+      </x:c>
+      <x:c r="Q19" t="str">
+        <x:v>只使用單一 CTA：完成 15 題測驗，找到你的情感守護者。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>publish_post</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>blocked_until_ready</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="E20" t="str">
+        <x:v>youtube_shorts</x:v>
+      </x:c>
+      <x:c r="F20" t="str">
+        <x:v>publish-lt-s03-iris-too-sensitive</x:v>
+      </x:c>
+      <x:c r="G20" t="str">
+        <x:v>lt-s03-iris-too-sensitive</x:v>
+      </x:c>
+      <x:c r="H20" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="I20" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="J20" t="str">
+        <x:v>你真的太敏感嗎？還是你只是等一句清楚的話？</x:v>
+      </x:c>
+      <x:c r="K20" t="str">
+        <x:v>2026-06-19</x:v>
+      </x:c>
+      <x:c r="L20" t="str">
+        <x:v>20:30</x:v>
+      </x:c>
+      <x:c r="M20" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_too_sensitive</x:v>
+      </x:c>
+      <x:c r="N20" t="str">
+        <x:v>依 YouTube Shorts caption 發布，確認連結與 UTM 未被改寫。</x:v>
+      </x:c>
+      <x:c r="O20" t="str">
+        <x:v>posting-queue.csv: status=published, published_date, post_url</x:v>
+      </x:c>
+      <x:c r="P20" t="str">
+        <x:v>profile_setup, asset_ready_check</x:v>
+      </x:c>
+      <x:c r="Q20" t="str">
+        <x:v>只使用單一 CTA：完成 15 題測驗，找到你的情感守護者。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>kpi_backfill</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>blocked_until_published</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="E21" t="str">
+        <x:v>youtube_shorts</x:v>
+      </x:c>
+      <x:c r="F21" t="str">
+        <x:v>publish-lt-s03-iris-too-sensitive</x:v>
+      </x:c>
+      <x:c r="G21" t="str">
+        <x:v>lt-s03-iris-too-sensitive</x:v>
+      </x:c>
+      <x:c r="H21" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="I21" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="J21" t="str">
+        <x:v>你真的太敏感嗎？還是你只是等一句清楚的話？</x:v>
+      </x:c>
+      <x:c r="K21" t="str">
+        <x:v>2026-06-19</x:v>
+      </x:c>
+      <x:c r="L21" t="str">
+        <x:v>20:30</x:v>
+      </x:c>
+      <x:c r="M21" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_too_sensitive</x:v>
+      </x:c>
+      <x:c r="N21" t="str">
+        <x:v>發布後回填貼文 URL 與最小 KPI：site_clicks、quiz_starts、quiz_completions。</x:v>
+      </x:c>
+      <x:c r="O21" t="str">
+        <x:v>kpi-tracker.csv: platform, post_url, site_clicks, quiz_starts, quiz_completions</x:v>
+      </x:c>
+      <x:c r="P21" t="str">
+        <x:v>post_url</x:v>
+      </x:c>
+      <x:c r="Q21" t="str">
+        <x:v>只使用單一 CTA：完成 15 題測驗，找到你的情感守護者。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>publish_post</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>blocked_until_ready</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="E22" t="str">
+        <x:v>tiktok</x:v>
+      </x:c>
+      <x:c r="F22" t="str">
+        <x:v>publish-lt-s03-iris-too-sensitive</x:v>
+      </x:c>
+      <x:c r="G22" t="str">
+        <x:v>lt-s03-iris-too-sensitive</x:v>
+      </x:c>
+      <x:c r="H22" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="I22" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="J22" t="str">
+        <x:v>你真的太敏感嗎？還是你只是等一句清楚的話？</x:v>
+      </x:c>
+      <x:c r="K22" t="str">
+        <x:v>2026-06-19</x:v>
+      </x:c>
+      <x:c r="L22" t="str">
+        <x:v>21:00</x:v>
+      </x:c>
+      <x:c r="M22" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_too_sensitive</x:v>
+      </x:c>
+      <x:c r="N22" t="str">
+        <x:v>依 TikTok caption 發布，確認連結與 UTM 未被改寫。</x:v>
+      </x:c>
+      <x:c r="O22" t="str">
+        <x:v>posting-queue.csv: status=published, published_date, post_url</x:v>
+      </x:c>
+      <x:c r="P22" t="str">
+        <x:v>profile_setup, asset_ready_check</x:v>
+      </x:c>
+      <x:c r="Q22" t="str">
+        <x:v>只使用單一 CTA：完成 15 題測驗，找到你的情感守護者。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>kpi_backfill</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>blocked_until_published</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="E23" t="str">
+        <x:v>tiktok</x:v>
+      </x:c>
+      <x:c r="F23" t="str">
+        <x:v>publish-lt-s03-iris-too-sensitive</x:v>
+      </x:c>
+      <x:c r="G23" t="str">
+        <x:v>lt-s03-iris-too-sensitive</x:v>
+      </x:c>
+      <x:c r="H23" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="I23" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="J23" t="str">
+        <x:v>你真的太敏感嗎？還是你只是等一句清楚的話？</x:v>
+      </x:c>
+      <x:c r="K23" t="str">
+        <x:v>2026-06-19</x:v>
+      </x:c>
+      <x:c r="L23" t="str">
+        <x:v>21:00</x:v>
+      </x:c>
+      <x:c r="M23" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_too_sensitive</x:v>
+      </x:c>
+      <x:c r="N23" t="str">
+        <x:v>發布後回填貼文 URL 與最小 KPI：site_clicks、quiz_starts、quiz_completions。</x:v>
+      </x:c>
+      <x:c r="O23" t="str">
+        <x:v>kpi-tracker.csv: platform, post_url, site_clicks, quiz_starts, quiz_completions</x:v>
+      </x:c>
+      <x:c r="P23" t="str">
+        <x:v>post_url</x:v>
+      </x:c>
+      <x:c r="Q23" t="str">
+        <x:v>只使用單一 CTA：完成 15 題測驗，找到你的情感守護者。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>publish_post</x:v>
+      </x:c>
+      <x:c r="C24" t="str">
+        <x:v>blocked_until_ready</x:v>
+      </x:c>
+      <x:c r="D24" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="E24" t="str">
+        <x:v>instagram_reels</x:v>
+      </x:c>
+      <x:c r="F24" t="str">
+        <x:v>publish-lt-s03-iris-too-sensitive</x:v>
+      </x:c>
+      <x:c r="G24" t="str">
+        <x:v>lt-s03-iris-too-sensitive</x:v>
+      </x:c>
+      <x:c r="H24" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="I24" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="J24" t="str">
+        <x:v>你真的太敏感嗎？還是你只是等一句清楚的話？</x:v>
+      </x:c>
+      <x:c r="K24" t="str">
+        <x:v>2026-06-19</x:v>
+      </x:c>
+      <x:c r="L24" t="str">
+        <x:v>21:30</x:v>
+      </x:c>
+      <x:c r="M24" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_too_sensitive</x:v>
+      </x:c>
+      <x:c r="N24" t="str">
+        <x:v>依 Instagram Reels caption 發布，確認連結與 UTM 未被改寫。</x:v>
+      </x:c>
+      <x:c r="O24" t="str">
+        <x:v>posting-queue.csv: status=published, published_date, post_url</x:v>
+      </x:c>
+      <x:c r="P24" t="str">
+        <x:v>profile_setup, asset_ready_check</x:v>
+      </x:c>
+      <x:c r="Q24" t="str">
+        <x:v>只使用單一 CTA：完成 15 題測驗，找到你的情感守護者。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="str">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>kpi_backfill</x:v>
+      </x:c>
+      <x:c r="C25" t="str">
+        <x:v>blocked_until_published</x:v>
+      </x:c>
+      <x:c r="D25" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="E25" t="str">
+        <x:v>instagram_reels</x:v>
+      </x:c>
+      <x:c r="F25" t="str">
+        <x:v>publish-lt-s03-iris-too-sensitive</x:v>
+      </x:c>
+      <x:c r="G25" t="str">
+        <x:v>lt-s03-iris-too-sensitive</x:v>
+      </x:c>
+      <x:c r="H25" t="str">
+        <x:v>iris</x:v>
+      </x:c>
+      <x:c r="I25" t="str">
+        <x:v>艾莉絲</x:v>
+      </x:c>
+      <x:c r="J25" t="str">
+        <x:v>你真的太敏感嗎？還是你只是等一句清楚的話？</x:v>
+      </x:c>
+      <x:c r="K25" t="str">
+        <x:v>2026-06-19</x:v>
+      </x:c>
+      <x:c r="L25" t="str">
+        <x:v>21:30</x:v>
+      </x:c>
+      <x:c r="M25" t="str">
+        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_too_sensitive</x:v>
+      </x:c>
+      <x:c r="N25" t="str">
+        <x:v>發布後回填貼文 URL 與最小 KPI：site_clicks、quiz_starts、quiz_completions。</x:v>
+      </x:c>
+      <x:c r="O25" t="str">
+        <x:v>kpi-tracker.csv: platform, post_url, site_clicks, quiz_starts, quiz_completions</x:v>
+      </x:c>
+      <x:c r="P25" t="str">
+        <x:v>post_url</x:v>
+      </x:c>
+      <x:c r="Q25" t="str">
+        <x:v>只使用單一 CTA：完成 15 題測驗，找到你的情感守護者。</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
         <x:v>Week 1 Profile Gates</x:v>
       </x:c>
       <x:c r="B1" t="str"/>
@@ -8069,177 +9539,4 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" t="str">
-        <x:v>taskId</x:v>
-      </x:c>
-      <x:c r="B1" t="str">
-        <x:v>week</x:v>
-      </x:c>
-      <x:c r="C1" t="str">
-        <x:v>slot</x:v>
-      </x:c>
-      <x:c r="D1" t="str">
-        <x:v>guardianId</x:v>
-      </x:c>
-      <x:c r="E1" t="str">
-        <x:v>guardianName</x:v>
-      </x:c>
-      <x:c r="F1" t="str">
-        <x:v>contentAngle</x:v>
-      </x:c>
-      <x:c r="G1" t="str">
-        <x:v>title</x:v>
-      </x:c>
-      <x:c r="H1" t="str">
-        <x:v>trackedUrl</x:v>
-      </x:c>
-      <x:c r="I1" t="str">
-        <x:v>primaryFreeItemId</x:v>
-      </x:c>
-      <x:c r="J1" t="str">
-        <x:v>ownedLeadItemId</x:v>
-      </x:c>
-      <x:c r="K1" t="str">
-        <x:v>supplyRoute</x:v>
-      </x:c>
-      <x:c r="L1" t="str">
-        <x:v>lunaScene</x:v>
-      </x:c>
-      <x:c r="M1" t="str">
-        <x:v>keepsake</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" t="str">
-        <x:v>publish-lt-s01-iris-silence</x:v>
-      </x:c>
-      <x:c r="B2" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C2" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D2" t="str">
-        <x:v>iris</x:v>
-      </x:c>
-      <x:c r="E2" t="str">
-        <x:v>艾莉絲</x:v>
-      </x:c>
-      <x:c r="F2" t="str">
-        <x:v>情感錯頻情境</x:v>
-      </x:c>
-      <x:c r="G2" t="str">
-        <x:v>他沉默時，你最想聽見哪一句話？</x:v>
-      </x:c>
-      <x:c r="H2" t="str">
-        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_silence</x:v>
-      </x:c>
-      <x:c r="I2" t="str">
-        <x:v>free-keepsake-iris</x:v>
-      </x:c>
-      <x:c r="J2" t="str">
-        <x:v>supply-wishlist-iris</x:v>
-      </x:c>
-      <x:c r="K2" t="str">
-        <x:v>https://lovetypes.tw/resources/#supply-iris</x:v>
-      </x:c>
-      <x:c r="L2" t="str">
-        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-iris</x:v>
-      </x:c>
-      <x:c r="M2" t="str">
-        <x:v>https://lovetypes.tw/keepsakes/#keepsake-iris</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" t="str">
-        <x:v>publish-lt-s02-iris-affirmation</x:v>
-      </x:c>
-      <x:c r="B3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C3" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D3" t="str">
-        <x:v>iris</x:v>
-      </x:c>
-      <x:c r="E3" t="str">
-        <x:v>艾莉絲</x:v>
-      </x:c>
-      <x:c r="F3" t="str">
-        <x:v>守護者人格認同</x:v>
-      </x:c>
-      <x:c r="G3" t="str">
-        <x:v>哪一句肯定，會讓你瞬間安心？</x:v>
-      </x:c>
-      <x:c r="H3" t="str">
-        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_affirmation</x:v>
-      </x:c>
-      <x:c r="I3" t="str">
-        <x:v>free-keepsake-iris</x:v>
-      </x:c>
-      <x:c r="J3" t="str">
-        <x:v>supply-wishlist-iris</x:v>
-      </x:c>
-      <x:c r="K3" t="str">
-        <x:v>https://lovetypes.tw/resources/#supply-iris</x:v>
-      </x:c>
-      <x:c r="L3" t="str">
-        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-iris</x:v>
-      </x:c>
-      <x:c r="M3" t="str">
-        <x:v>https://lovetypes.tw/keepsakes/#keepsake-iris</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" t="str">
-        <x:v>publish-lt-s03-iris-too-sensitive</x:v>
-      </x:c>
-      <x:c r="B4" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C4" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D4" t="str">
-        <x:v>iris</x:v>
-      </x:c>
-      <x:c r="E4" t="str">
-        <x:v>艾莉絲</x:v>
-      </x:c>
-      <x:c r="F4" t="str">
-        <x:v>測驗入口</x:v>
-      </x:c>
-      <x:c r="G4" t="str">
-        <x:v>你真的太敏感嗎？還是你只是等一句清楚的話？</x:v>
-      </x:c>
-      <x:c r="H4" t="str">
-        <x:v>https://lovetypes.tw/start/?utm_source=shorts&amp;utm_medium=social&amp;utm_campaign=first_round_quiz_completion&amp;utm_content=iris_too_sensitive</x:v>
-      </x:c>
-      <x:c r="I4" t="str">
-        <x:v>free-keepsake-iris</x:v>
-      </x:c>
-      <x:c r="J4" t="str">
-        <x:v>supply-wishlist-iris</x:v>
-      </x:c>
-      <x:c r="K4" t="str">
-        <x:v>https://lovetypes.tw/resources/#supply-iris</x:v>
-      </x:c>
-      <x:c r="L4" t="str">
-        <x:v>https://lovetypes.tw/luna-yoga-music/#luna-iris</x:v>
-      </x:c>
-      <x:c r="M4" t="str">
-        <x:v>https://lovetypes.tw/keepsakes/#keepsake-iris</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add weekly promotion asset briefs
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R75b9cfccbcf84696"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R2c76153eee054350"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R12d2bd2376574a9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R5c861a12aac44df7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="R7d5de031636c44d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="R7b3b549dac914ec4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="R9c3e424ac65540bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="Ra2a9aee467334bf7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="Ra6ae868120ef4219"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="R1017824211a4425c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="R7f594d6e68b74b49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Ra28f90f5be394c09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rb0cf442b4eb44f2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R52cdf6abf47142ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="Ref793ca834ce4ac7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="R0d197455fd754be8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="R702f93fed73642cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="Rb6504c539f784e11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="R085ab1dc53dd4fc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="Rdb11fcb8be4949da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="R3f0a3866997a42df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="Read63e8ad2e14394"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Add promotion launch link QA
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Ra28f90f5be394c09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rb0cf442b4eb44f2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R52cdf6abf47142ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="Ref793ca834ce4ac7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="R0d197455fd754be8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="R702f93fed73642cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="Rb6504c539f784e11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="R085ab1dc53dd4fc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="Rdb11fcb8be4949da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="R3f0a3866997a42df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="Read63e8ad2e14394"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R712526274c274ece"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R23fee7f6bbc14b79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R543acd7b8e4f484f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="Rc1d86b3b4ddb4fa5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="Ra206e7636acd4509"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="R101ca69e7b1342a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="R1f87bfce9e414a17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="R0fdebe37109d447d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="R60b9ff95f0264eb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="R57a279aa80304496"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="R78917d16794849e4"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Preserve quiz campaign attribution
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R712526274c274ece"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R23fee7f6bbc14b79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R543acd7b8e4f484f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="Rc1d86b3b4ddb4fa5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="Ra206e7636acd4509"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="R101ca69e7b1342a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="R1f87bfce9e414a17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="R0fdebe37109d447d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="R60b9ff95f0264eb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="R57a279aa80304496"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="R78917d16794849e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R15bd2bdaa3b84e1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rfff8ff1174c6420e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R5ca5500d5d104881"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R30dc3157d5914270"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="R591252f783134dca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="Rc7da25f5326d4d44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="Ra95620e0bad14ad6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="Rdbebd2b81e7d4a77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="R4e54c72bf1f8418c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="Refb22c9809124920"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="R0d9383da1f2046bc"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Add promotion attribution reconciliation
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R15bd2bdaa3b84e1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rfff8ff1174c6420e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R5ca5500d5d104881"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R30dc3157d5914270"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="R591252f783134dca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="Rc7da25f5326d4d44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="Ra95620e0bad14ad6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="Rdbebd2b81e7d4a77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="R4e54c72bf1f8418c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="Refb22c9809124920"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="R0d9383da1f2046bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R23b9945fe5e7478a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rc28bee63035f4785"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R85b3f90910054f39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R5dee2d76405046ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="R714fc4534073440e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="Rbc8fe139f0af489e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="Ra788870c50d34bd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="Rd689b0e2aafe4f24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="R723d06d1e2624c55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="R2b7ee18031c44b29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="Rd37b3140738c4370"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Add lead intake KPI writeback mapping
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R23b9945fe5e7478a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rc28bee63035f4785"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R85b3f90910054f39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R5dee2d76405046ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="R714fc4534073440e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="Rbc8fe139f0af489e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="Ra788870c50d34bd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="Rd689b0e2aafe4f24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="R723d06d1e2624c55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="R2b7ee18031c44b29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="Rd37b3140738c4370"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R0818d3cfe95946f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R58f7716cef0a41bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="Reacd67030471492d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R3878b2e4ffe04bac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="R7bf7fe22284d4266"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="Rc6b2cc306a884edc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="R5a92f9328ef646bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="Rd62e6dc311634f2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="Rfbcbd0d3647e47b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="R3e72e1aae68f4603"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="R74bb4ac307d64860"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1873,45 +1873,57 @@
         <x:v>source</x:v>
       </x:c>
       <x:c r="D1" t="str">
+        <x:v>utm_content</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
+        <x:v>contact_campaign_content</x:v>
+      </x:c>
+      <x:c r="F1" t="str">
         <x:v>guardian_id</x:v>
       </x:c>
-      <x:c r="E1" t="str">
+      <x:c r="G1" t="str">
         <x:v>guardian_name</x:v>
       </x:c>
-      <x:c r="F1" t="str">
+      <x:c r="H1" t="str">
         <x:v>intake_type</x:v>
       </x:c>
-      <x:c r="G1" t="str">
+      <x:c r="I1" t="str">
         <x:v>requested_asset</x:v>
       </x:c>
-      <x:c r="H1" t="str">
+      <x:c r="J1" t="str">
         <x:v>related_route</x:v>
       </x:c>
-      <x:c r="I1" t="str">
+      <x:c r="K1" t="str">
+        <x:v>kpi_writeback_field</x:v>
+      </x:c>
+      <x:c r="L1" t="str">
+        <x:v>kpi_writeback_rule</x:v>
+      </x:c>
+      <x:c r="M1" t="str">
         <x:v>email_status</x:v>
       </x:c>
-      <x:c r="J1" t="str">
+      <x:c r="N1" t="str">
         <x:v>consent_status</x:v>
       </x:c>
-      <x:c r="K1" t="str">
+      <x:c r="O1" t="str">
         <x:v>priority</x:v>
       </x:c>
-      <x:c r="L1" t="str">
+      <x:c r="P1" t="str">
         <x:v>status</x:v>
       </x:c>
-      <x:c r="M1" t="str">
+      <x:c r="Q1" t="str">
         <x:v>first_response</x:v>
       </x:c>
-      <x:c r="N1" t="str">
+      <x:c r="R1" t="str">
         <x:v>next_action</x:v>
       </x:c>
-      <x:c r="O1" t="str">
+      <x:c r="S1" t="str">
         <x:v>follow_up_deadline</x:v>
       </x:c>
-      <x:c r="P1" t="str">
+      <x:c r="T1" t="str">
         <x:v>fulfillment_asset</x:v>
       </x:c>
-      <x:c r="Q1" t="str">
+      <x:c r="U1" t="str">
         <x:v>notes</x:v>
       </x:c>
     </x:row>
@@ -1923,42 +1935,52 @@
       <x:c r="C2" t="str">
         <x:v>contact_or_waitlist</x:v>
       </x:c>
-      <x:c r="D2" t="str">
+      <x:c r="D2" t="str"/>
+      <x:c r="E2" t="str">
+        <x:v>Copy from Contact email Campaign content / 推廣內容. Valid examples: iris_affirmation, iris_silence, iris_too_sensitive</x:v>
+      </x:c>
+      <x:c r="F2" t="str">
         <x:v>iris</x:v>
       </x:c>
-      <x:c r="E2" t="str">
+      <x:c r="G2" t="str">
         <x:v>艾莉絲</x:v>
       </x:c>
-      <x:c r="F2" t="str">
+      <x:c r="H2" t="str">
         <x:v>owned_asset_request</x:v>
       </x:c>
-      <x:c r="G2" t="str">
+      <x:c r="I2" t="str">
         <x:v>guardian PDF / wallpaper / short ritual</x:v>
       </x:c>
-      <x:c r="H2" t="str">
+      <x:c r="J2" t="str">
         <x:v>https://lovetypes.tw/keepsakes/#keepsake-iris</x:v>
       </x:c>
-      <x:c r="I2" t="str">
+      <x:c r="K2" t="str">
+        <x:v>supply_lead_requests</x:v>
+      </x:c>
+      <x:c r="L2" t="str">
+        <x:v>If utm_content matches attribution-reconciliation.csv, increment this field on the matching kpi-tracker.csv row; otherwise record as manual lead and do not choose a winning script.</x:v>
+      </x:c>
+      <x:c r="M2" t="str">
         <x:v>not_received</x:v>
       </x:c>
-      <x:c r="J2" t="str">
+      <x:c r="N2" t="str">
         <x:v>not_applicable_until_user_contacts</x:v>
       </x:c>
-      <x:c r="K2" t="str">
+      <x:c r="O2" t="str">
         <x:v>medium</x:v>
       </x:c>
-      <x:c r="L2" t="str">
+      <x:c r="P2" t="str">
         <x:v>template</x:v>
       </x:c>
-      <x:c r="M2" t="str">
+      <x:c r="Q2" t="str">
         <x:v>確認想收到的守護者素材，回覆預計製作方向與安全邊界。</x:v>
       </x:c>
-      <x:c r="N2" t="str">
+      <x:c r="R2" t="str">
         <x:v>累積同守護者重複需求後，排進 asset-build-backlog 的 build_owned_asset。</x:v>
       </x:c>
-      <x:c r="O2" t="str"/>
-      <x:c r="P2" t="str"/>
-      <x:c r="Q2" t="str">
+      <x:c r="S2" t="str"/>
+      <x:c r="T2" t="str"/>
+      <x:c r="U2" t="str">
         <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
       </x:c>
     </x:row>
@@ -1970,42 +1992,52 @@
       <x:c r="C3" t="str">
         <x:v>contact_or_waitlist</x:v>
       </x:c>
-      <x:c r="D3" t="str">
+      <x:c r="D3" t="str"/>
+      <x:c r="E3" t="str">
+        <x:v>Copy from Contact email Campaign content / 推廣內容. Valid examples: iris_affirmation, iris_silence, iris_too_sensitive</x:v>
+      </x:c>
+      <x:c r="F3" t="str">
         <x:v>iris</x:v>
       </x:c>
-      <x:c r="E3" t="str">
+      <x:c r="G3" t="str">
         <x:v>艾莉絲</x:v>
       </x:c>
-      <x:c r="F3" t="str">
+      <x:c r="H3" t="str">
         <x:v>luna_scene_request</x:v>
       </x:c>
-      <x:c r="G3" t="str">
+      <x:c r="I3" t="str">
         <x:v>Luna bedtime / conflict cooldown / quiz aftercare pack</x:v>
       </x:c>
-      <x:c r="H3" t="str">
+      <x:c r="J3" t="str">
         <x:v>https://lovetypes.tw/luna-yoga-music/#luna-iris</x:v>
       </x:c>
-      <x:c r="I3" t="str">
+      <x:c r="K3" t="str">
+        <x:v>luna_pack_clicks</x:v>
+      </x:c>
+      <x:c r="L3" t="str">
+        <x:v>If utm_content matches attribution-reconciliation.csv, increment this field on the matching kpi-tracker.csv row; otherwise record as manual lead and do not choose a winning script.</x:v>
+      </x:c>
+      <x:c r="M3" t="str">
         <x:v>not_received</x:v>
       </x:c>
-      <x:c r="J3" t="str">
+      <x:c r="N3" t="str">
         <x:v>not_applicable_until_user_contacts</x:v>
       </x:c>
-      <x:c r="K3" t="str">
+      <x:c r="O3" t="str">
         <x:v>medium</x:v>
       </x:c>
-      <x:c r="L3" t="str">
+      <x:c r="P3" t="str">
         <x:v>template</x:v>
       </x:c>
-      <x:c r="M3" t="str">
+      <x:c r="Q3" t="str">
         <x:v>確認使用情境，不承諾療效，只提供夜間整理或冷卻素材方向。</x:v>
       </x:c>
-      <x:c r="N3" t="str">
+      <x:c r="R3" t="str">
         <x:v>若同守護者 Luna 需求重複，才測試結果後柔性商品承接。</x:v>
       </x:c>
-      <x:c r="O3" t="str"/>
-      <x:c r="P3" t="str"/>
-      <x:c r="Q3" t="str">
+      <x:c r="S3" t="str"/>
+      <x:c r="T3" t="str"/>
+      <x:c r="U3" t="str">
         <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
       </x:c>
     </x:row>
@@ -2017,42 +2049,52 @@
       <x:c r="C4" t="str">
         <x:v>contact_or_waitlist</x:v>
       </x:c>
-      <x:c r="D4" t="str">
+      <x:c r="D4" t="str"/>
+      <x:c r="E4" t="str">
+        <x:v>Copy from Contact email Campaign content / 推廣內容. Valid examples: iris_affirmation, iris_silence, iris_too_sensitive</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
         <x:v>iris</x:v>
       </x:c>
-      <x:c r="E4" t="str">
+      <x:c r="G4" t="str">
         <x:v>艾莉絲</x:v>
       </x:c>
-      <x:c r="F4" t="str">
+      <x:c r="H4" t="str">
         <x:v>repair_or_contact_request</x:v>
       </x:c>
-      <x:c r="G4" t="str">
+      <x:c r="I4" t="str">
         <x:v>relationship repair prompt / supply route guidance</x:v>
       </x:c>
-      <x:c r="H4" t="str">
+      <x:c r="J4" t="str">
         <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
       </x:c>
-      <x:c r="I4" t="str">
+      <x:c r="K4" t="str">
+        <x:v>contact_requests</x:v>
+      </x:c>
+      <x:c r="L4" t="str">
+        <x:v>If utm_content matches attribution-reconciliation.csv, increment this field on the matching kpi-tracker.csv row; otherwise record as manual lead and do not choose a winning script.</x:v>
+      </x:c>
+      <x:c r="M4" t="str">
         <x:v>not_received</x:v>
       </x:c>
-      <x:c r="J4" t="str">
+      <x:c r="N4" t="str">
         <x:v>not_applicable_until_user_contacts</x:v>
       </x:c>
-      <x:c r="K4" t="str">
+      <x:c r="O4" t="str">
         <x:v>high</x:v>
       </x:c>
-      <x:c r="L4" t="str">
+      <x:c r="P4" t="str">
         <x:v>template</x:v>
       </x:c>
-      <x:c r="M4" t="str">
+      <x:c r="Q4" t="str">
         <x:v>回覆可提供的網站路線與自助素材，不收集敏感個資，不取代諮商。</x:v>
       </x:c>
-      <x:c r="N4" t="str">
+      <x:c r="R4" t="str">
         <x:v>整理成 FAQ、修復計畫或 Contact 模板，不把個案內容公開。</x:v>
       </x:c>
-      <x:c r="O4" t="str"/>
-      <x:c r="P4" t="str"/>
-      <x:c r="Q4" t="str">
+      <x:c r="S4" t="str"/>
+      <x:c r="T4" t="str"/>
+      <x:c r="U4" t="str">
         <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
       </x:c>
     </x:row>
@@ -2064,42 +2106,52 @@
       <x:c r="C5" t="str">
         <x:v>contact_or_waitlist</x:v>
       </x:c>
-      <x:c r="D5" t="str">
+      <x:c r="D5" t="str"/>
+      <x:c r="E5" t="str">
+        <x:v>Copy from Contact email Campaign content / 推廣內容. Valid examples: noah_cancel, noah_phone, noah_quiet_time</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
         <x:v>noah</x:v>
       </x:c>
-      <x:c r="E5" t="str">
+      <x:c r="G5" t="str">
         <x:v>諾雅</x:v>
       </x:c>
-      <x:c r="F5" t="str">
+      <x:c r="H5" t="str">
         <x:v>owned_asset_request</x:v>
       </x:c>
-      <x:c r="G5" t="str">
+      <x:c r="I5" t="str">
         <x:v>guardian PDF / wallpaper / short ritual</x:v>
       </x:c>
-      <x:c r="H5" t="str">
+      <x:c r="J5" t="str">
         <x:v>https://lovetypes.tw/keepsakes/#keepsake-noah</x:v>
       </x:c>
-      <x:c r="I5" t="str">
+      <x:c r="K5" t="str">
+        <x:v>supply_lead_requests</x:v>
+      </x:c>
+      <x:c r="L5" t="str">
+        <x:v>If utm_content matches attribution-reconciliation.csv, increment this field on the matching kpi-tracker.csv row; otherwise record as manual lead and do not choose a winning script.</x:v>
+      </x:c>
+      <x:c r="M5" t="str">
         <x:v>not_received</x:v>
       </x:c>
-      <x:c r="J5" t="str">
+      <x:c r="N5" t="str">
         <x:v>not_applicable_until_user_contacts</x:v>
       </x:c>
-      <x:c r="K5" t="str">
+      <x:c r="O5" t="str">
         <x:v>medium</x:v>
       </x:c>
-      <x:c r="L5" t="str">
+      <x:c r="P5" t="str">
         <x:v>template</x:v>
       </x:c>
-      <x:c r="M5" t="str">
+      <x:c r="Q5" t="str">
         <x:v>確認想收到的守護者素材，回覆預計製作方向與安全邊界。</x:v>
       </x:c>
-      <x:c r="N5" t="str">
+      <x:c r="R5" t="str">
         <x:v>累積同守護者重複需求後，排進 asset-build-backlog 的 build_owned_asset。</x:v>
       </x:c>
-      <x:c r="O5" t="str"/>
-      <x:c r="P5" t="str"/>
-      <x:c r="Q5" t="str">
+      <x:c r="S5" t="str"/>
+      <x:c r="T5" t="str"/>
+      <x:c r="U5" t="str">
         <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
       </x:c>
     </x:row>
@@ -2111,42 +2163,52 @@
       <x:c r="C6" t="str">
         <x:v>contact_or_waitlist</x:v>
       </x:c>
-      <x:c r="D6" t="str">
+      <x:c r="D6" t="str"/>
+      <x:c r="E6" t="str">
+        <x:v>Copy from Contact email Campaign content / 推廣內容. Valid examples: noah_cancel, noah_phone, noah_quiet_time</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
         <x:v>noah</x:v>
       </x:c>
-      <x:c r="E6" t="str">
+      <x:c r="G6" t="str">
         <x:v>諾雅</x:v>
       </x:c>
-      <x:c r="F6" t="str">
+      <x:c r="H6" t="str">
         <x:v>luna_scene_request</x:v>
       </x:c>
-      <x:c r="G6" t="str">
+      <x:c r="I6" t="str">
         <x:v>Luna bedtime / conflict cooldown / quiz aftercare pack</x:v>
       </x:c>
-      <x:c r="H6" t="str">
+      <x:c r="J6" t="str">
         <x:v>https://lovetypes.tw/luna-yoga-music/#luna-noah</x:v>
       </x:c>
-      <x:c r="I6" t="str">
+      <x:c r="K6" t="str">
+        <x:v>luna_pack_clicks</x:v>
+      </x:c>
+      <x:c r="L6" t="str">
+        <x:v>If utm_content matches attribution-reconciliation.csv, increment this field on the matching kpi-tracker.csv row; otherwise record as manual lead and do not choose a winning script.</x:v>
+      </x:c>
+      <x:c r="M6" t="str">
         <x:v>not_received</x:v>
       </x:c>
-      <x:c r="J6" t="str">
+      <x:c r="N6" t="str">
         <x:v>not_applicable_until_user_contacts</x:v>
       </x:c>
-      <x:c r="K6" t="str">
+      <x:c r="O6" t="str">
         <x:v>medium</x:v>
       </x:c>
-      <x:c r="L6" t="str">
+      <x:c r="P6" t="str">
         <x:v>template</x:v>
       </x:c>
-      <x:c r="M6" t="str">
+      <x:c r="Q6" t="str">
         <x:v>確認使用情境，不承諾療效，只提供夜間整理或冷卻素材方向。</x:v>
       </x:c>
-      <x:c r="N6" t="str">
+      <x:c r="R6" t="str">
         <x:v>若同守護者 Luna 需求重複，才測試結果後柔性商品承接。</x:v>
       </x:c>
-      <x:c r="O6" t="str"/>
-      <x:c r="P6" t="str"/>
-      <x:c r="Q6" t="str">
+      <x:c r="S6" t="str"/>
+      <x:c r="T6" t="str"/>
+      <x:c r="U6" t="str">
         <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
       </x:c>
     </x:row>
@@ -2158,42 +2220,52 @@
       <x:c r="C7" t="str">
         <x:v>contact_or_waitlist</x:v>
       </x:c>
-      <x:c r="D7" t="str">
+      <x:c r="D7" t="str"/>
+      <x:c r="E7" t="str">
+        <x:v>Copy from Contact email Campaign content / 推廣內容. Valid examples: noah_cancel, noah_phone, noah_quiet_time</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
         <x:v>noah</x:v>
       </x:c>
-      <x:c r="E7" t="str">
+      <x:c r="G7" t="str">
         <x:v>諾雅</x:v>
       </x:c>
-      <x:c r="F7" t="str">
+      <x:c r="H7" t="str">
         <x:v>repair_or_contact_request</x:v>
       </x:c>
-      <x:c r="G7" t="str">
+      <x:c r="I7" t="str">
         <x:v>relationship repair prompt / supply route guidance</x:v>
       </x:c>
-      <x:c r="H7" t="str">
+      <x:c r="J7" t="str">
         <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
       </x:c>
-      <x:c r="I7" t="str">
+      <x:c r="K7" t="str">
+        <x:v>contact_requests</x:v>
+      </x:c>
+      <x:c r="L7" t="str">
+        <x:v>If utm_content matches attribution-reconciliation.csv, increment this field on the matching kpi-tracker.csv row; otherwise record as manual lead and do not choose a winning script.</x:v>
+      </x:c>
+      <x:c r="M7" t="str">
         <x:v>not_received</x:v>
       </x:c>
-      <x:c r="J7" t="str">
+      <x:c r="N7" t="str">
         <x:v>not_applicable_until_user_contacts</x:v>
       </x:c>
-      <x:c r="K7" t="str">
+      <x:c r="O7" t="str">
         <x:v>high</x:v>
       </x:c>
-      <x:c r="L7" t="str">
+      <x:c r="P7" t="str">
         <x:v>template</x:v>
       </x:c>
-      <x:c r="M7" t="str">
+      <x:c r="Q7" t="str">
         <x:v>回覆可提供的網站路線與自助素材，不收集敏感個資，不取代諮商。</x:v>
       </x:c>
-      <x:c r="N7" t="str">
+      <x:c r="R7" t="str">
         <x:v>整理成 FAQ、修復計畫或 Contact 模板，不把個案內容公開。</x:v>
       </x:c>
-      <x:c r="O7" t="str"/>
-      <x:c r="P7" t="str"/>
-      <x:c r="Q7" t="str">
+      <x:c r="S7" t="str"/>
+      <x:c r="T7" t="str"/>
+      <x:c r="U7" t="str">
         <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
       </x:c>
     </x:row>
@@ -2205,42 +2277,52 @@
       <x:c r="C8" t="str">
         <x:v>contact_or_waitlist</x:v>
       </x:c>
-      <x:c r="D8" t="str">
+      <x:c r="D8" t="str"/>
+      <x:c r="E8" t="str">
+        <x:v>Copy from Contact email Campaign content / 推廣內容. Valid examples: vivian_forgotten_date, vivian_remembered, vivian_ritual</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
         <x:v>vivian</x:v>
       </x:c>
-      <x:c r="E8" t="str">
+      <x:c r="G8" t="str">
         <x:v>薇薇安</x:v>
       </x:c>
-      <x:c r="F8" t="str">
+      <x:c r="H8" t="str">
         <x:v>owned_asset_request</x:v>
       </x:c>
-      <x:c r="G8" t="str">
+      <x:c r="I8" t="str">
         <x:v>guardian PDF / wallpaper / short ritual</x:v>
       </x:c>
-      <x:c r="H8" t="str">
+      <x:c r="J8" t="str">
         <x:v>https://lovetypes.tw/keepsakes/#keepsake-vivian</x:v>
       </x:c>
-      <x:c r="I8" t="str">
+      <x:c r="K8" t="str">
+        <x:v>supply_lead_requests</x:v>
+      </x:c>
+      <x:c r="L8" t="str">
+        <x:v>If utm_content matches attribution-reconciliation.csv, increment this field on the matching kpi-tracker.csv row; otherwise record as manual lead and do not choose a winning script.</x:v>
+      </x:c>
+      <x:c r="M8" t="str">
         <x:v>not_received</x:v>
       </x:c>
-      <x:c r="J8" t="str">
+      <x:c r="N8" t="str">
         <x:v>not_applicable_until_user_contacts</x:v>
       </x:c>
-      <x:c r="K8" t="str">
+      <x:c r="O8" t="str">
         <x:v>medium</x:v>
       </x:c>
-      <x:c r="L8" t="str">
+      <x:c r="P8" t="str">
         <x:v>template</x:v>
       </x:c>
-      <x:c r="M8" t="str">
+      <x:c r="Q8" t="str">
         <x:v>確認想收到的守護者素材，回覆預計製作方向與安全邊界。</x:v>
       </x:c>
-      <x:c r="N8" t="str">
+      <x:c r="R8" t="str">
         <x:v>累積同守護者重複需求後，排進 asset-build-backlog 的 build_owned_asset。</x:v>
       </x:c>
-      <x:c r="O8" t="str"/>
-      <x:c r="P8" t="str"/>
-      <x:c r="Q8" t="str">
+      <x:c r="S8" t="str"/>
+      <x:c r="T8" t="str"/>
+      <x:c r="U8" t="str">
         <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
       </x:c>
     </x:row>
@@ -2252,42 +2334,52 @@
       <x:c r="C9" t="str">
         <x:v>contact_or_waitlist</x:v>
       </x:c>
-      <x:c r="D9" t="str">
+      <x:c r="D9" t="str"/>
+      <x:c r="E9" t="str">
+        <x:v>Copy from Contact email Campaign content / 推廣內容. Valid examples: vivian_forgotten_date, vivian_remembered, vivian_ritual</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
         <x:v>vivian</x:v>
       </x:c>
-      <x:c r="E9" t="str">
+      <x:c r="G9" t="str">
         <x:v>薇薇安</x:v>
       </x:c>
-      <x:c r="F9" t="str">
+      <x:c r="H9" t="str">
         <x:v>luna_scene_request</x:v>
       </x:c>
-      <x:c r="G9" t="str">
+      <x:c r="I9" t="str">
         <x:v>Luna bedtime / conflict cooldown / quiz aftercare pack</x:v>
       </x:c>
-      <x:c r="H9" t="str">
+      <x:c r="J9" t="str">
         <x:v>https://lovetypes.tw/luna-yoga-music/#luna-vivian</x:v>
       </x:c>
-      <x:c r="I9" t="str">
+      <x:c r="K9" t="str">
+        <x:v>luna_pack_clicks</x:v>
+      </x:c>
+      <x:c r="L9" t="str">
+        <x:v>If utm_content matches attribution-reconciliation.csv, increment this field on the matching kpi-tracker.csv row; otherwise record as manual lead and do not choose a winning script.</x:v>
+      </x:c>
+      <x:c r="M9" t="str">
         <x:v>not_received</x:v>
       </x:c>
-      <x:c r="J9" t="str">
+      <x:c r="N9" t="str">
         <x:v>not_applicable_until_user_contacts</x:v>
       </x:c>
-      <x:c r="K9" t="str">
+      <x:c r="O9" t="str">
         <x:v>medium</x:v>
       </x:c>
-      <x:c r="L9" t="str">
+      <x:c r="P9" t="str">
         <x:v>template</x:v>
       </x:c>
-      <x:c r="M9" t="str">
+      <x:c r="Q9" t="str">
         <x:v>確認使用情境，不承諾療效，只提供夜間整理或冷卻素材方向。</x:v>
       </x:c>
-      <x:c r="N9" t="str">
+      <x:c r="R9" t="str">
         <x:v>若同守護者 Luna 需求重複，才測試結果後柔性商品承接。</x:v>
       </x:c>
-      <x:c r="O9" t="str"/>
-      <x:c r="P9" t="str"/>
-      <x:c r="Q9" t="str">
+      <x:c r="S9" t="str"/>
+      <x:c r="T9" t="str"/>
+      <x:c r="U9" t="str">
         <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
       </x:c>
     </x:row>
@@ -2299,42 +2391,52 @@
       <x:c r="C10" t="str">
         <x:v>contact_or_waitlist</x:v>
       </x:c>
-      <x:c r="D10" t="str">
+      <x:c r="D10" t="str"/>
+      <x:c r="E10" t="str">
+        <x:v>Copy from Contact email Campaign content / 推廣內容. Valid examples: vivian_forgotten_date, vivian_remembered, vivian_ritual</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
         <x:v>vivian</x:v>
       </x:c>
-      <x:c r="E10" t="str">
+      <x:c r="G10" t="str">
         <x:v>薇薇安</x:v>
       </x:c>
-      <x:c r="F10" t="str">
+      <x:c r="H10" t="str">
         <x:v>repair_or_contact_request</x:v>
       </x:c>
-      <x:c r="G10" t="str">
+      <x:c r="I10" t="str">
         <x:v>relationship repair prompt / supply route guidance</x:v>
       </x:c>
-      <x:c r="H10" t="str">
+      <x:c r="J10" t="str">
         <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
       </x:c>
-      <x:c r="I10" t="str">
+      <x:c r="K10" t="str">
+        <x:v>contact_requests</x:v>
+      </x:c>
+      <x:c r="L10" t="str">
+        <x:v>If utm_content matches attribution-reconciliation.csv, increment this field on the matching kpi-tracker.csv row; otherwise record as manual lead and do not choose a winning script.</x:v>
+      </x:c>
+      <x:c r="M10" t="str">
         <x:v>not_received</x:v>
       </x:c>
-      <x:c r="J10" t="str">
+      <x:c r="N10" t="str">
         <x:v>not_applicable_until_user_contacts</x:v>
       </x:c>
-      <x:c r="K10" t="str">
+      <x:c r="O10" t="str">
         <x:v>high</x:v>
       </x:c>
-      <x:c r="L10" t="str">
+      <x:c r="P10" t="str">
         <x:v>template</x:v>
       </x:c>
-      <x:c r="M10" t="str">
+      <x:c r="Q10" t="str">
         <x:v>回覆可提供的網站路線與自助素材，不收集敏感個資，不取代諮商。</x:v>
       </x:c>
-      <x:c r="N10" t="str">
+      <x:c r="R10" t="str">
         <x:v>整理成 FAQ、修復計畫或 Contact 模板，不把個案內容公開。</x:v>
       </x:c>
-      <x:c r="O10" t="str"/>
-      <x:c r="P10" t="str"/>
-      <x:c r="Q10" t="str">
+      <x:c r="S10" t="str"/>
+      <x:c r="T10" t="str"/>
+      <x:c r="U10" t="str">
         <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
       </x:c>
     </x:row>
@@ -2346,42 +2448,52 @@
       <x:c r="C11" t="str">
         <x:v>contact_or_waitlist</x:v>
       </x:c>
-      <x:c r="D11" t="str">
+      <x:c r="D11" t="str"/>
+      <x:c r="E11" t="str">
+        <x:v>Copy from Contact email Campaign content / 推廣內容. Valid examples: claire_ask_help, claire_promises, claire_tired</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
         <x:v>claire</x:v>
       </x:c>
-      <x:c r="E11" t="str">
+      <x:c r="G11" t="str">
         <x:v>克萊兒</x:v>
       </x:c>
-      <x:c r="F11" t="str">
+      <x:c r="H11" t="str">
         <x:v>owned_asset_request</x:v>
       </x:c>
-      <x:c r="G11" t="str">
+      <x:c r="I11" t="str">
         <x:v>guardian PDF / wallpaper / short ritual</x:v>
       </x:c>
-      <x:c r="H11" t="str">
+      <x:c r="J11" t="str">
         <x:v>https://lovetypes.tw/keepsakes/#keepsake-claire</x:v>
       </x:c>
-      <x:c r="I11" t="str">
+      <x:c r="K11" t="str">
+        <x:v>supply_lead_requests</x:v>
+      </x:c>
+      <x:c r="L11" t="str">
+        <x:v>If utm_content matches attribution-reconciliation.csv, increment this field on the matching kpi-tracker.csv row; otherwise record as manual lead and do not choose a winning script.</x:v>
+      </x:c>
+      <x:c r="M11" t="str">
         <x:v>not_received</x:v>
       </x:c>
-      <x:c r="J11" t="str">
+      <x:c r="N11" t="str">
         <x:v>not_applicable_until_user_contacts</x:v>
       </x:c>
-      <x:c r="K11" t="str">
+      <x:c r="O11" t="str">
         <x:v>medium</x:v>
       </x:c>
-      <x:c r="L11" t="str">
+      <x:c r="P11" t="str">
         <x:v>template</x:v>
       </x:c>
-      <x:c r="M11" t="str">
+      <x:c r="Q11" t="str">
         <x:v>確認想收到的守護者素材，回覆預計製作方向與安全邊界。</x:v>
       </x:c>
-      <x:c r="N11" t="str">
+      <x:c r="R11" t="str">
         <x:v>累積同守護者重複需求後，排進 asset-build-backlog 的 build_owned_asset。</x:v>
       </x:c>
-      <x:c r="O11" t="str"/>
-      <x:c r="P11" t="str"/>
-      <x:c r="Q11" t="str">
+      <x:c r="S11" t="str"/>
+      <x:c r="T11" t="str"/>
+      <x:c r="U11" t="str">
         <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
       </x:c>
     </x:row>
@@ -2393,42 +2505,52 @@
       <x:c r="C12" t="str">
         <x:v>contact_or_waitlist</x:v>
       </x:c>
-      <x:c r="D12" t="str">
+      <x:c r="D12" t="str"/>
+      <x:c r="E12" t="str">
+        <x:v>Copy from Contact email Campaign content / 推廣內容. Valid examples: claire_ask_help, claire_promises, claire_tired</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
         <x:v>claire</x:v>
       </x:c>
-      <x:c r="E12" t="str">
+      <x:c r="G12" t="str">
         <x:v>克萊兒</x:v>
       </x:c>
-      <x:c r="F12" t="str">
+      <x:c r="H12" t="str">
         <x:v>luna_scene_request</x:v>
       </x:c>
-      <x:c r="G12" t="str">
+      <x:c r="I12" t="str">
         <x:v>Luna bedtime / conflict cooldown / quiz aftercare pack</x:v>
       </x:c>
-      <x:c r="H12" t="str">
+      <x:c r="J12" t="str">
         <x:v>https://lovetypes.tw/luna-yoga-music/#luna-claire</x:v>
       </x:c>
-      <x:c r="I12" t="str">
+      <x:c r="K12" t="str">
+        <x:v>luna_pack_clicks</x:v>
+      </x:c>
+      <x:c r="L12" t="str">
+        <x:v>If utm_content matches attribution-reconciliation.csv, increment this field on the matching kpi-tracker.csv row; otherwise record as manual lead and do not choose a winning script.</x:v>
+      </x:c>
+      <x:c r="M12" t="str">
         <x:v>not_received</x:v>
       </x:c>
-      <x:c r="J12" t="str">
+      <x:c r="N12" t="str">
         <x:v>not_applicable_until_user_contacts</x:v>
       </x:c>
-      <x:c r="K12" t="str">
+      <x:c r="O12" t="str">
         <x:v>medium</x:v>
       </x:c>
-      <x:c r="L12" t="str">
+      <x:c r="P12" t="str">
         <x:v>template</x:v>
       </x:c>
-      <x:c r="M12" t="str">
+      <x:c r="Q12" t="str">
         <x:v>確認使用情境，不承諾療效，只提供夜間整理或冷卻素材方向。</x:v>
       </x:c>
-      <x:c r="N12" t="str">
+      <x:c r="R12" t="str">
         <x:v>若同守護者 Luna 需求重複，才測試結果後柔性商品承接。</x:v>
       </x:c>
-      <x:c r="O12" t="str"/>
-      <x:c r="P12" t="str"/>
-      <x:c r="Q12" t="str">
+      <x:c r="S12" t="str"/>
+      <x:c r="T12" t="str"/>
+      <x:c r="U12" t="str">
         <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
       </x:c>
     </x:row>
@@ -2440,42 +2562,52 @@
       <x:c r="C13" t="str">
         <x:v>contact_or_waitlist</x:v>
       </x:c>
-      <x:c r="D13" t="str">
+      <x:c r="D13" t="str"/>
+      <x:c r="E13" t="str">
+        <x:v>Copy from Contact email Campaign content / 推廣內容. Valid examples: claire_ask_help, claire_promises, claire_tired</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
         <x:v>claire</x:v>
       </x:c>
-      <x:c r="E13" t="str">
+      <x:c r="G13" t="str">
         <x:v>克萊兒</x:v>
       </x:c>
-      <x:c r="F13" t="str">
+      <x:c r="H13" t="str">
         <x:v>repair_or_contact_request</x:v>
       </x:c>
-      <x:c r="G13" t="str">
+      <x:c r="I13" t="str">
         <x:v>relationship repair prompt / supply route guidance</x:v>
       </x:c>
-      <x:c r="H13" t="str">
+      <x:c r="J13" t="str">
         <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
       </x:c>
-      <x:c r="I13" t="str">
+      <x:c r="K13" t="str">
+        <x:v>contact_requests</x:v>
+      </x:c>
+      <x:c r="L13" t="str">
+        <x:v>If utm_content matches attribution-reconciliation.csv, increment this field on the matching kpi-tracker.csv row; otherwise record as manual lead and do not choose a winning script.</x:v>
+      </x:c>
+      <x:c r="M13" t="str">
         <x:v>not_received</x:v>
       </x:c>
-      <x:c r="J13" t="str">
+      <x:c r="N13" t="str">
         <x:v>not_applicable_until_user_contacts</x:v>
       </x:c>
-      <x:c r="K13" t="str">
+      <x:c r="O13" t="str">
         <x:v>high</x:v>
       </x:c>
-      <x:c r="L13" t="str">
+      <x:c r="P13" t="str">
         <x:v>template</x:v>
       </x:c>
-      <x:c r="M13" t="str">
+      <x:c r="Q13" t="str">
         <x:v>回覆可提供的網站路線與自助素材，不收集敏感個資，不取代諮商。</x:v>
       </x:c>
-      <x:c r="N13" t="str">
+      <x:c r="R13" t="str">
         <x:v>整理成 FAQ、修復計畫或 Contact 模板，不把個案內容公開。</x:v>
       </x:c>
-      <x:c r="O13" t="str"/>
-      <x:c r="P13" t="str"/>
-      <x:c r="Q13" t="str">
+      <x:c r="S13" t="str"/>
+      <x:c r="T13" t="str"/>
+      <x:c r="U13" t="str">
         <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
       </x:c>
     </x:row>
@@ -2487,42 +2619,52 @@
       <x:c r="C14" t="str">
         <x:v>contact_or_waitlist</x:v>
       </x:c>
-      <x:c r="D14" t="str">
+      <x:c r="D14" t="str"/>
+      <x:c r="E14" t="str">
+        <x:v>Copy from Contact email Campaign content / 推廣內容. Valid examples: dora_after_conflict, dora_consent, dora_distance</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
         <x:v>dora</x:v>
       </x:c>
-      <x:c r="E14" t="str">
+      <x:c r="G14" t="str">
         <x:v>朵拉</x:v>
       </x:c>
-      <x:c r="F14" t="str">
+      <x:c r="H14" t="str">
         <x:v>owned_asset_request</x:v>
       </x:c>
-      <x:c r="G14" t="str">
+      <x:c r="I14" t="str">
         <x:v>guardian PDF / wallpaper / short ritual</x:v>
       </x:c>
-      <x:c r="H14" t="str">
+      <x:c r="J14" t="str">
         <x:v>https://lovetypes.tw/keepsakes/#keepsake-dora</x:v>
       </x:c>
-      <x:c r="I14" t="str">
+      <x:c r="K14" t="str">
+        <x:v>supply_lead_requests</x:v>
+      </x:c>
+      <x:c r="L14" t="str">
+        <x:v>If utm_content matches attribution-reconciliation.csv, increment this field on the matching kpi-tracker.csv row; otherwise record as manual lead and do not choose a winning script.</x:v>
+      </x:c>
+      <x:c r="M14" t="str">
         <x:v>not_received</x:v>
       </x:c>
-      <x:c r="J14" t="str">
+      <x:c r="N14" t="str">
         <x:v>not_applicable_until_user_contacts</x:v>
       </x:c>
-      <x:c r="K14" t="str">
+      <x:c r="O14" t="str">
         <x:v>medium</x:v>
       </x:c>
-      <x:c r="L14" t="str">
+      <x:c r="P14" t="str">
         <x:v>template</x:v>
       </x:c>
-      <x:c r="M14" t="str">
+      <x:c r="Q14" t="str">
         <x:v>確認想收到的守護者素材，回覆預計製作方向與安全邊界。</x:v>
       </x:c>
-      <x:c r="N14" t="str">
+      <x:c r="R14" t="str">
         <x:v>累積同守護者重複需求後，排進 asset-build-backlog 的 build_owned_asset。</x:v>
       </x:c>
-      <x:c r="O14" t="str"/>
-      <x:c r="P14" t="str"/>
-      <x:c r="Q14" t="str">
+      <x:c r="S14" t="str"/>
+      <x:c r="T14" t="str"/>
+      <x:c r="U14" t="str">
         <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
       </x:c>
     </x:row>
@@ -2534,42 +2676,52 @@
       <x:c r="C15" t="str">
         <x:v>contact_or_waitlist</x:v>
       </x:c>
-      <x:c r="D15" t="str">
+      <x:c r="D15" t="str"/>
+      <x:c r="E15" t="str">
+        <x:v>Copy from Contact email Campaign content / 推廣內容. Valid examples: dora_after_conflict, dora_consent, dora_distance</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
         <x:v>dora</x:v>
       </x:c>
-      <x:c r="E15" t="str">
+      <x:c r="G15" t="str">
         <x:v>朵拉</x:v>
       </x:c>
-      <x:c r="F15" t="str">
+      <x:c r="H15" t="str">
         <x:v>luna_scene_request</x:v>
       </x:c>
-      <x:c r="G15" t="str">
+      <x:c r="I15" t="str">
         <x:v>Luna bedtime / conflict cooldown / quiz aftercare pack</x:v>
       </x:c>
-      <x:c r="H15" t="str">
+      <x:c r="J15" t="str">
         <x:v>https://lovetypes.tw/luna-yoga-music/#luna-dora</x:v>
       </x:c>
-      <x:c r="I15" t="str">
+      <x:c r="K15" t="str">
+        <x:v>luna_pack_clicks</x:v>
+      </x:c>
+      <x:c r="L15" t="str">
+        <x:v>If utm_content matches attribution-reconciliation.csv, increment this field on the matching kpi-tracker.csv row; otherwise record as manual lead and do not choose a winning script.</x:v>
+      </x:c>
+      <x:c r="M15" t="str">
         <x:v>not_received</x:v>
       </x:c>
-      <x:c r="J15" t="str">
+      <x:c r="N15" t="str">
         <x:v>not_applicable_until_user_contacts</x:v>
       </x:c>
-      <x:c r="K15" t="str">
+      <x:c r="O15" t="str">
         <x:v>medium</x:v>
       </x:c>
-      <x:c r="L15" t="str">
+      <x:c r="P15" t="str">
         <x:v>template</x:v>
       </x:c>
-      <x:c r="M15" t="str">
+      <x:c r="Q15" t="str">
         <x:v>確認使用情境，不承諾療效，只提供夜間整理或冷卻素材方向。</x:v>
       </x:c>
-      <x:c r="N15" t="str">
+      <x:c r="R15" t="str">
         <x:v>若同守護者 Luna 需求重複，才測試結果後柔性商品承接。</x:v>
       </x:c>
-      <x:c r="O15" t="str"/>
-      <x:c r="P15" t="str"/>
-      <x:c r="Q15" t="str">
+      <x:c r="S15" t="str"/>
+      <x:c r="T15" t="str"/>
+      <x:c r="U15" t="str">
         <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
       </x:c>
     </x:row>
@@ -2581,42 +2733,52 @@
       <x:c r="C16" t="str">
         <x:v>contact_or_waitlist</x:v>
       </x:c>
-      <x:c r="D16" t="str">
+      <x:c r="D16" t="str"/>
+      <x:c r="E16" t="str">
+        <x:v>Copy from Contact email Campaign content / 推廣內容. Valid examples: dora_after_conflict, dora_consent, dora_distance</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
         <x:v>dora</x:v>
       </x:c>
-      <x:c r="E16" t="str">
+      <x:c r="G16" t="str">
         <x:v>朵拉</x:v>
       </x:c>
-      <x:c r="F16" t="str">
+      <x:c r="H16" t="str">
         <x:v>repair_or_contact_request</x:v>
       </x:c>
-      <x:c r="G16" t="str">
+      <x:c r="I16" t="str">
         <x:v>relationship repair prompt / supply route guidance</x:v>
       </x:c>
-      <x:c r="H16" t="str">
+      <x:c r="J16" t="str">
         <x:v>https://lovetypes.tw/contact/#luna-supply-request</x:v>
       </x:c>
-      <x:c r="I16" t="str">
+      <x:c r="K16" t="str">
+        <x:v>contact_requests</x:v>
+      </x:c>
+      <x:c r="L16" t="str">
+        <x:v>If utm_content matches attribution-reconciliation.csv, increment this field on the matching kpi-tracker.csv row; otherwise record as manual lead and do not choose a winning script.</x:v>
+      </x:c>
+      <x:c r="M16" t="str">
         <x:v>not_received</x:v>
       </x:c>
-      <x:c r="J16" t="str">
+      <x:c r="N16" t="str">
         <x:v>not_applicable_until_user_contacts</x:v>
       </x:c>
-      <x:c r="K16" t="str">
+      <x:c r="O16" t="str">
         <x:v>high</x:v>
       </x:c>
-      <x:c r="L16" t="str">
+      <x:c r="P16" t="str">
         <x:v>template</x:v>
       </x:c>
-      <x:c r="M16" t="str">
+      <x:c r="Q16" t="str">
         <x:v>回覆可提供的網站路線與自助素材，不收集敏感個資，不取代諮商。</x:v>
       </x:c>
-      <x:c r="N16" t="str">
+      <x:c r="R16" t="str">
         <x:v>整理成 FAQ、修復計畫或 Contact 模板，不把個案內容公開。</x:v>
       </x:c>
-      <x:c r="O16" t="str"/>
-      <x:c r="P16" t="str"/>
-      <x:c r="Q16" t="str">
+      <x:c r="S16" t="str"/>
+      <x:c r="T16" t="str"/>
+      <x:c r="U16" t="str">
         <x:v>No user data. Replace this template row only after a real request arrives.</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Map funnel events to promotion KPIs
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R0818d3cfe95946f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R58f7716cef0a41bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="Reacd67030471492d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R3878b2e4ffe04bac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="R7bf7fe22284d4266"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="Rc6b2cc306a884edc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="R5a92f9328ef646bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="Rd62e6dc311634f2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="Rfbcbd0d3647e47b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="R3e72e1aae68f4603"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="R74bb4ac307d64860"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rdfe867473a3c488e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R39782e59ea32436f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R6866c338046b417b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="Re03fb42f01724e44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="R81569948a70f4f26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="Rd26447b9422b4415"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="R4de83d6b5c3d4163"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="R0a83141764c245d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="R9c805dba3e6a494a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="R7771f3c7fb4d40ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="Rbd7bbfbee4124556"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Refresh LoveTypes KPI workbook
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rdfe867473a3c488e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R39782e59ea32436f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R6866c338046b417b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="Re03fb42f01724e44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="R81569948a70f4f26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="Rd26447b9422b4415"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="R4de83d6b5c3d4163"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="R0a83141764c245d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="R9c805dba3e6a494a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="R7771f3c7fb4d40ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="Rbd7bbfbee4124556"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6a40b811c9754aa6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R274eb5fd003541f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R3660b8f5acc7441c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R93bd023108d94647"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="Rc9d3177470ea4c4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="R4a276a4103524e9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="Re31cd35a218a4f21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="Recc9f1acabba49c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="R16fe99eacc5e44ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="R85fe2dca58804ba9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="Ra28338f070a145f9"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Validate promotion KPI event alignment
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6a40b811c9754aa6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R274eb5fd003541f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R3660b8f5acc7441c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R93bd023108d94647"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="Rc9d3177470ea4c4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="R4a276a4103524e9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="Re31cd35a218a4f21"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="Recc9f1acabba49c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="R16fe99eacc5e44ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="R85fe2dca58804ba9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="Ra28338f070a145f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R273c44b1f6394156"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R809df1f01a5a4efd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="Re5d81a6c8a6e4828"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="Rb294bfce5db54b7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="Rec80d5f736d44331"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="Rfabec37dd9fd420c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="R1ca66418f18f497c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="R3e95ee1cd235474d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="R0c8bcab83ca54b31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="R0bd33254ad474878"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="R9ffb287df5294764"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Cross-check discovery index routes
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R273c44b1f6394156"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R809df1f01a5a4efd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="Re5d81a6c8a6e4828"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="Rb294bfce5db54b7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="Rec80d5f736d44331"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="Rfabec37dd9fd420c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="R1ca66418f18f497c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="R3e95ee1cd235474d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="R0c8bcab83ca54b31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="R0bd33254ad474878"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="R9ffb287df5294764"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R0b660e3744c94353"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rc1b4f462b39b4a99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R17d9759a07e64c8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R15ecdb41b1f84c27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="R852c4bd69ef94411"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="Rfc1b61f8d45d474a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="Reb6dc5ab1bdb47cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="Rbd29e95eee494da7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="R7989271a6f694474"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="Re67ced4dcff54024"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="R163406d17da34ffb"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Add localized affiliate book links
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R0b660e3744c94353"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rc1b4f462b39b4a99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R17d9759a07e64c8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R15ecdb41b1f84c27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="R852c4bd69ef94411"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="Rfc1b61f8d45d474a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="Reb6dc5ab1bdb47cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="Rbd29e95eee494da7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="R7989271a6f694474"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="Re67ced4dcff54024"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="R163406d17da34ffb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R0c06dec3fffc47c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R18d9636118ad4000"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R6124306481ec4c91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R994756089ec040ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="Rb1641bcbab464020"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="R684c3df5490c486f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="R929dd2f9228a4c14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="Ra90ef1caf573422f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="R11dfa299db9b4a51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="R142ba72fe59240ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="R3e12288bab76490b"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Clarify localized affiliate discovery
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R0c06dec3fffc47c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R18d9636118ad4000"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R6124306481ec4c91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R994756089ec040ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="Rb1641bcbab464020"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="R684c3df5490c486f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="R929dd2f9228a4c14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="Ra90ef1caf573422f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="R11dfa299db9b4a51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="R142ba72fe59240ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="R3e12288bab76490b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R9a2cadde38ec4df3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R439315a1fc5949f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="Ra6bd2c9d94d54777"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R1537e8c6998b4f2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="Rb1479c074c2c472a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="Ra8c65dcef04c4420"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="Rfd98e67b2e0b4ef7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="R67a86233c18a41cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="R553b6fb9d9514298"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="Rb4dad8c6b33e41a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="Rdd5f76a3b5fc4883"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Speed up public internal link smoke
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R9a2cadde38ec4df3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R439315a1fc5949f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="Ra6bd2c9d94d54777"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R1537e8c6998b4f2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="Rb1479c074c2c472a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="Ra8c65dcef04c4420"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="Rfd98e67b2e0b4ef7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="R67a86233c18a41cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="R553b6fb9d9514298"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="Rb4dad8c6b33e41a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="Rdd5f76a3b5fc4883"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Ree5459e1fb8344a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R79e71874c34e45fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R5afdce89cde6460a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R30d7b74ec0214714"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="Rcc4fe77d75284a86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="Rff22422243ac4d0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="R0b4f3a9c9dd84d8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="Re1544862cef44df2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="R3ddfc5bbb39e4bb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="R37c35aaaba69475f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="R731aab57235646bd"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Optimize LoveTypes hero image delivery
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb600bf9b84da487b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R946eb202880d4463"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="Rb921e879bc4a4de7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R2e58fba31a634b41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="Rb1698d7894e0402b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="R39d20af021ba47de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="R3a0cb10eca554a56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="Rd789b09492674871"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="R1409a4d1667e47dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="Rd9e04fb9bf1f4aac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="R53118ec982264c6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8a42cb84ecfc4a50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R8463fb0f4f254d47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="Re9b0fa3e3dab4e78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R77d77498da794df9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="R9386a6ecfb334ec9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="Ra32acd8d192b4bd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="Rd93fb5ea0e994d38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="R4b9bc553b49a47a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="R273fe12bf2e1408a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="Rc41329c4524c4672"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="R1a6db0f2b1454f9f"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Deepen guide-specific repair copy
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8a42cb84ecfc4a50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R8463fb0f4f254d47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="Re9b0fa3e3dab4e78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R77d77498da794df9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="R9386a6ecfb334ec9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="Ra32acd8d192b4bd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="Rd93fb5ea0e994d38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="R4b9bc553b49a47a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="R273fe12bf2e1408a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="Rc41329c4524c4672"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="R1a6db0f2b1454f9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R18f6d34e7f2840b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R1d2e4b99aa854f97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="Rda5617f566304088"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R52e78313f1cb486c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="Rd78b7f47ef2e4034"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="R1c33c56add8e488c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="R0d65c503199946f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="Rc7ed4ccb81ba4aa0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="R597bc77068df4490"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="R08374292e8ed4a09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="Recbc6c0a0a7d489b"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Guard guide copy depth in site audit
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R18f6d34e7f2840b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R1d2e4b99aa854f97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="Rda5617f566304088"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R52e78313f1cb486c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="Rd78b7f47ef2e4034"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="R1c33c56add8e488c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="R0d65c503199946f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="Rc7ed4ccb81ba4aa0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="R597bc77068df4490"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="R08374292e8ed4a09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="Recbc6c0a0a7d489b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rfe81386822c04e87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rf192533aa5104568"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="Rf1459b48756b4404"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R0eddef6925554016"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="Rc9ed46b5d38f4083"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="Rca8bf9ff9d2f414c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="Re0e45425260542ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="R558fe0a3c75b4fda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="Rc576043cdd27482c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="R060375de2d974ca4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="R4bb261da207041e1"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Surface guide depth metrics in health summary
</commit_message>
<xml_diff>
--- a/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
+++ b/docs/promotion/first-round/lovetypes-first-round-kpi-workbook.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rfe81386822c04e87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="Rf192533aa5104568"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="Rf1459b48756b4404"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R0eddef6925554016"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="Rc9ed46b5d38f4083"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="Rca8bf9ff9d2f414c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="Re0e45425260542ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="R558fe0a3c75b4fda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="Rc576043cdd27482c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="R060375de2d974ca4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="R4bb261da207041e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R924223c67ea34c8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker" sheetId="2" r:id="R24f34621b1244d13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Profiles" sheetId="3" r:id="R13652bd4789d4506"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Intake" sheetId="4" r:id="R90075d5b6aa64bf4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Hypotheses" sheetId="5" r:id="R961dbb34d40d4c37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Experiments" sheetId="6" r:id="R1c9a6fb763cb4e03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Queue" sheetId="7" r:id="Rf7af24a10d63407c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Command" sheetId="8" r:id="R217576367ae34184"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Execution" sheetId="9" r:id="Re0761265e6964e39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Actions" sheetId="10" r:id="R847e264828ea4935"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="11" r:id="Rd002a5d918954237"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>